<commit_message>
Pre-fill Secondary Subjects from Department 2 data
5 teachers with dual departments now have Secondary Subjects populated:
- Ferrante-Martin (Theater), Judge (English), Konopelski (Mathematics),
  Kozak (Engineering), Mazella (English)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -185,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -281,6 +281,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5367,7 +5370,11 @@
           <t>English, Special Education</t>
         </is>
       </c>
-      <c r="AD29" s="11" t="n"/>
+      <c r="AD29" s="38" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
       <c r="AE29" s="9" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5707,7 +5714,11 @@
           <t>Mathematics, Social Studies</t>
         </is>
       </c>
-      <c r="AD31" s="11" t="n"/>
+      <c r="AD31" s="38" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
       <c r="AE31" s="9" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5881,7 +5892,11 @@
           <t>Engineering, Science</t>
         </is>
       </c>
-      <c r="AD32" s="11" t="n"/>
+      <c r="AD32" s="38" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
       <c r="AE32" s="16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -6889,7 +6904,11 @@
           <t>English</t>
         </is>
       </c>
-      <c r="AD38" s="11" t="n"/>
+      <c r="AD38" s="38" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
       <c r="AE38" s="16" t="inlineStr">
         <is>
           <t>N</t>
@@ -8083,7 +8102,11 @@
           <t>English</t>
         </is>
       </c>
-      <c r="AD45" s="11" t="n"/>
+      <c r="AD45" s="38" t="inlineStr">
+        <is>
+          <t>Theater</t>
+        </is>
+      </c>
       <c r="AE45" s="9" t="inlineStr">
         <is>
           <t>Y</t>
@@ -13397,8 +13420,6 @@
       </c>
       <c r="E43" s="21" t="inlineStr"/>
     </row>
-    <row r="44"/>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Insert Full-Year Load column between Unique Courses and S1 Load
- New column AP: Full-Year Load (reference field)
- Positioned between AO (Unique Courses) and AQ (S1 Load)
- 47 columns total (A-AU), Column Guide updated

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -91,7 +91,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -166,6 +166,12 @@
         <bgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E0E0"/>
+        <bgColor rgb="00E0E0E0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -185,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -284,6 +290,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -650,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT70"/>
+  <dimension ref="A1:AU70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -694,7 +703,7 @@
     <col width="8" customWidth="1" min="39" max="39"/>
     <col width="8" customWidth="1" min="40" max="40"/>
     <col width="18" customWidth="1" min="41" max="41"/>
-    <col width="8" customWidth="1" min="42" max="42"/>
+    <col width="10" customWidth="1" min="42" max="42"/>
     <col width="35" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
@@ -918,27 +927,32 @@
           <t>Unique Courses</t>
         </is>
       </c>
-      <c r="AP3" s="3" t="inlineStr">
+      <c r="AP3" s="30" t="inlineStr">
+        <is>
+          <t>Full-Year Load</t>
+        </is>
+      </c>
+      <c r="AQ3" s="3" t="inlineStr">
         <is>
           <t>S1 Load</t>
         </is>
       </c>
-      <c r="AQ3" s="3" t="inlineStr">
+      <c r="AR3" s="3" t="inlineStr">
         <is>
           <t>S2 Load</t>
         </is>
       </c>
-      <c r="AR3" s="3" t="inlineStr">
+      <c r="AS3" s="3" t="inlineStr">
         <is>
           <t>Singleton Courses</t>
         </is>
       </c>
-      <c r="AS3" s="3" t="inlineStr">
+      <c r="AT3" s="3" t="inlineStr">
         <is>
           <t>Computed MTP Score</t>
         </is>
       </c>
-      <c r="AT3" s="3" t="inlineStr">
+      <c r="AU3" s="3" t="inlineStr">
         <is>
           <t>Courses Assigned</t>
         </is>
@@ -1150,7 +1164,7 @@
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="AP4" s="6" t="inlineStr">
+      <c r="AP4" s="32" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
@@ -1171,6 +1185,11 @@
         </is>
       </c>
       <c r="AT4" s="6" t="inlineStr">
+        <is>
+          <t>REFERENCE</t>
+        </is>
+      </c>
+      <c r="AU4" s="6" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
@@ -1330,21 +1349,22 @@
       <c r="AO5" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP5" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP5" s="39" t="n"/>
       <c r="AQ5" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR5" s="14" t="inlineStr">
+      <c r="AR5" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS5" s="14" t="inlineStr">
         <is>
           <t>425, 445</t>
         </is>
       </c>
-      <c r="AS5" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT5" s="14" t="inlineStr">
+      <c r="AT5" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU5" s="14" t="inlineStr">
         <is>
           <t>421 Geometry H, 425 Adv Geometry H, 445 Adv Precalculus H</t>
         </is>
@@ -1492,17 +1512,18 @@
       <c r="AO6" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP6" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP6" s="39" t="n"/>
       <c r="AQ6" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR6" s="14" t="inlineStr"/>
-      <c r="AS6" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT6" s="14" t="inlineStr">
+      <c r="AR6" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS6" s="14" t="inlineStr"/>
+      <c r="AT6" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU6" s="14" t="inlineStr">
         <is>
           <t>321 Spanish II H, 330 Spanish III, 351 AP Spanish</t>
         </is>
@@ -1660,17 +1681,18 @@
       <c r="AO7" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP7" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP7" s="39" t="n"/>
       <c r="AQ7" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR7" s="14" t="inlineStr"/>
-      <c r="AS7" s="15" t="n">
+      <c r="AR7" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS7" s="14" t="inlineStr"/>
+      <c r="AT7" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT7" s="14" t="inlineStr">
+      <c r="AU7" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9</t>
         </is>
@@ -1826,17 +1848,18 @@
       <c r="AO8" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP8" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP8" s="39" t="n"/>
       <c r="AQ8" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR8" s="14" t="inlineStr"/>
-      <c r="AS8" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT8" s="14" t="inlineStr">
+      <c r="AR8" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS8" s="14" t="inlineStr"/>
+      <c r="AT8" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU8" s="14" t="inlineStr">
         <is>
           <t>610 Health/PE</t>
         </is>
@@ -1996,21 +2019,22 @@
       <c r="AO9" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AP9" s="15" t="n">
+      <c r="AP9" s="39" t="n"/>
+      <c r="AQ9" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AQ9" s="15" t="n">
+      <c r="AR9" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AR9" s="14" t="inlineStr">
+      <c r="AS9" s="14" t="inlineStr">
         <is>
           <t>472, 490, 491, 494, 496</t>
         </is>
       </c>
-      <c r="AS9" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT9" s="14" t="inlineStr">
+      <c r="AT9" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU9" s="14" t="inlineStr">
         <is>
           <t>472 Web Design, 473 Introduction to Programming, 490 AP Computer Science A, 491 AP Computer Science Principles, 494 Applied Programming, 496 AP Cybersecurity</t>
         </is>
@@ -2170,21 +2194,22 @@
       <c r="AO10" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP10" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP10" s="39" t="n"/>
       <c r="AQ10" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR10" s="14" t="inlineStr">
+      <c r="AR10" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS10" s="14" t="inlineStr">
         <is>
           <t>455</t>
         </is>
       </c>
-      <c r="AS10" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT10" s="14" t="inlineStr">
+      <c r="AT10" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU10" s="14" t="inlineStr">
         <is>
           <t>431 Algebra II/Trig H, 453 AP Calc AB, 455 AP Calc BC</t>
         </is>
@@ -2344,21 +2369,22 @@
       <c r="AO11" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP11" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP11" s="39" t="n"/>
       <c r="AQ11" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR11" s="14" t="inlineStr">
+      <c r="AR11" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS11" s="14" t="inlineStr">
         <is>
           <t>311</t>
         </is>
       </c>
-      <c r="AS11" s="15" t="n">
+      <c r="AT11" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT11" s="14" t="inlineStr">
+      <c r="AU11" s="14" t="inlineStr">
         <is>
           <t>311 Spanish I H, 320 Spanish II</t>
         </is>
@@ -2518,17 +2544,18 @@
       <c r="AO12" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP12" s="15" t="n">
+      <c r="AP12" s="39" t="n"/>
+      <c r="AQ12" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AQ12" s="15" t="n">
+      <c r="AR12" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AR12" s="14" t="inlineStr"/>
-      <c r="AS12" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT12" s="14" t="inlineStr">
+      <c r="AS12" s="14" t="inlineStr"/>
+      <c r="AT12" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU12" s="14" t="inlineStr">
         <is>
           <t>631 CPR-AED Training/PE, 642 Nutrition &amp; Fitness/PE</t>
         </is>
@@ -2688,21 +2715,22 @@
       <c r="AO13" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP13" s="15" t="n">
-        <v>3</v>
-      </c>
+      <c r="AP13" s="39" t="n"/>
       <c r="AQ13" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AR13" s="14" t="inlineStr">
+      <c r="AR13" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS13" s="14" t="inlineStr">
         <is>
           <t>544</t>
         </is>
       </c>
-      <c r="AS13" s="15" t="n">
+      <c r="AT13" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT13" s="14" t="inlineStr">
+      <c r="AU13" s="14" t="inlineStr">
         <is>
           <t>544 Sports Medicine, 546 Forensics</t>
         </is>
@@ -2862,17 +2890,18 @@
       <c r="AO14" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP14" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP14" s="39" t="n"/>
       <c r="AQ14" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR14" s="14" t="inlineStr"/>
-      <c r="AS14" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT14" s="14" t="inlineStr">
+      <c r="AR14" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS14" s="14" t="inlineStr"/>
+      <c r="AT14" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU14" s="14" t="inlineStr">
         <is>
           <t>727 Sports and Entertainment Marketing, 757 International Business Strategies, 758 Bloomberg Market Concepts</t>
         </is>
@@ -3032,17 +3061,18 @@
       <c r="AO15" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP15" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP15" s="39" t="n"/>
       <c r="AQ15" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR15" s="14" t="inlineStr"/>
-      <c r="AS15" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT15" s="14" t="inlineStr">
+      <c r="AR15" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS15" s="14" t="inlineStr"/>
+      <c r="AT15" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU15" s="14" t="inlineStr">
         <is>
           <t>620 Driver's Ed/PE</t>
         </is>
@@ -3190,17 +3220,18 @@
       <c r="AO16" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP16" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP16" s="39" t="n"/>
       <c r="AQ16" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR16" s="14" t="inlineStr"/>
-      <c r="AS16" s="15" t="n">
+      <c r="AR16" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS16" s="14" t="inlineStr"/>
+      <c r="AT16" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT16" s="14" t="inlineStr">
+      <c r="AU16" s="14" t="inlineStr">
         <is>
           <t>412 Algebra I, 432 Algebra II/Trig</t>
         </is>
@@ -3360,17 +3391,18 @@
       <c r="AO17" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP17" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP17" s="39" t="n"/>
       <c r="AQ17" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR17" s="14" t="inlineStr"/>
-      <c r="AS17" s="15" t="n">
+      <c r="AR17" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS17" s="14" t="inlineStr"/>
+      <c r="AT17" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT17" s="14" t="inlineStr">
+      <c r="AU17" s="14" t="inlineStr">
         <is>
           <t>111 Composition &amp; Literature H, 129 AP Seminar</t>
         </is>
@@ -3530,21 +3562,22 @@
       <c r="AO18" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="AP18" s="15" t="n">
+      <c r="AP18" s="39" t="n"/>
+      <c r="AQ18" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="AQ18" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AR18" s="14" t="inlineStr">
+      <c r="AR18" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS18" s="14" t="inlineStr">
         <is>
           <t>242, 243, 248, 249, 253, 254, 255, 764</t>
         </is>
       </c>
-      <c r="AS18" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT18" s="14" t="inlineStr">
+      <c r="AT18" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU18" s="14" t="inlineStr">
         <is>
           <t>241 Studio Art I, 242 Studio Art II, 243 Studio Art III, 248 Adv Drawing, 249 Adv Painting, 253 AP Drawing, 254 AP 2-D Art and Design, 255 AP 3-D Art and Design, 764 AP Art History</t>
         </is>
@@ -3704,17 +3737,18 @@
       <c r="AO19" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP19" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP19" s="39" t="n"/>
       <c r="AQ19" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR19" s="14" t="inlineStr"/>
-      <c r="AS19" s="15" t="n">
+      <c r="AR19" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS19" s="14" t="inlineStr"/>
+      <c r="AT19" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT19" s="14" t="inlineStr">
+      <c r="AU19" s="14" t="inlineStr">
         <is>
           <t>520 Chemistry</t>
         </is>
@@ -3874,17 +3908,18 @@
       <c r="AO20" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP20" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP20" s="39" t="n"/>
       <c r="AQ20" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR20" s="14" t="inlineStr"/>
-      <c r="AS20" s="15" t="n">
+      <c r="AR20" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS20" s="14" t="inlineStr"/>
+      <c r="AT20" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT20" s="14" t="inlineStr">
+      <c r="AU20" s="14" t="inlineStr">
         <is>
           <t>130 British Literature, 141 College English Honors</t>
         </is>
@@ -4044,17 +4079,18 @@
       <c r="AO21" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AP21" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP21" s="39" t="n"/>
       <c r="AQ21" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR21" s="14" t="inlineStr"/>
-      <c r="AS21" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT21" s="14" t="inlineStr">
+      <c r="AR21" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS21" s="14" t="inlineStr"/>
+      <c r="AT21" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU21" s="14" t="inlineStr">
         <is>
           <t>726 Business Concepts, 729 AP Business with Personal Finance, 734 Leadership, Entrepreneurship and Opportunity Program I, 745 Leadership, Entrepreneurship and Opportunity Program II</t>
         </is>
@@ -4214,17 +4250,18 @@
       <c r="AO22" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP22" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP22" s="39" t="n"/>
       <c r="AQ22" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR22" s="14" t="inlineStr"/>
-      <c r="AS22" s="15" t="n">
+      <c r="AR22" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS22" s="14" t="inlineStr"/>
+      <c r="AT22" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT22" s="14" t="inlineStr">
+      <c r="AU22" s="14" t="inlineStr">
         <is>
           <t>131 British Literature H, 139 AP English Language</t>
         </is>
@@ -4384,17 +4421,18 @@
       <c r="AO23" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP23" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP23" s="39" t="n"/>
       <c r="AQ23" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR23" s="14" t="inlineStr"/>
-      <c r="AS23" s="15" t="n">
+      <c r="AR23" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS23" s="14" t="inlineStr"/>
+      <c r="AT23" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT23" s="14" t="inlineStr">
+      <c r="AU23" s="14" t="inlineStr">
         <is>
           <t>420 Geometry, 440 Precalculus</t>
         </is>
@@ -4554,21 +4592,22 @@
       <c r="AO24" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP24" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP24" s="39" t="n"/>
       <c r="AQ24" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR24" s="14" t="inlineStr">
+      <c r="AR24" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS24" s="14" t="inlineStr">
         <is>
           <t>435</t>
         </is>
       </c>
-      <c r="AS24" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT24" s="14" t="inlineStr">
+      <c r="AT24" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU24" s="14" t="inlineStr">
         <is>
           <t>435 Adv Algebra II / Trig H, 440 Precalculus, 448 Pre-college Math</t>
         </is>
@@ -4716,21 +4755,22 @@
       <c r="AO25" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP25" s="15" t="n">
-        <v>3</v>
-      </c>
+      <c r="AP25" s="39" t="n"/>
       <c r="AQ25" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AR25" s="14" t="inlineStr">
+      <c r="AR25" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS25" s="14" t="inlineStr">
         <is>
           <t>542</t>
         </is>
       </c>
-      <c r="AS25" s="15" t="n">
+      <c r="AT25" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT25" s="14" t="inlineStr">
+      <c r="AU25" s="14" t="inlineStr">
         <is>
           <t>542 Anatomy/Physiology, 543 Anatomy/Physiology H</t>
         </is>
@@ -4890,17 +4930,18 @@
       <c r="AO26" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP26" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP26" s="39" t="n"/>
       <c r="AQ26" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR26" s="14" t="inlineStr"/>
-      <c r="AS26" s="15" t="n">
+      <c r="AR26" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS26" s="14" t="inlineStr"/>
+      <c r="AT26" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT26" s="14" t="inlineStr">
+      <c r="AU26" s="14" t="inlineStr">
         <is>
           <t>430 Algebra II/Trig, 443 AP Precalculus</t>
         </is>
@@ -5060,21 +5101,22 @@
       <c r="AO27" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP27" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP27" s="39" t="n"/>
       <c r="AQ27" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR27" s="14" t="inlineStr">
+      <c r="AR27" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS27" s="14" t="inlineStr">
         <is>
           <t>761</t>
         </is>
       </c>
-      <c r="AS27" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT27" s="14" t="inlineStr">
+      <c r="AT27" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU27" s="14" t="inlineStr">
         <is>
           <t>730 U.S. History II, 731 U.S. History II H, 761 AP Psychology</t>
         </is>
@@ -5234,21 +5276,22 @@
       <c r="AO28" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP28" s="15" t="n">
-        <v>6</v>
-      </c>
+      <c r="AP28" s="39" t="n"/>
       <c r="AQ28" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AR28" s="14" t="inlineStr">
+      <c r="AR28" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS28" s="14" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="AS28" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT28" s="14" t="inlineStr">
+      <c r="AT28" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU28" s="14" t="inlineStr">
         <is>
           <t>500 Earth Science, 510 Biology</t>
         </is>
@@ -5404,21 +5447,22 @@
       <c r="AO29" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP29" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP29" s="39" t="n"/>
       <c r="AQ29" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR29" s="14" t="inlineStr">
+      <c r="AR29" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS29" s="14" t="inlineStr">
         <is>
           <t>112, 122</t>
         </is>
       </c>
-      <c r="AS29" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT29" s="14" t="inlineStr">
+      <c r="AT29" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU29" s="14" t="inlineStr">
         <is>
           <t>112 Composition &amp; Literature, 122 American Literature, 955 Academic Support</t>
         </is>
@@ -5578,21 +5622,22 @@
       <c r="AO30" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP30" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP30" s="39" t="n"/>
       <c r="AQ30" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR30" s="14" t="inlineStr">
+      <c r="AR30" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS30" s="14" t="inlineStr">
         <is>
           <t>553</t>
         </is>
       </c>
-      <c r="AS30" s="15" t="n">
+      <c r="AT30" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT30" s="14" t="inlineStr">
+      <c r="AU30" s="14" t="inlineStr">
         <is>
           <t>511 Biology H, 553 AP Chemistry</t>
         </is>
@@ -5748,21 +5793,22 @@
       <c r="AO31" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP31" s="15" t="n">
-        <v>2</v>
-      </c>
+      <c r="AP31" s="39" t="n"/>
       <c r="AQ31" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AR31" s="14" t="inlineStr">
+      <c r="AR31" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS31" s="14" t="inlineStr">
         <is>
           <t>456, 765, 766</t>
         </is>
       </c>
-      <c r="AS31" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT31" s="14" t="inlineStr">
+      <c r="AT31" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU31" s="14" t="inlineStr">
         <is>
           <t>456 AP Statistics, 765 AP Macroeconomics, 766 AP Microeconomics</t>
         </is>
@@ -5930,21 +5976,22 @@
       <c r="AO32" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP32" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP32" s="39" t="n"/>
       <c r="AQ32" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR32" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AR32" s="14" t="inlineStr">
+      <c r="AS32" s="14" t="inlineStr">
         <is>
           <t>595</t>
         </is>
       </c>
-      <c r="AS32" s="15" t="n">
+      <c r="AT32" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT32" s="14" t="inlineStr">
+      <c r="AU32" s="14" t="inlineStr">
         <is>
           <t>530 Physics, 595 Engineering Design</t>
         </is>
@@ -6100,17 +6147,18 @@
       <c r="AO33" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP33" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP33" s="39" t="n"/>
       <c r="AQ33" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR33" s="14" t="inlineStr"/>
-      <c r="AS33" s="15" t="n">
+      <c r="AR33" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS33" s="14" t="inlineStr"/>
+      <c r="AT33" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT33" s="14" t="inlineStr">
+      <c r="AU33" s="14" t="inlineStr">
         <is>
           <t>820 Theology 10, 830 Theology 11</t>
         </is>
@@ -6270,17 +6318,18 @@
       <c r="AO34" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP34" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP34" s="39" t="n"/>
       <c r="AQ34" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR34" s="14" t="inlineStr"/>
-      <c r="AS34" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT34" s="14" t="inlineStr">
+      <c r="AR34" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS34" s="14" t="inlineStr"/>
+      <c r="AT34" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU34" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11, 851 Spirituality of Vocation</t>
         </is>
@@ -6436,17 +6485,18 @@
       <c r="AO35" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP35" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP35" s="39" t="n"/>
       <c r="AQ35" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR35" s="14" t="inlineStr"/>
-      <c r="AS35" s="15" t="n">
+      <c r="AR35" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS35" s="14" t="inlineStr"/>
+      <c r="AT35" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT35" s="14" t="inlineStr">
+      <c r="AU35" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9, 820 Theology 10</t>
         </is>
@@ -6602,21 +6652,22 @@
       <c r="AO36" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AP36" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP36" s="39" t="n"/>
       <c r="AQ36" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR36" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AR36" s="14" t="inlineStr">
+      <c r="AS36" s="14" t="inlineStr">
         <is>
           <t>201, 203, 206, 209, 220</t>
         </is>
       </c>
-      <c r="AS36" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT36" s="14" t="inlineStr">
+      <c r="AT36" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU36" s="14" t="inlineStr">
         <is>
           <t>201 Introduction to Guitar, 203 Guitar Ensemble, 206 Band, 209 String Orchestra, 220 Music Theory</t>
         </is>
@@ -6764,17 +6815,18 @@
       <c r="AO37" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP37" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP37" s="39" t="n"/>
       <c r="AQ37" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR37" s="14" t="inlineStr"/>
-      <c r="AS37" s="15" t="n">
+      <c r="AR37" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS37" s="14" t="inlineStr"/>
+      <c r="AT37" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT37" s="14" t="inlineStr">
+      <c r="AU37" s="14" t="inlineStr">
         <is>
           <t>721 U.S. History I H, 763 AP U.S. Government &amp; Politics</t>
         </is>
@@ -6938,17 +6990,18 @@
       <c r="AO38" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP38" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP38" s="39" t="n"/>
       <c r="AQ38" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR38" s="14" t="inlineStr"/>
-      <c r="AS38" s="15" t="n">
+      <c r="AR38" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS38" s="14" t="inlineStr"/>
+      <c r="AT38" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT38" s="14" t="inlineStr">
+      <c r="AU38" s="14" t="inlineStr">
         <is>
           <t>120 American Literature</t>
         </is>
@@ -7108,21 +7161,22 @@
       <c r="AO39" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AP39" s="15" t="n">
+      <c r="AP39" s="39" t="n"/>
+      <c r="AQ39" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AQ39" s="15" t="n">
+      <c r="AR39" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AR39" s="14" t="inlineStr">
+      <c r="AS39" s="14" t="inlineStr">
         <is>
           <t>585, 590, 591</t>
         </is>
       </c>
-      <c r="AS39" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT39" s="14" t="inlineStr">
+      <c r="AT39" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU39" s="14" t="inlineStr">
         <is>
           <t>570 Introduction to Robotics, 580 Robotics Engineering, 585 Robotics Design, 590 Robotics Project, 591 Robotics Project II</t>
         </is>
@@ -7282,17 +7336,18 @@
       <c r="AO40" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP40" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP40" s="39" t="n"/>
       <c r="AQ40" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR40" s="14" t="inlineStr"/>
-      <c r="AS40" s="15" t="n">
+      <c r="AR40" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS40" s="14" t="inlineStr"/>
+      <c r="AT40" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT40" s="14" t="inlineStr">
+      <c r="AU40" s="14" t="inlineStr">
         <is>
           <t>521 Chemistry H</t>
         </is>
@@ -7452,17 +7507,18 @@
       <c r="AO41" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP41" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP41" s="39" t="n"/>
       <c r="AQ41" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR41" s="14" t="inlineStr"/>
-      <c r="AS41" s="15" t="n">
+      <c r="AR41" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS41" s="14" t="inlineStr"/>
+      <c r="AT41" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT41" s="14" t="inlineStr">
+      <c r="AU41" s="14" t="inlineStr">
         <is>
           <t>720 U.S. History I</t>
         </is>
@@ -7622,21 +7678,22 @@
       <c r="AO42" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AP42" s="15" t="n">
-        <v>6</v>
-      </c>
+      <c r="AP42" s="39" t="n"/>
       <c r="AQ42" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AR42" s="14" t="inlineStr">
+      <c r="AR42" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS42" s="14" t="inlineStr">
         <is>
           <t>323, 332, 333, 352</t>
         </is>
       </c>
-      <c r="AS42" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT42" s="14" t="inlineStr">
+      <c r="AT42" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU42" s="14" t="inlineStr">
         <is>
           <t>322 Italian II, 323 Italian II H, 332 Italian III, 333 Italian III H, 352 AP Italian</t>
         </is>
@@ -7796,21 +7853,22 @@
       <c r="AO43" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP43" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP43" s="39" t="n"/>
       <c r="AQ43" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR43" s="14" t="inlineStr">
+      <c r="AR43" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS43" s="14" t="inlineStr">
         <is>
           <t>722</t>
         </is>
       </c>
-      <c r="AS43" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT43" s="14" t="inlineStr">
+      <c r="AT43" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU43" s="14" t="inlineStr">
         <is>
           <t>722 Adv U.S. History I H, 731 U.S. History II H, 733 AP U.S. History</t>
         </is>
@@ -7958,21 +8016,22 @@
       <c r="AO44" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AP44" s="15" t="n">
+      <c r="AP44" s="39" t="n"/>
+      <c r="AQ44" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AQ44" s="15" t="n">
+      <c r="AR44" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AR44" s="14" t="inlineStr">
+      <c r="AS44" s="14" t="inlineStr">
         <is>
           <t>132, 143, 145</t>
         </is>
       </c>
-      <c r="AS44" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT44" s="14" t="inlineStr">
+      <c r="AT44" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU44" s="14" t="inlineStr">
         <is>
           <t>130 British Literature, 132 British Literature, 143 Creative Writing, 145 Journalism</t>
         </is>
@@ -8140,17 +8199,18 @@
       <c r="AO45" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP45" s="15" t="n">
+      <c r="AP45" s="39" t="n"/>
+      <c r="AQ45" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AQ45" s="15" t="n">
+      <c r="AR45" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AR45" s="14" t="inlineStr"/>
-      <c r="AS45" s="15" t="n">
+      <c r="AS45" s="14" t="inlineStr"/>
+      <c r="AT45" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT45" s="14" t="inlineStr">
+      <c r="AU45" s="14" t="inlineStr">
         <is>
           <t>144 Public Speaking</t>
         </is>
@@ -8300,17 +8360,18 @@
       <c r="AO46" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP46" s="15" t="n">
-        <v>1</v>
-      </c>
+      <c r="AP46" s="39" t="n"/>
       <c r="AQ46" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AR46" s="14" t="inlineStr"/>
-      <c r="AS46" s="15" t="n">
+      <c r="AR46" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS46" s="14" t="inlineStr"/>
+      <c r="AT46" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT46" s="14" t="inlineStr">
+      <c r="AU46" s="14" t="inlineStr">
         <is>
           <t>955 Academic Support</t>
         </is>
@@ -8458,17 +8519,18 @@
       <c r="AO47" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP47" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP47" s="39" t="n"/>
       <c r="AQ47" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR47" s="14" t="inlineStr"/>
-      <c r="AS47" s="15" t="n">
+      <c r="AR47" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS47" s="14" t="inlineStr"/>
+      <c r="AT47" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT47" s="14" t="inlineStr">
+      <c r="AU47" s="14" t="inlineStr">
         <is>
           <t>410 Algebra I, 422 Geometry</t>
         </is>
@@ -8616,21 +8678,22 @@
       <c r="AO48" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP48" s="15" t="n">
-        <v>4</v>
-      </c>
+      <c r="AP48" s="39" t="n"/>
       <c r="AQ48" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AR48" s="14" t="inlineStr">
+      <c r="AR48" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS48" s="14" t="inlineStr">
         <is>
           <t>450</t>
         </is>
       </c>
-      <c r="AS48" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT48" s="14" t="inlineStr">
+      <c r="AT48" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU48" s="14" t="inlineStr">
         <is>
           <t>431 Algebra II/Trig H, 440 Precalculus, 450 Calculus H</t>
         </is>
@@ -8786,21 +8849,22 @@
       <c r="AO49" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP49" s="15" t="n">
+      <c r="AP49" s="39" t="n"/>
+      <c r="AQ49" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AQ49" s="15" t="n">
+      <c r="AR49" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AR49" s="14" t="inlineStr">
+      <c r="AS49" s="14" t="inlineStr">
         <is>
           <t>225, 228</t>
         </is>
       </c>
-      <c r="AS49" s="15" t="n">
+      <c r="AT49" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT49" s="14" t="inlineStr">
+      <c r="AU49" s="14" t="inlineStr">
         <is>
           <t>225 Tech Theater Level 1, 228 Adv Theater Production</t>
         </is>
@@ -8944,17 +9008,18 @@
       <c r="AO50" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP50" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP50" s="39" t="n"/>
       <c r="AQ50" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR50" s="14" t="inlineStr"/>
-      <c r="AS50" s="15" t="n">
+      <c r="AR50" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS50" s="14" t="inlineStr"/>
+      <c r="AT50" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT50" s="14" t="inlineStr">
+      <c r="AU50" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9, 820 Theology 10</t>
         </is>
@@ -9102,17 +9167,18 @@
       <c r="AO51" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP51" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP51" s="39" t="n"/>
       <c r="AQ51" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR51" s="14" t="inlineStr"/>
-      <c r="AS51" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT51" s="14" t="inlineStr">
+      <c r="AR51" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS51" s="14" t="inlineStr"/>
+      <c r="AT51" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU51" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11, 849 Catholic Social Teaching</t>
         </is>
@@ -9272,21 +9338,22 @@
       <c r="AO52" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP52" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP52" s="39" t="n"/>
       <c r="AQ52" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR52" s="14" t="inlineStr">
+      <c r="AR52" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS52" s="14" t="inlineStr">
         <is>
           <t>146</t>
         </is>
       </c>
-      <c r="AS52" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT52" s="14" t="inlineStr">
+      <c r="AT52" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU52" s="14" t="inlineStr">
         <is>
           <t>120 American Literature, 140 World Literature, 146 World Literature</t>
         </is>
@@ -9446,17 +9513,18 @@
       <c r="AO53" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP53" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP53" s="39" t="n"/>
       <c r="AQ53" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR53" s="14" t="inlineStr"/>
-      <c r="AS53" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT53" s="14" t="inlineStr">
+      <c r="AR53" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS53" s="14" t="inlineStr"/>
+      <c r="AT53" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU53" s="14" t="inlineStr">
         <is>
           <t>110 Composition &amp; Literature, 121 American Literature H, 149 AP English Literature</t>
         </is>
@@ -9612,17 +9680,18 @@
       <c r="AO54" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP54" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP54" s="39" t="n"/>
       <c r="AQ54" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR54" s="14" t="inlineStr"/>
-      <c r="AS54" s="15" t="n">
+      <c r="AR54" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS54" s="14" t="inlineStr"/>
+      <c r="AT54" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT54" s="14" t="inlineStr">
+      <c r="AU54" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11</t>
         </is>
@@ -9784,21 +9853,22 @@
       <c r="AO55" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AP55" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP55" s="39" t="n"/>
       <c r="AQ55" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR55" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AR55" s="14" t="inlineStr">
+      <c r="AS55" s="14" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="AS55" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT55" s="14" t="inlineStr">
+      <c r="AT55" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU55" s="14" t="inlineStr">
         <is>
           <t>2014 Multi-Media Production, 2024 TV/Film Process and Principles, 2034 TV/Film Production &amp; Editing I, 2044 TV/Film Production II, 2054 Digital Media</t>
         </is>
@@ -9958,21 +10028,22 @@
       <c r="AO56" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AP56" s="15" t="n">
+      <c r="AP56" s="39" t="n"/>
+      <c r="AQ56" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AQ56" s="15" t="n">
+      <c r="AR56" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AR56" s="14" t="inlineStr">
+      <c r="AS56" s="14" t="inlineStr">
         <is>
           <t>713, 743, 744</t>
         </is>
       </c>
-      <c r="AS56" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT56" s="14" t="inlineStr">
+      <c r="AT56" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU56" s="14" t="inlineStr">
         <is>
           <t>711 World History H, 713 AP World History, 743 AP European History, 744 Sociology, 751 American Government &amp; Politics</t>
         </is>
@@ -10132,17 +10203,18 @@
       <c r="AO57" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP57" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP57" s="39" t="n"/>
       <c r="AQ57" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR57" s="14" t="inlineStr"/>
-      <c r="AS57" s="15" t="n">
+      <c r="AR57" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS57" s="14" t="inlineStr"/>
+      <c r="AT57" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT57" s="14" t="inlineStr">
+      <c r="AU57" s="14" t="inlineStr">
         <is>
           <t>330 Spanish III, 331 Spanish III H</t>
         </is>
@@ -10290,17 +10362,18 @@
       <c r="AO58" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP58" s="15" t="n">
+      <c r="AP58" s="39" t="n"/>
+      <c r="AQ58" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AQ58" s="15" t="n">
+      <c r="AR58" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AR58" s="14" t="inlineStr"/>
-      <c r="AS58" s="15" t="n">
+      <c r="AS58" s="14" t="inlineStr"/>
+      <c r="AT58" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT58" s="14" t="inlineStr">
+      <c r="AU58" s="14" t="inlineStr">
         <is>
           <t>708 Introduction to Business</t>
         </is>
@@ -10448,17 +10521,18 @@
       <c r="AO59" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP59" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP59" s="39" t="n"/>
       <c r="AQ59" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR59" s="14" t="inlineStr"/>
-      <c r="AS59" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT59" s="14" t="inlineStr">
+      <c r="AR59" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS59" s="14" t="inlineStr"/>
+      <c r="AT59" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU59" s="14" t="inlineStr">
         <is>
           <t>710 World History, 741 Psychology, 751 American Government &amp; Politics</t>
         </is>
@@ -10614,17 +10688,18 @@
       <c r="AO60" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP60" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP60" s="39" t="n"/>
       <c r="AQ60" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR60" s="14" t="inlineStr"/>
-      <c r="AS60" s="15" t="n">
+      <c r="AR60" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS60" s="14" t="inlineStr"/>
+      <c r="AT60" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT60" s="14" t="inlineStr">
+      <c r="AU60" s="14" t="inlineStr">
         <is>
           <t>110 Composition &amp; Literature</t>
         </is>
@@ -10784,21 +10859,22 @@
       <c r="AO61" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP61" s="15" t="n">
-        <v>1</v>
-      </c>
+      <c r="AP61" s="39" t="n"/>
       <c r="AQ61" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AR61" s="14" t="inlineStr">
+      <c r="AR61" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS61" s="14" t="inlineStr">
         <is>
           <t>551</t>
         </is>
       </c>
-      <c r="AS61" s="15" t="n">
+      <c r="AT61" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT61" s="14" t="inlineStr">
+      <c r="AU61" s="14" t="inlineStr">
         <is>
           <t>551 AP Biology</t>
         </is>
@@ -10958,21 +11034,22 @@
       <c r="AO62" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP62" s="15" t="n">
-        <v>6</v>
-      </c>
+      <c r="AP62" s="39" t="n"/>
       <c r="AQ62" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AR62" s="14" t="inlineStr">
+      <c r="AR62" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS62" s="14" t="inlineStr">
         <is>
           <t>558</t>
         </is>
       </c>
-      <c r="AS62" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT62" s="14" t="inlineStr">
+      <c r="AT62" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU62" s="14" t="inlineStr">
         <is>
           <t>531 Physics H, 557 AP Physics 1, 558 AP Physics C</t>
         </is>
@@ -11132,17 +11209,18 @@
       <c r="AO63" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AP63" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP63" s="39" t="n"/>
       <c r="AQ63" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR63" s="14" t="inlineStr"/>
-      <c r="AS63" s="15" t="n">
+      <c r="AR63" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS63" s="14" t="inlineStr"/>
+      <c r="AT63" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT63" s="14" t="inlineStr">
+      <c r="AU63" s="14" t="inlineStr">
         <is>
           <t>310 Spanish I</t>
         </is>
@@ -11284,17 +11362,18 @@
       <c r="AO64" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AP64" s="15" t="n">
-        <v>0</v>
-      </c>
+      <c r="AP64" s="39" t="n"/>
       <c r="AQ64" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AR64" s="14" t="inlineStr"/>
-      <c r="AS64" s="15" t="n">
+      <c r="AR64" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS64" s="14" t="inlineStr"/>
+      <c r="AT64" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AT64" s="14" t="inlineStr"/>
+      <c r="AU64" s="14" t="inlineStr"/>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="8" t="n">
@@ -11450,17 +11529,18 @@
       <c r="AO65" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP65" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP65" s="39" t="n"/>
       <c r="AQ65" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR65" s="14" t="inlineStr"/>
-      <c r="AS65" s="15" t="n">
+      <c r="AR65" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS65" s="14" t="inlineStr"/>
+      <c r="AT65" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT65" s="14" t="inlineStr">
+      <c r="AU65" s="14" t="inlineStr">
         <is>
           <t>410 Algebra I, 411 Algebra I H</t>
         </is>
@@ -11620,21 +11700,22 @@
       <c r="AO66" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AP66" s="15" t="n">
+      <c r="AP66" s="39" t="n"/>
+      <c r="AQ66" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AQ66" s="15" t="n">
+      <c r="AR66" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AR66" s="14" t="inlineStr">
+      <c r="AS66" s="14" t="inlineStr">
         <is>
           <t>756</t>
         </is>
       </c>
-      <c r="AS66" s="15" t="n">
+      <c r="AT66" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AT66" s="14" t="inlineStr">
+      <c r="AU66" s="14" t="inlineStr">
         <is>
           <t>710 World History, 756 Introduction to Law</t>
         </is>
@@ -11794,17 +11875,18 @@
       <c r="AO67" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AP67" s="15" t="n">
-        <v>5</v>
-      </c>
+      <c r="AP67" s="39" t="n"/>
       <c r="AQ67" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AR67" s="14" t="inlineStr"/>
-      <c r="AS67" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT67" s="14" t="inlineStr">
+      <c r="AR67" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS67" s="14" t="inlineStr"/>
+      <c r="AT67" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU67" s="14" t="inlineStr">
         <is>
           <t>732 Business Law, 742 Economics, 752 Economics H</t>
         </is>
@@ -11964,21 +12046,22 @@
       <c r="AO68" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AP68" s="15" t="n">
-        <v>6</v>
-      </c>
+      <c r="AP68" s="39" t="n"/>
       <c r="AQ68" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="AR68" s="14" t="inlineStr">
+      <c r="AR68" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS68" s="14" t="inlineStr">
         <is>
           <t>315, 327, 339, 359</t>
         </is>
       </c>
-      <c r="AS68" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AT68" s="14" t="inlineStr">
+      <c r="AT68" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU68" s="14" t="inlineStr">
         <is>
           <t>312 Italian I, 315 Latin I H, 327 Latin II H, 339 Latin III H, 359 AP Latin</t>
         </is>
@@ -12116,11 +12199,12 @@
       <c r="AM69" s="36" t="n"/>
       <c r="AN69" s="36" t="n"/>
       <c r="AO69" s="36" t="n"/>
-      <c r="AP69" s="36" t="n"/>
+      <c r="AP69" s="39" t="n"/>
       <c r="AQ69" s="36" t="n"/>
       <c r="AR69" s="36" t="n"/>
       <c r="AS69" s="36" t="n"/>
       <c r="AT69" s="36" t="n"/>
+      <c r="AU69" s="36" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="35" t="n">
@@ -12254,11 +12338,12 @@
       <c r="AM70" s="36" t="n"/>
       <c r="AN70" s="36" t="n"/>
       <c r="AO70" s="36" t="n"/>
-      <c r="AP70" s="36" t="n"/>
+      <c r="AP70" s="39" t="n"/>
       <c r="AQ70" s="36" t="n"/>
       <c r="AR70" s="36" t="n"/>
       <c r="AS70" s="36" t="n"/>
       <c r="AT70" s="36" t="n"/>
+      <c r="AU70" s="36" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="21">
@@ -12336,7 +12421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13306,27 +13391,31 @@
       <c r="E38" s="21" t="inlineStr"/>
     </row>
     <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="18" t="inlineStr">
+      <c r="A39" s="20" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>S1 Load</t>
-        </is>
-      </c>
-      <c r="C39" s="24" t="inlineStr">
+      <c r="B39" s="20" t="inlineStr">
+        <is>
+          <t>Full-Year Load</t>
+        </is>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
       <c r="D39" s="20" t="inlineStr">
         <is>
-          <t>Fall semester sections. Read-only.</t>
-        </is>
-      </c>
-      <c r="E39" s="21" t="inlineStr"/>
+          <t>Total teaching periods across both semesters (full-year equivalent load)</t>
+        </is>
+      </c>
+      <c r="E39" s="20" t="inlineStr">
+        <is>
+          <t>Derived from Template 1</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="18" t="inlineStr">
@@ -13336,7 +13425,7 @@
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>S2 Load</t>
+          <t>S1 Load</t>
         </is>
       </c>
       <c r="C40" s="24" t="inlineStr">
@@ -13346,7 +13435,7 @@
       </c>
       <c r="D40" s="20" t="inlineStr">
         <is>
-          <t>Spring semester sections. Read-only.</t>
+          <t>Fall semester sections. Read-only.</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr"/>
@@ -13359,7 +13448,7 @@
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>Singleton Courses</t>
+          <t>S2 Load</t>
         </is>
       </c>
       <c r="C41" s="24" t="inlineStr">
@@ -13369,7 +13458,7 @@
       </c>
       <c r="D41" s="20" t="inlineStr">
         <is>
-          <t>Courses with only 1 section. Read-only.</t>
+          <t>Spring semester sections. Read-only.</t>
         </is>
       </c>
       <c r="E41" s="21" t="inlineStr"/>
@@ -13382,7 +13471,7 @@
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>Computed MTP Score</t>
+          <t>Singleton Courses</t>
         </is>
       </c>
       <c r="C42" s="24" t="inlineStr">
@@ -13392,7 +13481,7 @@
       </c>
       <c r="D42" s="20" t="inlineStr">
         <is>
-          <t>Engine-computed MTP (0-5). Read-only.</t>
+          <t>Courses with only 1 section. Read-only.</t>
         </is>
       </c>
       <c r="E42" s="21" t="inlineStr"/>
@@ -13405,7 +13494,7 @@
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>Courses Assigned</t>
+          <t>Computed MTP Score</t>
         </is>
       </c>
       <c r="C43" s="24" t="inlineStr">
@@ -13415,65 +13504,90 @@
       </c>
       <c r="D43" s="20" t="inlineStr">
         <is>
-          <t>Full course list from Template 1. Read-only.</t>
+          <t>Engine-computed MTP (0-5). Read-only.</t>
         </is>
       </c>
       <c r="E43" s="21" t="inlineStr"/>
     </row>
-    <row r="46">
-      <c r="A46" s="25" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="B44" s="19" t="inlineStr">
+        <is>
+          <t>Courses Assigned</t>
+        </is>
+      </c>
+      <c r="C44" s="24" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D44" s="20" t="inlineStr">
+        <is>
+          <t>Full course list from Template 1. Read-only.</t>
+        </is>
+      </c>
+      <c r="E44" s="21" t="inlineStr"/>
+    </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="25" t="inlineStr">
         <is>
           <t>COLOR LEGEND</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="26" t="n"/>
-      <c r="B47" s="19" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
-      <c r="C47" s="20" t="inlineStr">
-        <is>
-          <t>Pre-populated from engine. Do not edit unless correcting an error.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="27" t="n"/>
+      <c r="A48" s="26" t="n"/>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="C48" s="20" t="inlineStr">
         <is>
-          <t>Needs your input — currently empty.</t>
+          <t>Pre-populated from engine. Do not edit unless correcting an error.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="28" t="n"/>
+      <c r="A49" s="27" t="n"/>
       <c r="B49" s="19" t="inlineStr">
         <is>
-          <t>Light Yellow</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="C49" s="20" t="inlineStr">
         <is>
-          <t>Optional — fill in if you have the information.</t>
+          <t>Needs your input — currently empty.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="29" t="n"/>
+      <c r="A50" s="28" t="n"/>
       <c r="B50" s="19" t="inlineStr">
         <is>
+          <t>Light Yellow</t>
+        </is>
+      </c>
+      <c r="C50" s="20" t="inlineStr">
+        <is>
+          <t>Optional — fill in if you have the information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="29" t="n"/>
+      <c r="B51" s="19" t="inlineStr">
+        <is>
           <t>Gray</t>
         </is>
       </c>
-      <c r="C50" s="20" t="inlineStr">
+      <c r="C51" s="20" t="inlineStr">
         <is>
           <t>Read-only reference derived from Template 1. Do not edit.</t>
         </is>

</xml_diff>

<commit_message>
Rename Robotics/StringOrchestra to Pathway, add Teacher SSP (TSSP) scoring
Student SSP revised:
- SSP=5 LEO, SSP=4 Pathway (was Robotics/StringOrch), SSP=3 Academic Support, SSP=1 Standard
- 129 student population entries renamed in priority_assignments.json

Teacher TSSP added (mirrors student SSP):
- TSSP=5 for teachers who teach LEO courses (29 teachers)
- TSSP=4 for teachers who teach Pathway courses (34 teachers)
- TSSP=3 for teachers who teach Academic Support courses (0 — all also teach Pathway)
- TSSP=1 for standard teachers (1 teacher: Sabella)
- TSSP and Serving Populations added to teacher_priorities in JSON
- Columns AU (Computed TSSP Score) and AV (Serving Populations) added to Template 6

Updated COMMERCIAL_PRODUCT_SPEC.md references to match

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -191,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -293,6 +293,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -659,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU70"/>
+  <dimension ref="A1:AW70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -705,6 +708,8 @@
     <col width="18" customWidth="1" min="41" max="41"/>
     <col width="10" customWidth="1" min="42" max="42"/>
     <col width="35" customWidth="1" min="43" max="43"/>
+    <col width="10" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -952,7 +957,17 @@
           <t>Computed MTP Score</t>
         </is>
       </c>
-      <c r="AU3" s="3" t="inlineStr">
+      <c r="AU3" s="30" t="inlineStr">
+        <is>
+          <t>Computed TSSP Score</t>
+        </is>
+      </c>
+      <c r="AV3" s="30" t="inlineStr">
+        <is>
+          <t>Serving Populations</t>
+        </is>
+      </c>
+      <c r="AW3" s="3" t="inlineStr">
         <is>
           <t>Courses Assigned</t>
         </is>
@@ -1189,7 +1204,17 @@
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="AU4" s="6" t="inlineStr">
+      <c r="AU4" s="32" t="inlineStr">
+        <is>
+          <t>REFERENCE</t>
+        </is>
+      </c>
+      <c r="AV4" s="32" t="inlineStr">
+        <is>
+          <t>REFERENCE</t>
+        </is>
+      </c>
+      <c r="AW4" s="6" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
@@ -1364,7 +1389,15 @@
       <c r="AT5" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU5" s="14" t="inlineStr">
+      <c r="AU5" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV5" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW5" s="14" t="inlineStr">
         <is>
           <t>421 Geometry H, 425 Adv Geometry H, 445 Adv Precalculus H</t>
         </is>
@@ -1523,7 +1556,15 @@
       <c r="AT6" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU6" s="14" t="inlineStr">
+      <c r="AU6" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV6" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW6" s="14" t="inlineStr">
         <is>
           <t>321 Spanish II H, 330 Spanish III, 351 AP Spanish</t>
         </is>
@@ -1692,7 +1733,15 @@
       <c r="AT7" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU7" s="14" t="inlineStr">
+      <c r="AU7" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV7" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW7" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9</t>
         </is>
@@ -1859,7 +1908,15 @@
       <c r="AT8" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU8" s="14" t="inlineStr">
+      <c r="AU8" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV8" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW8" s="14" t="inlineStr">
         <is>
           <t>610 Health/PE</t>
         </is>
@@ -2034,7 +2091,15 @@
       <c r="AT9" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU9" s="14" t="inlineStr">
+      <c r="AU9" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV9" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW9" s="14" t="inlineStr">
         <is>
           <t>472 Web Design, 473 Introduction to Programming, 490 AP Computer Science A, 491 AP Computer Science Principles, 494 Applied Programming, 496 AP Cybersecurity</t>
         </is>
@@ -2209,7 +2274,15 @@
       <c r="AT10" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU10" s="14" t="inlineStr">
+      <c r="AU10" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV10" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW10" s="14" t="inlineStr">
         <is>
           <t>431 Algebra II/Trig H, 453 AP Calc AB, 455 AP Calc BC</t>
         </is>
@@ -2384,7 +2457,15 @@
       <c r="AT11" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU11" s="14" t="inlineStr">
+      <c r="AU11" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV11" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW11" s="14" t="inlineStr">
         <is>
           <t>311 Spanish I H, 320 Spanish II</t>
         </is>
@@ -2555,7 +2636,15 @@
       <c r="AT12" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU12" s="14" t="inlineStr">
+      <c r="AU12" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV12" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW12" s="14" t="inlineStr">
         <is>
           <t>631 CPR-AED Training/PE, 642 Nutrition &amp; Fitness/PE</t>
         </is>
@@ -2730,7 +2819,15 @@
       <c r="AT13" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU13" s="14" t="inlineStr">
+      <c r="AU13" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV13" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW13" s="14" t="inlineStr">
         <is>
           <t>544 Sports Medicine, 546 Forensics</t>
         </is>
@@ -2901,7 +2998,15 @@
       <c r="AT14" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU14" s="14" t="inlineStr">
+      <c r="AU14" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV14" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW14" s="14" t="inlineStr">
         <is>
           <t>727 Sports and Entertainment Marketing, 757 International Business Strategies, 758 Bloomberg Market Concepts</t>
         </is>
@@ -3072,7 +3177,15 @@
       <c r="AT15" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU15" s="14" t="inlineStr">
+      <c r="AU15" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV15" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW15" s="14" t="inlineStr">
         <is>
           <t>620 Driver's Ed/PE</t>
         </is>
@@ -3231,7 +3344,15 @@
       <c r="AT16" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU16" s="14" t="inlineStr">
+      <c r="AU16" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV16" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW16" s="14" t="inlineStr">
         <is>
           <t>412 Algebra I, 432 Algebra II/Trig</t>
         </is>
@@ -3402,7 +3523,15 @@
       <c r="AT17" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU17" s="14" t="inlineStr">
+      <c r="AU17" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV17" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW17" s="14" t="inlineStr">
         <is>
           <t>111 Composition &amp; Literature H, 129 AP Seminar</t>
         </is>
@@ -3577,7 +3706,15 @@
       <c r="AT18" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU18" s="14" t="inlineStr">
+      <c r="AU18" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV18" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW18" s="14" t="inlineStr">
         <is>
           <t>241 Studio Art I, 242 Studio Art II, 243 Studio Art III, 248 Adv Drawing, 249 Adv Painting, 253 AP Drawing, 254 AP 2-D Art and Design, 255 AP 3-D Art and Design, 764 AP Art History</t>
         </is>
@@ -3748,7 +3885,15 @@
       <c r="AT19" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU19" s="14" t="inlineStr">
+      <c r="AU19" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV19" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW19" s="14" t="inlineStr">
         <is>
           <t>520 Chemistry</t>
         </is>
@@ -3919,7 +4064,15 @@
       <c r="AT20" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU20" s="14" t="inlineStr">
+      <c r="AU20" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV20" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW20" s="14" t="inlineStr">
         <is>
           <t>130 British Literature, 141 College English Honors</t>
         </is>
@@ -4090,7 +4243,15 @@
       <c r="AT21" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU21" s="14" t="inlineStr">
+      <c r="AU21" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV21" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW21" s="14" t="inlineStr">
         <is>
           <t>726 Business Concepts, 729 AP Business with Personal Finance, 734 Leadership, Entrepreneurship and Opportunity Program I, 745 Leadership, Entrepreneurship and Opportunity Program II</t>
         </is>
@@ -4261,7 +4422,15 @@
       <c r="AT22" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU22" s="14" t="inlineStr">
+      <c r="AU22" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV22" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW22" s="14" t="inlineStr">
         <is>
           <t>131 British Literature H, 139 AP English Language</t>
         </is>
@@ -4432,7 +4601,15 @@
       <c r="AT23" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU23" s="14" t="inlineStr">
+      <c r="AU23" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV23" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW23" s="14" t="inlineStr">
         <is>
           <t>420 Geometry, 440 Precalculus</t>
         </is>
@@ -4607,7 +4784,15 @@
       <c r="AT24" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU24" s="14" t="inlineStr">
+      <c r="AU24" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV24" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW24" s="14" t="inlineStr">
         <is>
           <t>435 Adv Algebra II / Trig H, 440 Precalculus, 448 Pre-college Math</t>
         </is>
@@ -4770,7 +4955,15 @@
       <c r="AT25" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU25" s="14" t="inlineStr">
+      <c r="AU25" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV25" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW25" s="14" t="inlineStr">
         <is>
           <t>542 Anatomy/Physiology, 543 Anatomy/Physiology H</t>
         </is>
@@ -4941,7 +5134,15 @@
       <c r="AT26" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU26" s="14" t="inlineStr">
+      <c r="AU26" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV26" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW26" s="14" t="inlineStr">
         <is>
           <t>430 Algebra II/Trig, 443 AP Precalculus</t>
         </is>
@@ -5116,7 +5317,15 @@
       <c r="AT27" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU27" s="14" t="inlineStr">
+      <c r="AU27" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV27" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW27" s="14" t="inlineStr">
         <is>
           <t>730 U.S. History II, 731 U.S. History II H, 761 AP Psychology</t>
         </is>
@@ -5291,7 +5500,15 @@
       <c r="AT28" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU28" s="14" t="inlineStr">
+      <c r="AU28" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV28" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW28" s="14" t="inlineStr">
         <is>
           <t>500 Earth Science, 510 Biology</t>
         </is>
@@ -5462,7 +5679,15 @@
       <c r="AT29" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU29" s="14" t="inlineStr">
+      <c r="AU29" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV29" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW29" s="14" t="inlineStr">
         <is>
           <t>112 Composition &amp; Literature, 122 American Literature, 955 Academic Support</t>
         </is>
@@ -5637,7 +5862,15 @@
       <c r="AT30" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU30" s="14" t="inlineStr">
+      <c r="AU30" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV30" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW30" s="14" t="inlineStr">
         <is>
           <t>511 Biology H, 553 AP Chemistry</t>
         </is>
@@ -5808,7 +6041,15 @@
       <c r="AT31" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU31" s="14" t="inlineStr">
+      <c r="AU31" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV31" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW31" s="14" t="inlineStr">
         <is>
           <t>456 AP Statistics, 765 AP Macroeconomics, 766 AP Microeconomics</t>
         </is>
@@ -5991,7 +6232,15 @@
       <c r="AT32" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU32" s="14" t="inlineStr">
+      <c r="AU32" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV32" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW32" s="14" t="inlineStr">
         <is>
           <t>530 Physics, 595 Engineering Design</t>
         </is>
@@ -6158,7 +6407,15 @@
       <c r="AT33" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU33" s="14" t="inlineStr">
+      <c r="AU33" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV33" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW33" s="14" t="inlineStr">
         <is>
           <t>820 Theology 10, 830 Theology 11</t>
         </is>
@@ -6329,7 +6586,15 @@
       <c r="AT34" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU34" s="14" t="inlineStr">
+      <c r="AU34" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV34" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW34" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11, 851 Spirituality of Vocation</t>
         </is>
@@ -6496,7 +6761,15 @@
       <c r="AT35" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU35" s="14" t="inlineStr">
+      <c r="AU35" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV35" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW35" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9, 820 Theology 10</t>
         </is>
@@ -6667,7 +6940,15 @@
       <c r="AT36" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU36" s="14" t="inlineStr">
+      <c r="AU36" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV36" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW36" s="14" t="inlineStr">
         <is>
           <t>201 Introduction to Guitar, 203 Guitar Ensemble, 206 Band, 209 String Orchestra, 220 Music Theory</t>
         </is>
@@ -6826,7 +7107,15 @@
       <c r="AT37" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU37" s="14" t="inlineStr">
+      <c r="AU37" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV37" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW37" s="14" t="inlineStr">
         <is>
           <t>721 U.S. History I H, 763 AP U.S. Government &amp; Politics</t>
         </is>
@@ -7001,7 +7290,15 @@
       <c r="AT38" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU38" s="14" t="inlineStr">
+      <c r="AU38" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV38" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW38" s="14" t="inlineStr">
         <is>
           <t>120 American Literature</t>
         </is>
@@ -7176,7 +7473,15 @@
       <c r="AT39" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU39" s="14" t="inlineStr">
+      <c r="AU39" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV39" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW39" s="14" t="inlineStr">
         <is>
           <t>570 Introduction to Robotics, 580 Robotics Engineering, 585 Robotics Design, 590 Robotics Project, 591 Robotics Project II</t>
         </is>
@@ -7347,7 +7652,15 @@
       <c r="AT40" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU40" s="14" t="inlineStr">
+      <c r="AU40" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV40" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW40" s="14" t="inlineStr">
         <is>
           <t>521 Chemistry H</t>
         </is>
@@ -7518,7 +7831,15 @@
       <c r="AT41" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU41" s="14" t="inlineStr">
+      <c r="AU41" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV41" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW41" s="14" t="inlineStr">
         <is>
           <t>720 U.S. History I</t>
         </is>
@@ -7693,7 +8014,15 @@
       <c r="AT42" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU42" s="14" t="inlineStr">
+      <c r="AU42" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV42" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW42" s="14" t="inlineStr">
         <is>
           <t>322 Italian II, 323 Italian II H, 332 Italian III, 333 Italian III H, 352 AP Italian</t>
         </is>
@@ -7868,7 +8197,15 @@
       <c r="AT43" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU43" s="14" t="inlineStr">
+      <c r="AU43" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV43" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW43" s="14" t="inlineStr">
         <is>
           <t>722 Adv U.S. History I H, 731 U.S. History II H, 733 AP U.S. History</t>
         </is>
@@ -8031,7 +8368,11 @@
       <c r="AT44" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU44" s="14" t="inlineStr">
+      <c r="AU44" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV44" s="40" t="inlineStr"/>
+      <c r="AW44" s="14" t="inlineStr">
         <is>
           <t>130 British Literature, 132 British Literature, 143 Creative Writing, 145 Journalism</t>
         </is>
@@ -8210,7 +8551,11 @@
       <c r="AT45" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU45" s="14" t="inlineStr">
+      <c r="AU45" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV45" s="40" t="inlineStr"/>
+      <c r="AW45" s="14" t="inlineStr">
         <is>
           <t>144 Public Speaking</t>
         </is>
@@ -8371,7 +8716,15 @@
       <c r="AT46" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU46" s="14" t="inlineStr">
+      <c r="AU46" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV46" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW46" s="14" t="inlineStr">
         <is>
           <t>955 Academic Support</t>
         </is>
@@ -8530,7 +8883,11 @@
       <c r="AT47" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU47" s="14" t="inlineStr">
+      <c r="AU47" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV47" s="40" t="inlineStr"/>
+      <c r="AW47" s="14" t="inlineStr">
         <is>
           <t>410 Algebra I, 422 Geometry</t>
         </is>
@@ -8693,7 +9050,11 @@
       <c r="AT48" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU48" s="14" t="inlineStr">
+      <c r="AU48" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV48" s="40" t="inlineStr"/>
+      <c r="AW48" s="14" t="inlineStr">
         <is>
           <t>431 Algebra II/Trig H, 440 Precalculus, 450 Calculus H</t>
         </is>
@@ -8864,7 +9225,11 @@
       <c r="AT49" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU49" s="14" t="inlineStr">
+      <c r="AU49" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV49" s="40" t="inlineStr"/>
+      <c r="AW49" s="14" t="inlineStr">
         <is>
           <t>225 Tech Theater Level 1, 228 Adv Theater Production</t>
         </is>
@@ -9019,7 +9384,11 @@
       <c r="AT50" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU50" s="14" t="inlineStr">
+      <c r="AU50" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV50" s="40" t="inlineStr"/>
+      <c r="AW50" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9, 820 Theology 10</t>
         </is>
@@ -9178,7 +9547,11 @@
       <c r="AT51" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU51" s="14" t="inlineStr">
+      <c r="AU51" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV51" s="40" t="inlineStr"/>
+      <c r="AW51" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11, 849 Catholic Social Teaching</t>
         </is>
@@ -9353,7 +9726,15 @@
       <c r="AT52" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU52" s="14" t="inlineStr">
+      <c r="AU52" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV52" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW52" s="14" t="inlineStr">
         <is>
           <t>120 American Literature, 140 World Literature, 146 World Literature</t>
         </is>
@@ -9524,7 +9905,15 @@
       <c r="AT53" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU53" s="14" t="inlineStr">
+      <c r="AU53" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV53" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW53" s="14" t="inlineStr">
         <is>
           <t>110 Composition &amp; Literature, 121 American Literature H, 149 AP English Literature</t>
         </is>
@@ -9691,7 +10080,15 @@
       <c r="AT54" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU54" s="14" t="inlineStr">
+      <c r="AU54" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV54" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW54" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11</t>
         </is>
@@ -9868,7 +10265,15 @@
       <c r="AT55" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU55" s="14" t="inlineStr">
+      <c r="AU55" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV55" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW55" s="14" t="inlineStr">
         <is>
           <t>2014 Multi-Media Production, 2024 TV/Film Process and Principles, 2034 TV/Film Production &amp; Editing I, 2044 TV/Film Production II, 2054 Digital Media</t>
         </is>
@@ -10043,7 +10448,15 @@
       <c r="AT56" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU56" s="14" t="inlineStr">
+      <c r="AU56" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV56" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW56" s="14" t="inlineStr">
         <is>
           <t>711 World History H, 713 AP World History, 743 AP European History, 744 Sociology, 751 American Government &amp; Politics</t>
         </is>
@@ -10214,7 +10627,15 @@
       <c r="AT57" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU57" s="14" t="inlineStr">
+      <c r="AU57" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV57" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW57" s="14" t="inlineStr">
         <is>
           <t>330 Spanish III, 331 Spanish III H</t>
         </is>
@@ -10373,7 +10794,11 @@
       <c r="AT58" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU58" s="14" t="inlineStr">
+      <c r="AU58" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV58" s="40" t="inlineStr"/>
+      <c r="AW58" s="14" t="inlineStr">
         <is>
           <t>708 Introduction to Business</t>
         </is>
@@ -10532,7 +10957,15 @@
       <c r="AT59" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU59" s="14" t="inlineStr">
+      <c r="AU59" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV59" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW59" s="14" t="inlineStr">
         <is>
           <t>710 World History, 741 Psychology, 751 American Government &amp; Politics</t>
         </is>
@@ -10699,7 +11132,15 @@
       <c r="AT60" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU60" s="14" t="inlineStr">
+      <c r="AU60" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV60" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW60" s="14" t="inlineStr">
         <is>
           <t>110 Composition &amp; Literature</t>
         </is>
@@ -10874,7 +11315,15 @@
       <c r="AT61" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU61" s="14" t="inlineStr">
+      <c r="AU61" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV61" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW61" s="14" t="inlineStr">
         <is>
           <t>551 AP Biology</t>
         </is>
@@ -11049,7 +11498,15 @@
       <c r="AT62" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU62" s="14" t="inlineStr">
+      <c r="AU62" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV62" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW62" s="14" t="inlineStr">
         <is>
           <t>531 Physics H, 557 AP Physics 1, 558 AP Physics C</t>
         </is>
@@ -11220,7 +11677,15 @@
       <c r="AT63" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU63" s="14" t="inlineStr">
+      <c r="AU63" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV63" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW63" s="14" t="inlineStr">
         <is>
           <t>310 Spanish I</t>
         </is>
@@ -11373,7 +11838,15 @@
       <c r="AT64" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU64" s="14" t="inlineStr"/>
+      <c r="AU64" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV64" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW64" s="14" t="inlineStr"/>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="8" t="n">
@@ -11540,7 +12013,15 @@
       <c r="AT65" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU65" s="14" t="inlineStr">
+      <c r="AU65" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV65" s="40" t="inlineStr">
+        <is>
+          <t>Pathway</t>
+        </is>
+      </c>
+      <c r="AW65" s="14" t="inlineStr">
         <is>
           <t>410 Algebra I, 411 Algebra I H</t>
         </is>
@@ -11715,7 +12196,15 @@
       <c r="AT66" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="AU66" s="14" t="inlineStr">
+      <c r="AU66" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV66" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW66" s="14" t="inlineStr">
         <is>
           <t>710 World History, 756 Introduction to Law</t>
         </is>
@@ -11886,7 +12375,15 @@
       <c r="AT67" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU67" s="14" t="inlineStr">
+      <c r="AU67" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV67" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW67" s="14" t="inlineStr">
         <is>
           <t>732 Business Law, 742 Economics, 752 Economics H</t>
         </is>
@@ -12061,7 +12558,15 @@
       <c r="AT68" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="AU68" s="14" t="inlineStr">
+      <c r="AU68" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV68" s="40" t="inlineStr">
+        <is>
+          <t>LEO, Pathway</t>
+        </is>
+      </c>
+      <c r="AW68" s="14" t="inlineStr">
         <is>
           <t>312 Italian I, 315 Latin I H, 327 Latin II H, 339 Latin III H, 359 AP Latin</t>
         </is>
@@ -12204,7 +12709,11 @@
       <c r="AR69" s="36" t="n"/>
       <c r="AS69" s="36" t="n"/>
       <c r="AT69" s="36" t="n"/>
-      <c r="AU69" s="36" t="n"/>
+      <c r="AU69" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV69" s="40" t="inlineStr"/>
+      <c r="AW69" s="36" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="35" t="n">
@@ -12343,7 +12852,11 @@
       <c r="AR70" s="36" t="n"/>
       <c r="AS70" s="36" t="n"/>
       <c r="AT70" s="36" t="n"/>
-      <c r="AU70" s="36" t="n"/>
+      <c r="AU70" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV70" s="40" t="inlineStr"/>
+      <c r="AW70" s="36" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="21">
@@ -12421,7 +12934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13510,84 +14023,138 @@
       <c r="E43" s="21" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="18" t="inlineStr">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>AU</t>
         </is>
       </c>
-      <c r="B44" s="19" t="inlineStr">
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>Computed TSSP Score</t>
+        </is>
+      </c>
+      <c r="C44" s="20" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D44" s="20" t="inlineStr">
+        <is>
+          <t>Teacher Special Population Priority: 5=teaches LEO courses, 4=teaches Pathway courses, 3=teaches Academic Support courses, 1=standard</t>
+        </is>
+      </c>
+      <c r="E44" s="20" t="inlineStr">
+        <is>
+          <t>1, 3, 4, 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>AV</t>
+        </is>
+      </c>
+      <c r="B45" s="20" t="inlineStr">
+        <is>
+          <t>Serving Populations</t>
+        </is>
+      </c>
+      <c r="C45" s="20" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D45" s="20" t="inlineStr">
+        <is>
+          <t>Which special populations this teacher serves based on their course assignments</t>
+        </is>
+      </c>
+      <c r="E45" s="20" t="inlineStr">
+        <is>
+          <t>LEO, Pathway, AcademicSupport</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="18" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="inlineStr">
         <is>
           <t>Courses Assigned</t>
         </is>
       </c>
-      <c r="C44" s="24" t="inlineStr">
+      <c r="C46" s="24" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="D44" s="20" t="inlineStr">
+      <c r="D46" s="20" t="inlineStr">
         <is>
           <t>Full course list from Template 1. Read-only.</t>
         </is>
       </c>
-      <c r="E44" s="21" t="inlineStr"/>
+      <c r="E46" s="21" t="inlineStr"/>
     </row>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47">
-      <c r="A47" s="25" t="inlineStr">
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="25" t="inlineStr">
         <is>
           <t>COLOR LEGEND</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="26" t="n"/>
-      <c r="B48" s="19" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
-      <c r="C48" s="20" t="inlineStr">
-        <is>
-          <t>Pre-populated from engine. Do not edit unless correcting an error.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="27" t="n"/>
-      <c r="B49" s="19" t="inlineStr">
-        <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="C49" s="20" t="inlineStr">
-        <is>
-          <t>Needs your input — currently empty.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="28" t="n"/>
+      <c r="A50" s="26" t="n"/>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>Light Yellow</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr">
         <is>
-          <t>Optional — fill in if you have the information.</t>
+          <t>Pre-populated from engine. Do not edit unless correcting an error.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="29" t="n"/>
+      <c r="A51" s="27" t="n"/>
       <c r="B51" s="19" t="inlineStr">
         <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="C51" s="20" t="inlineStr">
+        <is>
+          <t>Needs your input — currently empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="28" t="n"/>
+      <c r="B52" s="19" t="inlineStr">
+        <is>
+          <t>Light Yellow</t>
+        </is>
+      </c>
+      <c r="C52" s="20" t="inlineStr">
+        <is>
+          <t>Optional — fill in if you have the information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="29" t="n"/>
+      <c r="B53" s="19" t="inlineStr">
+        <is>
           <t>Gray</t>
         </is>
       </c>
-      <c r="C51" s="20" t="inlineStr">
+      <c r="C53" s="20" t="inlineStr">
         <is>
           <t>Read-only reference derived from Template 1. Do not edit.</t>
         </is>

</xml_diff>

<commit_message>
Add multi-membership SSP columns for students and teachers
Students (Template 8):
- Added column L: Pathway (Y/N) — 129 students pre-filled
- Added column M: Academic Support (Y/N) — 0 students (to be filled)
- SSP (col G) label updated to show MAX(LEO=5,Path=4,Acad=3,Std=1)
- A student can be a member of 1, 2, or all 3 populations

Teachers (Template 6):
- Replaced single "Serving Populations" text column with 3 editable Y/N
  columns: Teaches LEO (AV), Teaches Pathway (AW), Teaches Acad Support (AX)
- TSSP score (AU) = MAX of assigned populations
- Fixed 7 former-TBD teachers (Gioni, Ferrante-Martin, Oh, Hartmann,
  Austria, Granieri, Junis) whose TSSP was incorrectly 1
- A teacher can teach across 1, 2, or all 3 populations

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW70"/>
+  <dimension ref="A1:AY70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -709,7 +709,9 @@
     <col width="10" customWidth="1" min="42" max="42"/>
     <col width="35" customWidth="1" min="43" max="43"/>
     <col width="10" customWidth="1" min="47" max="47"/>
-    <col width="20" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
+    <col width="12" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -964,10 +966,20 @@
       </c>
       <c r="AV3" s="30" t="inlineStr">
         <is>
-          <t>Serving Populations</t>
-        </is>
-      </c>
-      <c r="AW3" s="3" t="inlineStr">
+          <t>Teaches LEO</t>
+        </is>
+      </c>
+      <c r="AW3" s="30" t="inlineStr">
+        <is>
+          <t>Teaches Pathway</t>
+        </is>
+      </c>
+      <c r="AX3" s="30" t="inlineStr">
+        <is>
+          <t>Teaches Acad Support</t>
+        </is>
+      </c>
+      <c r="AY3" s="3" t="inlineStr">
         <is>
           <t>Courses Assigned</t>
         </is>
@@ -1211,10 +1223,20 @@
       </c>
       <c r="AV4" s="32" t="inlineStr">
         <is>
-          <t>REFERENCE</t>
-        </is>
-      </c>
-      <c r="AW4" s="6" t="inlineStr">
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="AW4" s="32" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="AX4" s="32" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="AY4" s="6" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
@@ -1392,12 +1414,22 @@
       <c r="AU5" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV5" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW5" s="14" t="inlineStr">
+      <c r="AV5" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW5" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX5" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY5" s="14" t="inlineStr">
         <is>
           <t>421 Geometry H, 425 Adv Geometry H, 445 Adv Precalculus H</t>
         </is>
@@ -1559,12 +1591,22 @@
       <c r="AU6" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV6" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW6" s="14" t="inlineStr">
+      <c r="AV6" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW6" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX6" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY6" s="14" t="inlineStr">
         <is>
           <t>321 Spanish II H, 330 Spanish III, 351 AP Spanish</t>
         </is>
@@ -1736,12 +1778,22 @@
       <c r="AU7" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV7" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW7" s="14" t="inlineStr">
+      <c r="AV7" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW7" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX7" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY7" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9</t>
         </is>
@@ -1911,12 +1963,22 @@
       <c r="AU8" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV8" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW8" s="14" t="inlineStr">
+      <c r="AV8" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW8" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX8" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY8" s="14" t="inlineStr">
         <is>
           <t>610 Health/PE</t>
         </is>
@@ -2094,12 +2156,22 @@
       <c r="AU9" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV9" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW9" s="14" t="inlineStr">
+      <c r="AV9" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW9" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX9" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY9" s="14" t="inlineStr">
         <is>
           <t>472 Web Design, 473 Introduction to Programming, 490 AP Computer Science A, 491 AP Computer Science Principles, 494 Applied Programming, 496 AP Cybersecurity</t>
         </is>
@@ -2277,12 +2349,22 @@
       <c r="AU10" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV10" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW10" s="14" t="inlineStr">
+      <c r="AV10" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW10" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX10" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY10" s="14" t="inlineStr">
         <is>
           <t>431 Algebra II/Trig H, 453 AP Calc AB, 455 AP Calc BC</t>
         </is>
@@ -2460,12 +2542,22 @@
       <c r="AU11" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV11" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW11" s="14" t="inlineStr">
+      <c r="AV11" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW11" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX11" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY11" s="14" t="inlineStr">
         <is>
           <t>311 Spanish I H, 320 Spanish II</t>
         </is>
@@ -2639,12 +2731,22 @@
       <c r="AU12" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV12" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW12" s="14" t="inlineStr">
+      <c r="AV12" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW12" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX12" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY12" s="14" t="inlineStr">
         <is>
           <t>631 CPR-AED Training/PE, 642 Nutrition &amp; Fitness/PE</t>
         </is>
@@ -2822,12 +2924,22 @@
       <c r="AU13" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV13" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW13" s="14" t="inlineStr">
+      <c r="AV13" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW13" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX13" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY13" s="14" t="inlineStr">
         <is>
           <t>544 Sports Medicine, 546 Forensics</t>
         </is>
@@ -3001,12 +3113,22 @@
       <c r="AU14" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV14" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW14" s="14" t="inlineStr">
+      <c r="AV14" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW14" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX14" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY14" s="14" t="inlineStr">
         <is>
           <t>727 Sports and Entertainment Marketing, 757 International Business Strategies, 758 Bloomberg Market Concepts</t>
         </is>
@@ -3180,12 +3302,22 @@
       <c r="AU15" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV15" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW15" s="14" t="inlineStr">
+      <c r="AV15" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW15" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX15" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY15" s="14" t="inlineStr">
         <is>
           <t>620 Driver's Ed/PE</t>
         </is>
@@ -3347,12 +3479,22 @@
       <c r="AU16" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV16" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW16" s="14" t="inlineStr">
+      <c r="AV16" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW16" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX16" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY16" s="14" t="inlineStr">
         <is>
           <t>412 Algebra I, 432 Algebra II/Trig</t>
         </is>
@@ -3526,12 +3668,22 @@
       <c r="AU17" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV17" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW17" s="14" t="inlineStr">
+      <c r="AV17" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW17" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX17" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY17" s="14" t="inlineStr">
         <is>
           <t>111 Composition &amp; Literature H, 129 AP Seminar</t>
         </is>
@@ -3709,12 +3861,22 @@
       <c r="AU18" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV18" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW18" s="14" t="inlineStr">
+      <c r="AV18" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW18" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX18" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY18" s="14" t="inlineStr">
         <is>
           <t>241 Studio Art I, 242 Studio Art II, 243 Studio Art III, 248 Adv Drawing, 249 Adv Painting, 253 AP Drawing, 254 AP 2-D Art and Design, 255 AP 3-D Art and Design, 764 AP Art History</t>
         </is>
@@ -3888,12 +4050,22 @@
       <c r="AU19" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV19" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW19" s="14" t="inlineStr">
+      <c r="AV19" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW19" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX19" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY19" s="14" t="inlineStr">
         <is>
           <t>520 Chemistry</t>
         </is>
@@ -4067,12 +4239,22 @@
       <c r="AU20" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV20" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW20" s="14" t="inlineStr">
+      <c r="AV20" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW20" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX20" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY20" s="14" t="inlineStr">
         <is>
           <t>130 British Literature, 141 College English Honors</t>
         </is>
@@ -4246,12 +4428,22 @@
       <c r="AU21" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV21" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW21" s="14" t="inlineStr">
+      <c r="AV21" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW21" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX21" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY21" s="14" t="inlineStr">
         <is>
           <t>726 Business Concepts, 729 AP Business with Personal Finance, 734 Leadership, Entrepreneurship and Opportunity Program I, 745 Leadership, Entrepreneurship and Opportunity Program II</t>
         </is>
@@ -4425,12 +4617,22 @@
       <c r="AU22" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV22" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW22" s="14" t="inlineStr">
+      <c r="AV22" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW22" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX22" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY22" s="14" t="inlineStr">
         <is>
           <t>131 British Literature H, 139 AP English Language</t>
         </is>
@@ -4604,12 +4806,22 @@
       <c r="AU23" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV23" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW23" s="14" t="inlineStr">
+      <c r="AV23" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW23" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX23" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY23" s="14" t="inlineStr">
         <is>
           <t>420 Geometry, 440 Precalculus</t>
         </is>
@@ -4787,12 +4999,22 @@
       <c r="AU24" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV24" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW24" s="14" t="inlineStr">
+      <c r="AV24" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW24" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX24" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY24" s="14" t="inlineStr">
         <is>
           <t>435 Adv Algebra II / Trig H, 440 Precalculus, 448 Pre-college Math</t>
         </is>
@@ -4958,12 +5180,22 @@
       <c r="AU25" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV25" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW25" s="14" t="inlineStr">
+      <c r="AV25" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW25" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX25" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY25" s="14" t="inlineStr">
         <is>
           <t>542 Anatomy/Physiology, 543 Anatomy/Physiology H</t>
         </is>
@@ -5137,12 +5369,22 @@
       <c r="AU26" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV26" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW26" s="14" t="inlineStr">
+      <c r="AV26" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW26" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX26" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY26" s="14" t="inlineStr">
         <is>
           <t>430 Algebra II/Trig, 443 AP Precalculus</t>
         </is>
@@ -5320,12 +5562,22 @@
       <c r="AU27" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV27" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW27" s="14" t="inlineStr">
+      <c r="AV27" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW27" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX27" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY27" s="14" t="inlineStr">
         <is>
           <t>730 U.S. History II, 731 U.S. History II H, 761 AP Psychology</t>
         </is>
@@ -5503,12 +5755,22 @@
       <c r="AU28" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV28" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW28" s="14" t="inlineStr">
+      <c r="AV28" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW28" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX28" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY28" s="14" t="inlineStr">
         <is>
           <t>500 Earth Science, 510 Biology</t>
         </is>
@@ -5682,12 +5944,22 @@
       <c r="AU29" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV29" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW29" s="14" t="inlineStr">
+      <c r="AV29" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW29" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX29" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY29" s="14" t="inlineStr">
         <is>
           <t>112 Composition &amp; Literature, 122 American Literature, 955 Academic Support</t>
         </is>
@@ -5865,12 +6137,22 @@
       <c r="AU30" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV30" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW30" s="14" t="inlineStr">
+      <c r="AV30" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW30" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX30" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY30" s="14" t="inlineStr">
         <is>
           <t>511 Biology H, 553 AP Chemistry</t>
         </is>
@@ -6044,12 +6326,22 @@
       <c r="AU31" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV31" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW31" s="14" t="inlineStr">
+      <c r="AV31" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW31" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX31" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY31" s="14" t="inlineStr">
         <is>
           <t>456 AP Statistics, 765 AP Macroeconomics, 766 AP Microeconomics</t>
         </is>
@@ -6235,12 +6527,22 @@
       <c r="AU32" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV32" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW32" s="14" t="inlineStr">
+      <c r="AV32" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW32" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX32" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY32" s="14" t="inlineStr">
         <is>
           <t>530 Physics, 595 Engineering Design</t>
         </is>
@@ -6410,12 +6712,22 @@
       <c r="AU33" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV33" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW33" s="14" t="inlineStr">
+      <c r="AV33" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW33" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX33" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY33" s="14" t="inlineStr">
         <is>
           <t>820 Theology 10, 830 Theology 11</t>
         </is>
@@ -6589,12 +6901,22 @@
       <c r="AU34" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV34" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW34" s="14" t="inlineStr">
+      <c r="AV34" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW34" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX34" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY34" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11, 851 Spirituality of Vocation</t>
         </is>
@@ -6764,12 +7086,22 @@
       <c r="AU35" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV35" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW35" s="14" t="inlineStr">
+      <c r="AV35" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW35" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX35" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY35" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9, 820 Theology 10</t>
         </is>
@@ -6943,12 +7275,22 @@
       <c r="AU36" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV36" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW36" s="14" t="inlineStr">
+      <c r="AV36" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW36" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX36" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY36" s="14" t="inlineStr">
         <is>
           <t>201 Introduction to Guitar, 203 Guitar Ensemble, 206 Band, 209 String Orchestra, 220 Music Theory</t>
         </is>
@@ -7110,12 +7452,22 @@
       <c r="AU37" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV37" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW37" s="14" t="inlineStr">
+      <c r="AV37" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW37" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX37" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY37" s="14" t="inlineStr">
         <is>
           <t>721 U.S. History I H, 763 AP U.S. Government &amp; Politics</t>
         </is>
@@ -7293,12 +7645,22 @@
       <c r="AU38" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV38" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW38" s="14" t="inlineStr">
+      <c r="AV38" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW38" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX38" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY38" s="14" t="inlineStr">
         <is>
           <t>120 American Literature</t>
         </is>
@@ -7476,12 +7838,22 @@
       <c r="AU39" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV39" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW39" s="14" t="inlineStr">
+      <c r="AV39" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW39" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX39" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY39" s="14" t="inlineStr">
         <is>
           <t>570 Introduction to Robotics, 580 Robotics Engineering, 585 Robotics Design, 590 Robotics Project, 591 Robotics Project II</t>
         </is>
@@ -7655,12 +8027,22 @@
       <c r="AU40" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV40" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW40" s="14" t="inlineStr">
+      <c r="AV40" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW40" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX40" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY40" s="14" t="inlineStr">
         <is>
           <t>521 Chemistry H</t>
         </is>
@@ -7834,12 +8216,22 @@
       <c r="AU41" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV41" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW41" s="14" t="inlineStr">
+      <c r="AV41" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW41" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX41" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY41" s="14" t="inlineStr">
         <is>
           <t>720 U.S. History I</t>
         </is>
@@ -8017,12 +8409,22 @@
       <c r="AU42" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV42" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW42" s="14" t="inlineStr">
+      <c r="AV42" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW42" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX42" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY42" s="14" t="inlineStr">
         <is>
           <t>322 Italian II, 323 Italian II H, 332 Italian III, 333 Italian III H, 352 AP Italian</t>
         </is>
@@ -8200,12 +8602,22 @@
       <c r="AU43" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV43" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW43" s="14" t="inlineStr">
+      <c r="AV43" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW43" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX43" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY43" s="14" t="inlineStr">
         <is>
           <t>722 Adv U.S. History I H, 731 U.S. History II H, 733 AP U.S. History</t>
         </is>
@@ -8369,10 +8781,24 @@
         <v>5</v>
       </c>
       <c r="AU44" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV44" s="40" t="inlineStr"/>
-      <c r="AW44" s="14" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="AV44" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW44" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX44" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY44" s="14" t="inlineStr">
         <is>
           <t>130 British Literature, 132 British Literature, 143 Creative Writing, 145 Journalism</t>
         </is>
@@ -8552,10 +8978,24 @@
         <v>4</v>
       </c>
       <c r="AU45" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV45" s="40" t="inlineStr"/>
-      <c r="AW45" s="14" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="AV45" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW45" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX45" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY45" s="14" t="inlineStr">
         <is>
           <t>144 Public Speaking</t>
         </is>
@@ -8719,12 +9159,22 @@
       <c r="AU46" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV46" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW46" s="14" t="inlineStr">
+      <c r="AV46" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW46" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX46" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY46" s="14" t="inlineStr">
         <is>
           <t>955 Academic Support</t>
         </is>
@@ -8884,10 +9334,24 @@
         <v>4</v>
       </c>
       <c r="AU47" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV47" s="40" t="inlineStr"/>
-      <c r="AW47" s="14" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="AV47" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW47" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX47" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY47" s="14" t="inlineStr">
         <is>
           <t>410 Algebra I, 422 Geometry</t>
         </is>
@@ -9051,10 +9515,24 @@
         <v>5</v>
       </c>
       <c r="AU48" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV48" s="40" t="inlineStr"/>
-      <c r="AW48" s="14" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="AV48" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW48" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX48" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY48" s="14" t="inlineStr">
         <is>
           <t>431 Algebra II/Trig H, 440 Precalculus, 450 Calculus H</t>
         </is>
@@ -9226,10 +9704,24 @@
         <v>4</v>
       </c>
       <c r="AU49" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV49" s="40" t="inlineStr"/>
-      <c r="AW49" s="14" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="AV49" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW49" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX49" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY49" s="14" t="inlineStr">
         <is>
           <t>225 Tech Theater Level 1, 228 Adv Theater Production</t>
         </is>
@@ -9385,10 +9877,24 @@
         <v>3</v>
       </c>
       <c r="AU50" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV50" s="40" t="inlineStr"/>
-      <c r="AW50" s="14" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="AV50" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW50" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX50" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY50" s="14" t="inlineStr">
         <is>
           <t>810 Theology 9, 820 Theology 10</t>
         </is>
@@ -9548,10 +10054,24 @@
         <v>5</v>
       </c>
       <c r="AU51" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV51" s="40" t="inlineStr"/>
-      <c r="AW51" s="14" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="AV51" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW51" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX51" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY51" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11, 849 Catholic Social Teaching</t>
         </is>
@@ -9729,12 +10249,22 @@
       <c r="AU52" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV52" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW52" s="14" t="inlineStr">
+      <c r="AV52" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW52" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX52" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY52" s="14" t="inlineStr">
         <is>
           <t>120 American Literature, 140 World Literature, 146 World Literature</t>
         </is>
@@ -9908,12 +10438,22 @@
       <c r="AU53" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV53" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW53" s="14" t="inlineStr">
+      <c r="AV53" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW53" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX53" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY53" s="14" t="inlineStr">
         <is>
           <t>110 Composition &amp; Literature, 121 American Literature H, 149 AP English Literature</t>
         </is>
@@ -10083,12 +10623,22 @@
       <c r="AU54" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV54" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW54" s="14" t="inlineStr">
+      <c r="AV54" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW54" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX54" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY54" s="14" t="inlineStr">
         <is>
           <t>830 Theology 11</t>
         </is>
@@ -10268,12 +10818,22 @@
       <c r="AU55" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV55" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW55" s="14" t="inlineStr">
+      <c r="AV55" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW55" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX55" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY55" s="14" t="inlineStr">
         <is>
           <t>2014 Multi-Media Production, 2024 TV/Film Process and Principles, 2034 TV/Film Production &amp; Editing I, 2044 TV/Film Production II, 2054 Digital Media</t>
         </is>
@@ -10451,12 +11011,22 @@
       <c r="AU56" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV56" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW56" s="14" t="inlineStr">
+      <c r="AV56" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW56" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX56" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY56" s="14" t="inlineStr">
         <is>
           <t>711 World History H, 713 AP World History, 743 AP European History, 744 Sociology, 751 American Government &amp; Politics</t>
         </is>
@@ -10630,12 +11200,22 @@
       <c r="AU57" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV57" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW57" s="14" t="inlineStr">
+      <c r="AV57" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW57" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX57" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY57" s="14" t="inlineStr">
         <is>
           <t>330 Spanish III, 331 Spanish III H</t>
         </is>
@@ -10797,8 +11377,22 @@
       <c r="AU58" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="AV58" s="40" t="inlineStr"/>
-      <c r="AW58" s="14" t="inlineStr">
+      <c r="AV58" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW58" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX58" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY58" s="14" t="inlineStr">
         <is>
           <t>708 Introduction to Business</t>
         </is>
@@ -10960,12 +11554,22 @@
       <c r="AU59" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV59" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW59" s="14" t="inlineStr">
+      <c r="AV59" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW59" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX59" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY59" s="14" t="inlineStr">
         <is>
           <t>710 World History, 741 Psychology, 751 American Government &amp; Politics</t>
         </is>
@@ -11135,12 +11739,22 @@
       <c r="AU60" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV60" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW60" s="14" t="inlineStr">
+      <c r="AV60" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW60" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX60" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY60" s="14" t="inlineStr">
         <is>
           <t>110 Composition &amp; Literature</t>
         </is>
@@ -11318,12 +11932,22 @@
       <c r="AU61" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV61" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW61" s="14" t="inlineStr">
+      <c r="AV61" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW61" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX61" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY61" s="14" t="inlineStr">
         <is>
           <t>551 AP Biology</t>
         </is>
@@ -11501,12 +12125,22 @@
       <c r="AU62" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV62" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW62" s="14" t="inlineStr">
+      <c r="AV62" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW62" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX62" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY62" s="14" t="inlineStr">
         <is>
           <t>531 Physics H, 557 AP Physics 1, 558 AP Physics C</t>
         </is>
@@ -11680,12 +12314,22 @@
       <c r="AU63" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV63" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW63" s="14" t="inlineStr">
+      <c r="AV63" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW63" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX63" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY63" s="14" t="inlineStr">
         <is>
           <t>310 Spanish I</t>
         </is>
@@ -11839,14 +12483,24 @@
         <v>3</v>
       </c>
       <c r="AU64" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV64" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW64" s="14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AV64" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW64" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX64" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY64" s="14" t="inlineStr"/>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="8" t="n">
@@ -12016,12 +12670,22 @@
       <c r="AU65" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="AV65" s="40" t="inlineStr">
-        <is>
-          <t>Pathway</t>
-        </is>
-      </c>
-      <c r="AW65" s="14" t="inlineStr">
+      <c r="AV65" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW65" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX65" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY65" s="14" t="inlineStr">
         <is>
           <t>410 Algebra I, 411 Algebra I H</t>
         </is>
@@ -12199,12 +12863,22 @@
       <c r="AU66" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV66" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW66" s="14" t="inlineStr">
+      <c r="AV66" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW66" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX66" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY66" s="14" t="inlineStr">
         <is>
           <t>710 World History, 756 Introduction to Law</t>
         </is>
@@ -12378,12 +13052,22 @@
       <c r="AU67" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV67" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW67" s="14" t="inlineStr">
+      <c r="AV67" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW67" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX67" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY67" s="14" t="inlineStr">
         <is>
           <t>732 Business Law, 742 Economics, 752 Economics H</t>
         </is>
@@ -12561,12 +13245,22 @@
       <c r="AU68" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="AV68" s="40" t="inlineStr">
-        <is>
-          <t>LEO, Pathway</t>
-        </is>
-      </c>
-      <c r="AW68" s="14" t="inlineStr">
+      <c r="AV68" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AW68" s="35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AX68" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY68" s="14" t="inlineStr">
         <is>
           <t>312 Italian I, 315 Latin I H, 327 Latin II H, 339 Latin III H, 359 AP Latin</t>
         </is>
@@ -12712,8 +13406,22 @@
       <c r="AU69" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="AV69" s="40" t="inlineStr"/>
-      <c r="AW69" s="36" t="n"/>
+      <c r="AV69" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW69" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX69" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY69" s="36" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="35" t="n">
@@ -12855,17 +13563,25 @@
       <c r="AU70" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="AV70" s="40" t="inlineStr"/>
-      <c r="AW70" s="36" t="n"/>
+      <c r="AV70" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW70" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX70" s="37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY70" s="36" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="21">
-    <dataValidation sqref="D5:D75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
-      <formula1>"Art,Business,Communication Arts,Computer Science,Engineering,English,Mathematics,Media Arts,Music,Physical Education,Science,Social Studies,Special Education,Student Services,Theater,Theology,World Language"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E5:E75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
-      <formula1>"Art,Business,Communication Arts,Computer Science,Engineering,English,Mathematics,Media Arts,Music,Physical Education,Science,Social Studies,Special Education,Student Services,Theater,Theology,World Language"</formula1>
-    </dataValidation>
+  <dataValidations count="24">
     <dataValidation sqref="F5:F75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
       <formula1>"Active,Leave,Retiring,New Hire"</formula1>
     </dataValidation>
@@ -12923,6 +13639,21 @@
     <dataValidation sqref="AF5:AF75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
+    <dataValidation sqref="AV5:AV75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AW5:AW75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AX5:AX75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D5:D75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
+      <formula1>"Art,Business,Communication Arts,Computer Science,Engineering,English,Mathematics,Media Arts,Music,Physical Education,Science,Social Studies,Special Education,Student Services,Theater,Theology,World Language"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5:E75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list." type="list">
+      <formula1>"Art,Business,Communication Arts,Computer Science,Engineering,English,Mathematics,Media Arts,Music,Physical Education,Science,Social Studies,Special Education,Student Services,Theater,Theology,World Language"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12934,7 +13665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14057,104 +14788,156 @@
       </c>
       <c r="B45" s="20" t="inlineStr">
         <is>
-          <t>Serving Populations</t>
+          <t>Teaches LEO</t>
         </is>
       </c>
       <c r="C45" s="20" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Dropdown</t>
         </is>
       </c>
       <c r="D45" s="20" t="inlineStr">
         <is>
-          <t>Which special populations this teacher serves based on their course assignments</t>
+          <t>Does this teacher teach courses serving LEO cohort students?</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>LEO, Pathway, AcademicSupport</t>
+          <t>Y, N</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="18" t="inlineStr">
+      <c r="A46" s="20" t="inlineStr">
         <is>
           <t>AW</t>
         </is>
       </c>
-      <c r="B46" s="19" t="inlineStr">
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>Teaches Pathway</t>
+        </is>
+      </c>
+      <c r="C46" s="20" t="inlineStr">
+        <is>
+          <t>Dropdown</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="inlineStr">
+        <is>
+          <t>Does this teacher teach courses serving Pathway program students?</t>
+        </is>
+      </c>
+      <c r="E46" s="20" t="inlineStr">
+        <is>
+          <t>Y, N</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="inlineStr">
+        <is>
+          <t>Teaches Acad Support</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="inlineStr">
+        <is>
+          <t>Dropdown</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="inlineStr">
+        <is>
+          <t>Does this teacher teach courses serving Academic Support students?</t>
+        </is>
+      </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Y, N</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="inlineStr">
         <is>
           <t>Courses Assigned</t>
         </is>
       </c>
-      <c r="C46" s="24" t="inlineStr">
+      <c r="C48" s="24" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="D46" s="20" t="inlineStr">
+      <c r="D48" s="20" t="inlineStr">
         <is>
           <t>Full course list from Template 1. Read-only.</t>
         </is>
       </c>
-      <c r="E46" s="21" t="inlineStr"/>
-    </row>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49">
-      <c r="A49" s="25" t="inlineStr">
-        <is>
-          <t>COLOR LEGEND</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="26" t="n"/>
-      <c r="B50" s="19" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
-      <c r="C50" s="20" t="inlineStr">
-        <is>
-          <t>Pre-populated from engine. Do not edit unless correcting an error.</t>
-        </is>
-      </c>
+      <c r="E48" s="21" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="27" t="n"/>
-      <c r="B51" s="19" t="inlineStr">
-        <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="C51" s="20" t="inlineStr">
-        <is>
-          <t>Needs your input — currently empty.</t>
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>COLOR LEGEND</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="28" t="n"/>
+      <c r="A52" s="26" t="n"/>
       <c r="B52" s="19" t="inlineStr">
         <is>
-          <t>Light Yellow</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="C52" s="20" t="inlineStr">
         <is>
-          <t>Optional — fill in if you have the information.</t>
+          <t>Pre-populated from engine. Do not edit unless correcting an error.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="29" t="n"/>
+      <c r="A53" s="27" t="n"/>
       <c r="B53" s="19" t="inlineStr">
         <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>Needs your input — currently empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="28" t="n"/>
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t>Light Yellow</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>Optional — fill in if you have the information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="29" t="n"/>
+      <c r="B55" s="19" t="inlineStr">
+        <is>
           <t>Gray</t>
         </is>
       </c>
-      <c r="C53" s="20" t="inlineStr">
+      <c r="C55" s="20" t="inlineStr">
         <is>
           <t>Read-only reference derived from Template 1. Do not edit.</t>
         </is>

</xml_diff>

<commit_message>
Fix room mismatches, skip teacher-less sections, add missing rooms
- Fix 24 'GYM' → 'Gym' room ID mismatches in Template_6 Sheet 2
- Add missing rooms I-111 and J-223 to Template_9 (48 rooms total)
- Remove duplicate J-322 row from Template_9
- Skip section generation for courses with no teacher assignment
  (85 sections across 62 courses), freeing room slots for real sections
- Result: 312/342 sections placed (91%), down from 47 to 30 clashes
- Remaining gap: 62 courses need teacher assignments in Template_6

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -6092,7 +6092,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr"/>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr"/>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
@@ -6140,7 +6140,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr"/>
@@ -6156,7 +6156,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
@@ -6172,7 +6172,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr"/>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
@@ -6204,7 +6204,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr"/>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr"/>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr"/>
@@ -6572,7 +6572,7 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr"/>
@@ -6604,7 +6604,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr"/>
@@ -6852,7 +6852,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr"/>
@@ -6868,7 +6868,7 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr"/>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr"/>
@@ -6900,7 +6900,7 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr"/>
@@ -6916,7 +6916,7 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr"/>
@@ -6932,7 +6932,7 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr"/>
@@ -6948,7 +6948,7 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr"/>
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr"/>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>GYM</t>
+          <t>Gym</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Add 3rd section of 131 British Literature H for Fisk (105819)
- Template 6 Sheet 2: Added 1 row for 131 (was 2, now 3 sections)
- Template 7: Sections Needed for 131: 2→3
- semester_designations.json: Added 131 entry (3 FY sections)
- CLAUDE.md: Documented Fisk section prescription

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5832,7 +5832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F347"/>
+  <dimension ref="A1:F348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7877,27 +7877,24 @@
       <c r="F124" s="4" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" s="4" t="n">
-        <v>107125</v>
-      </c>
-      <c r="B125" s="4" t="n">
-        <v>430</v>
-      </c>
-      <c r="C125" s="4" t="inlineStr">
-        <is>
-          <t>D-107</t>
-        </is>
-      </c>
-      <c r="D125" s="4" t="inlineStr"/>
-      <c r="E125" s="4" t="inlineStr"/>
-      <c r="F125" s="4" t="inlineStr"/>
+      <c r="A125" t="n">
+        <v>105819</v>
+      </c>
+      <c r="B125" t="n">
+        <v>131</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>I-116</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n">
         <v>107125</v>
       </c>
       <c r="B126" s="4" t="n">
-        <v>450</v>
+        <v>430</v>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
@@ -7929,7 +7926,7 @@
         <v>107125</v>
       </c>
       <c r="B128" s="4" t="n">
-        <v>422</v>
+        <v>450</v>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
@@ -7958,14 +7955,14 @@
     </row>
     <row r="130">
       <c r="A130" s="4" t="n">
-        <v>105788</v>
+        <v>107125</v>
       </c>
       <c r="B130" s="4" t="n">
-        <v>435</v>
+        <v>422</v>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>D-105</t>
+          <t>D-107</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr"/>
@@ -7977,7 +7974,7 @@
         <v>105788</v>
       </c>
       <c r="B131" s="4" t="n">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
@@ -8009,7 +8006,7 @@
         <v>105788</v>
       </c>
       <c r="B133" s="4" t="n">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
@@ -8038,12 +8035,16 @@
     </row>
     <row r="135">
       <c r="A135" s="4" t="n">
-        <v>122119</v>
+        <v>105788</v>
       </c>
       <c r="B135" s="4" t="n">
-        <v>120</v>
-      </c>
-      <c r="C135" s="4" t="inlineStr"/>
+        <v>448</v>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>D-105</t>
+        </is>
+      </c>
       <c r="D135" s="4" t="inlineStr"/>
       <c r="E135" s="4" t="inlineStr"/>
       <c r="F135" s="4" t="inlineStr"/>
@@ -8098,10 +8099,10 @@
     </row>
     <row r="140">
       <c r="A140" s="4" t="n">
-        <v>122120</v>
+        <v>122119</v>
       </c>
       <c r="B140" s="4" t="n">
-        <v>820</v>
+        <v>120</v>
       </c>
       <c r="C140" s="4" t="inlineStr"/>
       <c r="D140" s="4" t="inlineStr"/>
@@ -8125,7 +8126,7 @@
         <v>122120</v>
       </c>
       <c r="B142" s="4" t="n">
-        <v>830</v>
+        <v>820</v>
       </c>
       <c r="C142" s="4" t="inlineStr"/>
       <c r="D142" s="4" t="inlineStr"/>
@@ -8137,7 +8138,7 @@
         <v>122120</v>
       </c>
       <c r="B143" s="4" t="n">
-        <v>810</v>
+        <v>830</v>
       </c>
       <c r="C143" s="4" t="inlineStr"/>
       <c r="D143" s="4" t="inlineStr"/>
@@ -8170,10 +8171,10 @@
     </row>
     <row r="146">
       <c r="A146" s="4" t="n">
-        <v>107126</v>
+        <v>122120</v>
       </c>
       <c r="B146" s="4" t="n">
-        <v>542</v>
+        <v>810</v>
       </c>
       <c r="C146" s="4" t="inlineStr"/>
       <c r="D146" s="4" t="inlineStr"/>
@@ -8185,7 +8186,7 @@
         <v>107126</v>
       </c>
       <c r="B147" s="4" t="n">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C147" s="4" t="inlineStr"/>
       <c r="D147" s="4" t="inlineStr"/>
@@ -8206,16 +8207,12 @@
     </row>
     <row r="149">
       <c r="A149" s="4" t="n">
-        <v>105669</v>
+        <v>107126</v>
       </c>
       <c r="B149" s="4" t="n">
-        <v>430</v>
-      </c>
-      <c r="C149" s="4" t="inlineStr">
-        <is>
-          <t>D-108</t>
-        </is>
-      </c>
+        <v>543</v>
+      </c>
+      <c r="C149" s="4" t="inlineStr"/>
       <c r="D149" s="4" t="inlineStr"/>
       <c r="E149" s="4" t="inlineStr"/>
       <c r="F149" s="4" t="inlineStr"/>
@@ -8257,7 +8254,7 @@
         <v>105669</v>
       </c>
       <c r="B152" s="4" t="n">
-        <v>443</v>
+        <v>430</v>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
@@ -8286,14 +8283,14 @@
     </row>
     <row r="154">
       <c r="A154" s="4" t="n">
-        <v>105832</v>
+        <v>105669</v>
       </c>
       <c r="B154" s="4" t="n">
-        <v>761</v>
+        <v>443</v>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>I-113</t>
+          <t>D-108</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr"/>
@@ -8305,7 +8302,7 @@
         <v>105832</v>
       </c>
       <c r="B155" s="4" t="n">
-        <v>730</v>
+        <v>761</v>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
@@ -8337,7 +8334,7 @@
         <v>105832</v>
       </c>
       <c r="B157" s="4" t="n">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
@@ -8366,12 +8363,16 @@
     </row>
     <row r="159">
       <c r="A159" s="4" t="n">
-        <v>115019</v>
+        <v>105832</v>
       </c>
       <c r="B159" s="4" t="n">
-        <v>412</v>
-      </c>
-      <c r="C159" s="4" t="inlineStr"/>
+        <v>731</v>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>I-113</t>
+        </is>
+      </c>
       <c r="D159" s="4" t="inlineStr"/>
       <c r="E159" s="4" t="inlineStr"/>
       <c r="F159" s="4" t="inlineStr"/>
@@ -8405,7 +8406,7 @@
         <v>115019</v>
       </c>
       <c r="B162" s="4" t="n">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="C162" s="4" t="inlineStr"/>
       <c r="D162" s="4" t="inlineStr"/>
@@ -8426,16 +8427,12 @@
     </row>
     <row r="164">
       <c r="A164" s="4" t="n">
-        <v>105829</v>
+        <v>115019</v>
       </c>
       <c r="B164" s="4" t="n">
-        <v>510</v>
-      </c>
-      <c r="C164" s="4" t="inlineStr">
-        <is>
-          <t>D-202</t>
-        </is>
-      </c>
+        <v>420</v>
+      </c>
+      <c r="C164" s="4" t="inlineStr"/>
       <c r="D164" s="4" t="inlineStr"/>
       <c r="E164" s="4" t="inlineStr"/>
       <c r="F164" s="4" t="inlineStr"/>
@@ -8477,7 +8474,7 @@
         <v>105829</v>
       </c>
       <c r="B167" s="4" t="n">
-        <v>500</v>
+        <v>510</v>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
@@ -8506,14 +8503,14 @@
     </row>
     <row r="169">
       <c r="A169" s="4" t="n">
-        <v>105767</v>
+        <v>105829</v>
       </c>
       <c r="B169" s="4" t="n">
-        <v>955</v>
+        <v>500</v>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Success Center</t>
+          <t>D-202</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr"/>
@@ -8573,19 +8570,23 @@
         <v>105767</v>
       </c>
       <c r="B173" s="4" t="n">
-        <v>112</v>
-      </c>
-      <c r="C173" s="4" t="inlineStr"/>
+        <v>955</v>
+      </c>
+      <c r="C173" s="4" t="inlineStr">
+        <is>
+          <t>Success Center</t>
+        </is>
+      </c>
       <c r="D173" s="4" t="inlineStr"/>
       <c r="E173" s="4" t="inlineStr"/>
       <c r="F173" s="4" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n">
-        <v>122084</v>
+        <v>105767</v>
       </c>
       <c r="B174" s="4" t="n">
-        <v>810</v>
+        <v>112</v>
       </c>
       <c r="C174" s="4" t="inlineStr"/>
       <c r="D174" s="4" t="inlineStr"/>
@@ -8642,16 +8643,12 @@
     </row>
     <row r="179">
       <c r="A179" s="4" t="n">
-        <v>105615</v>
+        <v>122084</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>553</v>
-      </c>
-      <c r="C179" s="4" t="inlineStr">
-        <is>
-          <t>D-201</t>
-        </is>
-      </c>
+        <v>810</v>
+      </c>
+      <c r="C179" s="4" t="inlineStr"/>
       <c r="D179" s="4" t="inlineStr"/>
       <c r="E179" s="4" t="inlineStr"/>
       <c r="F179" s="4" t="inlineStr"/>
@@ -8661,7 +8658,7 @@
         <v>105615</v>
       </c>
       <c r="B180" s="4" t="n">
-        <v>511</v>
+        <v>553</v>
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
@@ -8722,12 +8719,16 @@
     </row>
     <row r="184">
       <c r="A184" s="4" t="n">
-        <v>105625</v>
+        <v>105615</v>
       </c>
       <c r="B184" s="4" t="n">
-        <v>765</v>
-      </c>
-      <c r="C184" s="4" t="inlineStr"/>
+        <v>511</v>
+      </c>
+      <c r="C184" s="4" t="inlineStr">
+        <is>
+          <t>D-201</t>
+        </is>
+      </c>
       <c r="D184" s="4" t="inlineStr"/>
       <c r="E184" s="4" t="inlineStr"/>
       <c r="F184" s="4" t="inlineStr"/>
@@ -8749,7 +8750,7 @@
         <v>105625</v>
       </c>
       <c r="B186" s="4" t="n">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="C186" s="4" t="inlineStr"/>
       <c r="D186" s="4" t="inlineStr"/>
@@ -8773,7 +8774,7 @@
         <v>105625</v>
       </c>
       <c r="B188" s="4" t="n">
-        <v>456</v>
+        <v>766</v>
       </c>
       <c r="C188" s="4" t="inlineStr"/>
       <c r="D188" s="4" t="inlineStr"/>
@@ -8782,16 +8783,12 @@
     </row>
     <row r="189">
       <c r="A189" s="4" t="n">
-        <v>105628</v>
+        <v>105625</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>530</v>
-      </c>
-      <c r="C189" s="4" t="inlineStr">
-        <is>
-          <t>D-205</t>
-        </is>
-      </c>
+        <v>456</v>
+      </c>
+      <c r="C189" s="4" t="inlineStr"/>
       <c r="D189" s="4" t="inlineStr"/>
       <c r="E189" s="4" t="inlineStr"/>
       <c r="F189" s="4" t="inlineStr"/>
@@ -8846,14 +8843,14 @@
     </row>
     <row r="193">
       <c r="A193" s="4" t="n">
-        <v>111895</v>
+        <v>105628</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>820</v>
+        <v>530</v>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>J-323</t>
+          <t>D-205</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr"/>
@@ -8897,7 +8894,7 @@
         <v>111895</v>
       </c>
       <c r="B196" s="4" t="n">
-        <v>830</v>
+        <v>820</v>
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
@@ -8926,14 +8923,14 @@
     </row>
     <row r="198">
       <c r="A198" s="4" t="n">
-        <v>106760</v>
+        <v>111895</v>
       </c>
       <c r="B198" s="4" t="n">
         <v>830</v>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>J-020</t>
+          <t>J-323</t>
         </is>
       </c>
       <c r="D198" s="4" t="inlineStr"/>
@@ -8942,14 +8939,14 @@
     </row>
     <row r="199">
       <c r="A199" s="4" t="n">
-        <v>105666</v>
+        <v>106760</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>820</v>
+        <v>830</v>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>J-320</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr"/>
@@ -9009,7 +9006,7 @@
         <v>105666</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>810</v>
+        <v>820</v>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
@@ -9022,14 +9019,14 @@
     </row>
     <row r="204">
       <c r="A204" s="4" t="n">
-        <v>102255</v>
+        <v>105666</v>
       </c>
       <c r="B204" s="4" t="n">
-        <v>206</v>
+        <v>810</v>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>J-120</t>
+          <t>J-320</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr"/>
@@ -9041,7 +9038,7 @@
         <v>102255</v>
       </c>
       <c r="B205" s="4" t="n">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
@@ -9073,7 +9070,7 @@
         <v>102255</v>
       </c>
       <c r="B207" s="4" t="n">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
@@ -9089,7 +9086,7 @@
         <v>102255</v>
       </c>
       <c r="B208" s="4" t="n">
-        <v>220</v>
+        <v>201</v>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
@@ -9105,7 +9102,7 @@
         <v>102255</v>
       </c>
       <c r="B209" s="4" t="n">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
@@ -9118,14 +9115,14 @@
     </row>
     <row r="210">
       <c r="A210" s="4" t="n">
-        <v>117302</v>
+        <v>102255</v>
       </c>
       <c r="B210" s="4" t="n">
-        <v>763</v>
+        <v>209</v>
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>J-120</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr"/>
@@ -9153,7 +9150,7 @@
         <v>117302</v>
       </c>
       <c r="B212" s="4" t="n">
-        <v>721</v>
+        <v>763</v>
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
@@ -9198,14 +9195,14 @@
     </row>
     <row r="215">
       <c r="A215" s="4" t="n">
-        <v>105642</v>
+        <v>117302</v>
       </c>
       <c r="B215" s="4" t="n">
-        <v>955</v>
+        <v>721</v>
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>Success Center</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr"/>
@@ -9249,11 +9246,11 @@
         <v>105642</v>
       </c>
       <c r="B218" s="4" t="n">
-        <v>122</v>
+        <v>955</v>
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>Success Center</t>
         </is>
       </c>
       <c r="D218" s="4" t="inlineStr"/>
@@ -9262,14 +9259,14 @@
     </row>
     <row r="219">
       <c r="A219" s="4" t="n">
-        <v>117304</v>
+        <v>105642</v>
       </c>
       <c r="B219" s="4" t="n">
-        <v>570</v>
+        <v>122</v>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr"/>
@@ -9297,7 +9294,7 @@
         <v>117304</v>
       </c>
       <c r="B221" s="4" t="n">
-        <v>585</v>
+        <v>570</v>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
@@ -9329,7 +9326,7 @@
         <v>117304</v>
       </c>
       <c r="B223" s="4" t="n">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
@@ -9393,7 +9390,7 @@
         <v>117304</v>
       </c>
       <c r="B227" s="4" t="n">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
@@ -9401,11 +9398,7 @@
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr"/>
-      <c r="E227" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E227" s="4" t="inlineStr"/>
       <c r="F227" s="4" t="inlineStr"/>
     </row>
     <row r="228">
@@ -9433,7 +9426,7 @@
         <v>117304</v>
       </c>
       <c r="B229" s="4" t="n">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
@@ -9470,18 +9463,22 @@
     </row>
     <row r="231">
       <c r="A231" s="4" t="n">
-        <v>112092</v>
+        <v>117304</v>
       </c>
       <c r="B231" s="4" t="n">
-        <v>521</v>
+        <v>591</v>
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>D-204</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr"/>
-      <c r="E231" s="4" t="inlineStr"/>
+      <c r="E231" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F231" s="4" t="inlineStr"/>
     </row>
     <row r="232">
@@ -9537,7 +9534,7 @@
         <v>112092</v>
       </c>
       <c r="B235" s="4" t="n">
-        <v>531</v>
+        <v>521</v>
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
@@ -9550,14 +9547,14 @@
     </row>
     <row r="236">
       <c r="A236" s="4" t="n">
-        <v>105671</v>
+        <v>112092</v>
       </c>
       <c r="B236" s="4" t="n">
-        <v>720</v>
+        <v>531</v>
       </c>
       <c r="C236" s="4" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>D-204</t>
         </is>
       </c>
       <c r="D236" s="4" t="inlineStr"/>
@@ -9630,14 +9627,14 @@
     </row>
     <row r="241">
       <c r="A241" s="4" t="n">
-        <v>106762</v>
+        <v>105671</v>
       </c>
       <c r="B241" s="4" t="n">
-        <v>352</v>
+        <v>720</v>
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="D241" s="4" t="inlineStr"/>
@@ -9649,7 +9646,7 @@
         <v>106762</v>
       </c>
       <c r="B242" s="4" t="n">
-        <v>322</v>
+        <v>352</v>
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
@@ -9681,7 +9678,7 @@
         <v>106762</v>
       </c>
       <c r="B244" s="4" t="n">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
@@ -9697,7 +9694,7 @@
         <v>106762</v>
       </c>
       <c r="B245" s="4" t="n">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
@@ -9713,7 +9710,7 @@
         <v>106762</v>
       </c>
       <c r="B246" s="4" t="n">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
@@ -9726,14 +9723,14 @@
     </row>
     <row r="247">
       <c r="A247" s="4" t="n">
-        <v>105616</v>
+        <v>106762</v>
       </c>
       <c r="B247" s="4" t="n">
-        <v>722</v>
+        <v>333</v>
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>I-119</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr"/>
@@ -9761,7 +9758,7 @@
         <v>105616</v>
       </c>
       <c r="B249" s="4" t="n">
-        <v>733</v>
+        <v>722</v>
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
@@ -9806,14 +9803,14 @@
     </row>
     <row r="252">
       <c r="A252" s="4" t="n">
-        <v>108420</v>
+        <v>105616</v>
       </c>
       <c r="B252" s="4" t="n">
-        <v>120</v>
+        <v>733</v>
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>I-119</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr"/>
@@ -9825,7 +9822,7 @@
         <v>108420</v>
       </c>
       <c r="B253" s="4" t="n">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="C253" s="4" t="inlineStr">
         <is>
@@ -9873,7 +9870,7 @@
         <v>108420</v>
       </c>
       <c r="B256" s="4" t="n">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
@@ -9886,14 +9883,14 @@
     </row>
     <row r="257">
       <c r="A257" s="4" t="n">
-        <v>105617</v>
+        <v>108420</v>
       </c>
       <c r="B257" s="4" t="n">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
-          <t>D-101</t>
+          <t>D-104</t>
         </is>
       </c>
       <c r="D257" s="4" t="inlineStr"/>
@@ -9921,7 +9918,7 @@
         <v>105617</v>
       </c>
       <c r="B259" s="4" t="n">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
@@ -9953,7 +9950,7 @@
         <v>105617</v>
       </c>
       <c r="B261" s="4" t="n">
-        <v>110</v>
+        <v>149</v>
       </c>
       <c r="C261" s="4" t="inlineStr">
         <is>
@@ -9966,12 +9963,16 @@
     </row>
     <row r="262">
       <c r="A262" s="4" t="n">
-        <v>122121</v>
+        <v>105617</v>
       </c>
       <c r="B262" s="4" t="n">
-        <v>410</v>
-      </c>
-      <c r="C262" s="4" t="inlineStr"/>
+        <v>110</v>
+      </c>
+      <c r="C262" s="4" t="inlineStr">
+        <is>
+          <t>D-101</t>
+        </is>
+      </c>
       <c r="D262" s="4" t="inlineStr"/>
       <c r="E262" s="4" t="inlineStr"/>
       <c r="F262" s="4" t="inlineStr"/>
@@ -10005,7 +10006,7 @@
         <v>122121</v>
       </c>
       <c r="B265" s="4" t="n">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C265" s="4" t="inlineStr"/>
       <c r="D265" s="4" t="inlineStr"/>
@@ -10026,16 +10027,12 @@
     </row>
     <row r="267">
       <c r="A267" s="4" t="n">
-        <v>105624</v>
+        <v>122121</v>
       </c>
       <c r="B267" s="4" t="n">
-        <v>830</v>
-      </c>
-      <c r="C267" s="4" t="inlineStr">
-        <is>
-          <t>J-221</t>
-        </is>
-      </c>
+        <v>420</v>
+      </c>
+      <c r="C267" s="4" t="inlineStr"/>
       <c r="D267" s="4" t="inlineStr"/>
       <c r="E267" s="4" t="inlineStr"/>
       <c r="F267" s="4" t="inlineStr"/>
@@ -10106,14 +10103,14 @@
     </row>
     <row r="272">
       <c r="A272" s="4" t="n">
-        <v>122122</v>
+        <v>105624</v>
       </c>
       <c r="B272" s="4" t="n">
-        <v>2054</v>
+        <v>830</v>
       </c>
       <c r="C272" s="4" t="inlineStr">
         <is>
-          <t>I-111</t>
+          <t>J-221</t>
         </is>
       </c>
       <c r="D272" s="4" t="inlineStr"/>
@@ -10141,7 +10138,7 @@
         <v>122122</v>
       </c>
       <c r="B274" s="4" t="n">
-        <v>2014</v>
+        <v>2054</v>
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
@@ -10173,7 +10170,7 @@
         <v>122122</v>
       </c>
       <c r="B276" s="4" t="n">
-        <v>2024</v>
+        <v>2014</v>
       </c>
       <c r="C276" s="4" t="inlineStr">
         <is>
@@ -10205,7 +10202,7 @@
         <v>122122</v>
       </c>
       <c r="B278" s="4" t="n">
-        <v>2034</v>
+        <v>2024</v>
       </c>
       <c r="C278" s="4" t="inlineStr">
         <is>
@@ -10221,7 +10218,7 @@
         <v>122122</v>
       </c>
       <c r="B279" s="4" t="n">
-        <v>2044</v>
+        <v>2034</v>
       </c>
       <c r="C279" s="4" t="inlineStr">
         <is>
@@ -10250,14 +10247,14 @@
     </row>
     <row r="281">
       <c r="A281" s="4" t="n">
-        <v>105651</v>
+        <v>122122</v>
       </c>
       <c r="B281" s="4" t="n">
-        <v>743</v>
+        <v>2044</v>
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr"/>
@@ -10269,7 +10266,7 @@
         <v>105651</v>
       </c>
       <c r="B282" s="4" t="n">
-        <v>713</v>
+        <v>743</v>
       </c>
       <c r="C282" s="4" t="inlineStr">
         <is>
@@ -10301,7 +10298,7 @@
         <v>105651</v>
       </c>
       <c r="B284" s="4" t="n">
-        <v>744</v>
+        <v>713</v>
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
@@ -10333,7 +10330,7 @@
         <v>105651</v>
       </c>
       <c r="B286" s="4" t="n">
-        <v>711</v>
+        <v>744</v>
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
@@ -10362,14 +10359,14 @@
     </row>
     <row r="288">
       <c r="A288" s="4" t="n">
-        <v>105618</v>
+        <v>105651</v>
       </c>
       <c r="B288" s="4" t="n">
-        <v>330</v>
+        <v>711</v>
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>S-232</t>
+          <t>I-117</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr"/>
@@ -10397,7 +10394,7 @@
         <v>105618</v>
       </c>
       <c r="B290" s="4" t="n">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
@@ -10442,18 +10439,18 @@
     </row>
     <row r="293">
       <c r="A293" s="4" t="n">
-        <v>105808</v>
+        <v>105618</v>
       </c>
       <c r="B293" s="4" t="n">
-        <v>708</v>
-      </c>
-      <c r="C293" s="4" t="inlineStr"/>
+        <v>331</v>
+      </c>
+      <c r="C293" s="4" t="inlineStr">
+        <is>
+          <t>S-232</t>
+        </is>
+      </c>
       <c r="D293" s="4" t="inlineStr"/>
-      <c r="E293" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E293" s="4" t="inlineStr"/>
       <c r="F293" s="4" t="inlineStr"/>
     </row>
     <row r="294">
@@ -10483,7 +10480,7 @@
       <c r="D295" s="4" t="inlineStr"/>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F295" s="4" t="inlineStr"/>
@@ -10522,14 +10519,18 @@
     </row>
     <row r="298">
       <c r="A298" s="4" t="n">
-        <v>117711</v>
+        <v>105808</v>
       </c>
       <c r="B298" s="4" t="n">
-        <v>751</v>
+        <v>708</v>
       </c>
       <c r="C298" s="4" t="inlineStr"/>
       <c r="D298" s="4" t="inlineStr"/>
-      <c r="E298" s="4" t="inlineStr"/>
+      <c r="E298" s="4" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
       <c r="F298" s="4" t="inlineStr"/>
     </row>
     <row r="299">
@@ -10537,7 +10538,7 @@
         <v>117711</v>
       </c>
       <c r="B299" s="4" t="n">
-        <v>741</v>
+        <v>751</v>
       </c>
       <c r="C299" s="4" t="inlineStr"/>
       <c r="D299" s="4" t="inlineStr"/>
@@ -10573,7 +10574,7 @@
         <v>117711</v>
       </c>
       <c r="B302" s="4" t="n">
-        <v>710</v>
+        <v>741</v>
       </c>
       <c r="C302" s="4" t="inlineStr"/>
       <c r="D302" s="4" t="inlineStr"/>
@@ -10606,16 +10607,12 @@
     </row>
     <row r="305">
       <c r="A305" s="4" t="n">
-        <v>105803</v>
+        <v>117711</v>
       </c>
       <c r="B305" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C305" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
+        <v>710</v>
+      </c>
+      <c r="C305" s="4" t="inlineStr"/>
       <c r="D305" s="4" t="inlineStr"/>
       <c r="E305" s="4" t="inlineStr"/>
       <c r="F305" s="4" t="inlineStr"/>
@@ -10686,28 +10683,28 @@
     </row>
     <row r="310">
       <c r="A310" s="4" t="n">
-        <v>105623</v>
+        <v>105803</v>
       </c>
       <c r="B310" s="4" t="n">
-        <v>551</v>
-      </c>
-      <c r="C310" s="4" t="inlineStr"/>
+        <v>110</v>
+      </c>
+      <c r="C310" s="4" t="inlineStr">
+        <is>
+          <t>D-102</t>
+        </is>
+      </c>
       <c r="D310" s="4" t="inlineStr"/>
       <c r="E310" s="4" t="inlineStr"/>
       <c r="F310" s="4" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" s="4" t="n">
-        <v>105746</v>
+        <v>105623</v>
       </c>
       <c r="B311" s="4" t="n">
-        <v>556</v>
-      </c>
-      <c r="C311" s="4" t="inlineStr">
-        <is>
-          <t>D-210</t>
-        </is>
-      </c>
+        <v>551</v>
+      </c>
+      <c r="C311" s="4" t="inlineStr"/>
       <c r="D311" s="4" t="inlineStr"/>
       <c r="E311" s="4" t="inlineStr"/>
       <c r="F311" s="4" t="inlineStr"/>
@@ -10733,7 +10730,7 @@
         <v>105746</v>
       </c>
       <c r="B313" s="4" t="n">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
@@ -10749,7 +10746,7 @@
         <v>105746</v>
       </c>
       <c r="B314" s="4" t="n">
-        <v>531</v>
+        <v>558</v>
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
@@ -10778,14 +10775,14 @@
     </row>
     <row r="316">
       <c r="A316" s="4" t="n">
-        <v>106765</v>
+        <v>105746</v>
       </c>
       <c r="B316" s="4" t="n">
-        <v>310</v>
+        <v>531</v>
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>S-235</t>
+          <t>D-210</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr"/>
@@ -10858,12 +10855,16 @@
     </row>
     <row r="321">
       <c r="A321" s="4" t="n">
-        <v>105768</v>
+        <v>106765</v>
       </c>
       <c r="B321" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="C321" s="4" t="inlineStr"/>
+        <v>310</v>
+      </c>
+      <c r="C321" s="4" t="inlineStr">
+        <is>
+          <t>S-235</t>
+        </is>
+      </c>
       <c r="D321" s="4" t="inlineStr"/>
       <c r="E321" s="4" t="inlineStr"/>
       <c r="F321" s="4" t="inlineStr"/>
@@ -10873,7 +10874,7 @@
         <v>105768</v>
       </c>
       <c r="B322" s="4" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C322" s="4" t="inlineStr"/>
       <c r="D322" s="4" t="inlineStr"/>
@@ -10885,7 +10886,7 @@
         <v>105768</v>
       </c>
       <c r="B323" s="4" t="n">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="C323" s="4" t="inlineStr"/>
       <c r="D323" s="4" t="inlineStr"/>
@@ -10897,7 +10898,7 @@
         <v>105768</v>
       </c>
       <c r="B324" s="4" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C324" s="4" t="inlineStr"/>
       <c r="D324" s="4" t="inlineStr"/>
@@ -10906,16 +10907,12 @@
     </row>
     <row r="325">
       <c r="A325" s="4" t="n">
-        <v>106623</v>
+        <v>105768</v>
       </c>
       <c r="B325" s="4" t="n">
-        <v>410</v>
-      </c>
-      <c r="C325" s="4" t="inlineStr">
-        <is>
-          <t>D-110</t>
-        </is>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="C325" s="4" t="inlineStr"/>
       <c r="D325" s="4" t="inlineStr"/>
       <c r="E325" s="4" t="inlineStr"/>
       <c r="F325" s="4" t="inlineStr"/>
@@ -10957,7 +10954,7 @@
         <v>106623</v>
       </c>
       <c r="B328" s="4" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
@@ -10973,7 +10970,7 @@
         <v>106623</v>
       </c>
       <c r="B329" s="4" t="n">
-        <v>420</v>
+        <v>411</v>
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
@@ -10986,14 +10983,14 @@
     </row>
     <row r="330">
       <c r="A330" s="4" t="n">
-        <v>105883</v>
+        <v>106623</v>
       </c>
       <c r="B330" s="4" t="n">
-        <v>756</v>
+        <v>420</v>
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>I-012</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr"/>
@@ -11005,7 +11002,7 @@
         <v>105883</v>
       </c>
       <c r="B331" s="4" t="n">
-        <v>730</v>
+        <v>756</v>
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
@@ -11021,7 +11018,7 @@
         <v>105883</v>
       </c>
       <c r="B332" s="4" t="n">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
@@ -11037,7 +11034,7 @@
         <v>105883</v>
       </c>
       <c r="B333" s="4" t="n">
-        <v>710</v>
+        <v>731</v>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
@@ -11082,14 +11079,14 @@
     </row>
     <row r="336">
       <c r="A336" s="4" t="n">
-        <v>105620</v>
+        <v>105883</v>
       </c>
       <c r="B336" s="4" t="n">
-        <v>732</v>
+        <v>710</v>
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>S-233</t>
+          <t>I-012</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr"/>
@@ -11117,7 +11114,7 @@
         <v>105620</v>
       </c>
       <c r="B338" s="4" t="n">
-        <v>742</v>
+        <v>732</v>
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
@@ -11149,7 +11146,7 @@
         <v>105620</v>
       </c>
       <c r="B340" s="4" t="n">
-        <v>752</v>
+        <v>742</v>
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
@@ -11178,14 +11175,14 @@
     </row>
     <row r="342">
       <c r="A342" s="4" t="n">
-        <v>105729</v>
+        <v>105620</v>
       </c>
       <c r="B342" s="4" t="n">
-        <v>359</v>
+        <v>752</v>
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
-          <t>S-236</t>
+          <t>S-233</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr"/>
@@ -11197,7 +11194,7 @@
         <v>105729</v>
       </c>
       <c r="B343" s="4" t="n">
-        <v>312</v>
+        <v>359</v>
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
@@ -11229,7 +11226,7 @@
         <v>105729</v>
       </c>
       <c r="B345" s="4" t="n">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
@@ -11245,7 +11242,7 @@
         <v>105729</v>
       </c>
       <c r="B346" s="4" t="n">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="C346" s="4" t="inlineStr">
         <is>
@@ -11261,7 +11258,7 @@
         <v>105729</v>
       </c>
       <c r="B347" s="4" t="n">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="C347" s="4" t="inlineStr">
         <is>
@@ -11271,6 +11268,22 @@
       <c r="D347" s="4" t="inlineStr"/>
       <c r="E347" s="4" t="inlineStr"/>
       <c r="F347" s="4" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="4" t="n">
+        <v>105729</v>
+      </c>
+      <c r="B348" s="4" t="n">
+        <v>339</v>
+      </c>
+      <c r="C348" s="4" t="inlineStr">
+        <is>
+          <t>S-236</t>
+        </is>
+      </c>
+      <c r="D348" s="4" t="inlineStr"/>
+      <c r="E348" s="4" t="inlineStr"/>
+      <c r="F348" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add sections for Kozak/Laracy/Umbrino/Lopez, re-run engine v2.4
Template 6 Sheet 2 additions:
- Kozak (105628): +2 sections 595 Engineering Design (S1+S2)
- Laracy (106760): +8 sections 851 Spirituality of Vocation
- Umbrino (105768): +2 sections 130 British Literature (FY)
- Lopez (102255): +2 sections 201 Intro Guitar (S1+S2, co-sched w/ 203)

Template 7: Updated Sections Needed (130→5, 201→3)
Engine v2.4: 69 clashes, 98.9% placement, 360 sections, 0 grad req clashes

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5832,7 +5832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F348"/>
+  <dimension ref="A1:F362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8858,36 +8858,40 @@
       <c r="F193" s="4" t="inlineStr"/>
     </row>
     <row r="194">
-      <c r="A194" s="4" t="n">
-        <v>111895</v>
-      </c>
-      <c r="B194" s="4" t="n">
-        <v>820</v>
-      </c>
-      <c r="C194" s="4" t="inlineStr">
-        <is>
-          <t>J-323</t>
-        </is>
-      </c>
-      <c r="D194" s="4" t="inlineStr"/>
-      <c r="E194" s="4" t="inlineStr"/>
-      <c r="F194" s="4" t="inlineStr"/>
+      <c r="A194" t="n">
+        <v>105628</v>
+      </c>
+      <c r="B194" t="n">
+        <v>595</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>D-205</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
     </row>
     <row r="195">
-      <c r="A195" s="4" t="n">
-        <v>111895</v>
-      </c>
-      <c r="B195" s="4" t="n">
-        <v>820</v>
-      </c>
-      <c r="C195" s="4" t="inlineStr">
-        <is>
-          <t>J-323</t>
-        </is>
-      </c>
-      <c r="D195" s="4" t="inlineStr"/>
-      <c r="E195" s="4" t="inlineStr"/>
-      <c r="F195" s="4" t="inlineStr"/>
+      <c r="A195" t="n">
+        <v>105628</v>
+      </c>
+      <c r="B195" t="n">
+        <v>595</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>D-205</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n">
@@ -8910,7 +8914,7 @@
         <v>111895</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>830</v>
+        <v>820</v>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
@@ -8926,7 +8930,7 @@
         <v>111895</v>
       </c>
       <c r="B198" s="4" t="n">
-        <v>830</v>
+        <v>820</v>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
@@ -8939,14 +8943,14 @@
     </row>
     <row r="199">
       <c r="A199" s="4" t="n">
-        <v>106760</v>
+        <v>111895</v>
       </c>
       <c r="B199" s="4" t="n">
         <v>830</v>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>J-020</t>
+          <t>J-323</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr"/>
@@ -8955,14 +8959,14 @@
     </row>
     <row r="200">
       <c r="A200" s="4" t="n">
-        <v>105666</v>
+        <v>111895</v>
       </c>
       <c r="B200" s="4" t="n">
-        <v>820</v>
+        <v>830</v>
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t>J-320</t>
+          <t>J-323</t>
         </is>
       </c>
       <c r="D200" s="4" t="inlineStr"/>
@@ -8971,14 +8975,14 @@
     </row>
     <row r="201">
       <c r="A201" s="4" t="n">
-        <v>105666</v>
+        <v>106760</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>820</v>
+        <v>830</v>
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t>J-320</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="D201" s="4" t="inlineStr"/>
@@ -8986,143 +8990,119 @@
       <c r="F201" s="4" t="inlineStr"/>
     </row>
     <row r="202">
-      <c r="A202" s="4" t="n">
-        <v>105666</v>
-      </c>
-      <c r="B202" s="4" t="n">
-        <v>820</v>
-      </c>
-      <c r="C202" s="4" t="inlineStr">
-        <is>
-          <t>J-320</t>
-        </is>
-      </c>
-      <c r="D202" s="4" t="inlineStr"/>
-      <c r="E202" s="4" t="inlineStr"/>
-      <c r="F202" s="4" t="inlineStr"/>
+      <c r="A202" t="n">
+        <v>106760</v>
+      </c>
+      <c r="B202" t="n">
+        <v>851</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
     </row>
     <row r="203">
-      <c r="A203" s="4" t="n">
-        <v>105666</v>
-      </c>
-      <c r="B203" s="4" t="n">
-        <v>820</v>
-      </c>
-      <c r="C203" s="4" t="inlineStr">
-        <is>
-          <t>J-320</t>
-        </is>
-      </c>
-      <c r="D203" s="4" t="inlineStr"/>
-      <c r="E203" s="4" t="inlineStr"/>
-      <c r="F203" s="4" t="inlineStr"/>
+      <c r="A203" t="n">
+        <v>106760</v>
+      </c>
+      <c r="B203" t="n">
+        <v>851</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
     </row>
     <row r="204">
-      <c r="A204" s="4" t="n">
-        <v>105666</v>
-      </c>
-      <c r="B204" s="4" t="n">
-        <v>810</v>
-      </c>
-      <c r="C204" s="4" t="inlineStr">
-        <is>
-          <t>J-320</t>
-        </is>
-      </c>
-      <c r="D204" s="4" t="inlineStr"/>
-      <c r="E204" s="4" t="inlineStr"/>
-      <c r="F204" s="4" t="inlineStr"/>
+      <c r="A204" t="n">
+        <v>106760</v>
+      </c>
+      <c r="B204" t="n">
+        <v>851</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
     </row>
     <row r="205">
-      <c r="A205" s="4" t="n">
-        <v>102255</v>
-      </c>
-      <c r="B205" s="4" t="n">
-        <v>206</v>
-      </c>
-      <c r="C205" s="4" t="inlineStr">
-        <is>
-          <t>J-120</t>
-        </is>
-      </c>
-      <c r="D205" s="4" t="inlineStr"/>
-      <c r="E205" s="4" t="inlineStr"/>
-      <c r="F205" s="4" t="inlineStr"/>
+      <c r="A205" t="n">
+        <v>106760</v>
+      </c>
+      <c r="B205" t="n">
+        <v>851</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
     </row>
     <row r="206">
-      <c r="A206" s="4" t="n">
-        <v>102255</v>
-      </c>
-      <c r="B206" s="4" t="n">
-        <v>203</v>
-      </c>
-      <c r="C206" s="4" t="inlineStr">
-        <is>
-          <t>J-120</t>
-        </is>
-      </c>
-      <c r="D206" s="4" t="inlineStr"/>
-      <c r="E206" s="4" t="inlineStr"/>
-      <c r="F206" s="4" t="inlineStr"/>
+      <c r="A206" t="n">
+        <v>106760</v>
+      </c>
+      <c r="B206" t="n">
+        <v>851</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
     </row>
     <row r="207">
-      <c r="A207" s="4" t="n">
-        <v>102255</v>
-      </c>
-      <c r="B207" s="4" t="n">
-        <v>203</v>
-      </c>
-      <c r="C207" s="4" t="inlineStr">
-        <is>
-          <t>J-120</t>
-        </is>
-      </c>
-      <c r="D207" s="4" t="inlineStr"/>
-      <c r="E207" s="4" t="inlineStr"/>
-      <c r="F207" s="4" t="inlineStr"/>
+      <c r="A207" t="n">
+        <v>106760</v>
+      </c>
+      <c r="B207" t="n">
+        <v>851</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
     </row>
     <row r="208">
-      <c r="A208" s="4" t="n">
-        <v>102255</v>
-      </c>
-      <c r="B208" s="4" t="n">
-        <v>201</v>
-      </c>
-      <c r="C208" s="4" t="inlineStr">
-        <is>
-          <t>J-120</t>
-        </is>
-      </c>
-      <c r="D208" s="4" t="inlineStr"/>
-      <c r="E208" s="4" t="inlineStr"/>
-      <c r="F208" s="4" t="inlineStr"/>
+      <c r="A208" t="n">
+        <v>106760</v>
+      </c>
+      <c r="B208" t="n">
+        <v>851</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
     </row>
     <row r="209">
-      <c r="A209" s="4" t="n">
-        <v>102255</v>
-      </c>
-      <c r="B209" s="4" t="n">
-        <v>220</v>
-      </c>
-      <c r="C209" s="4" t="inlineStr">
-        <is>
-          <t>J-120</t>
-        </is>
-      </c>
-      <c r="D209" s="4" t="inlineStr"/>
-      <c r="E209" s="4" t="inlineStr"/>
-      <c r="F209" s="4" t="inlineStr"/>
+      <c r="A209" t="n">
+        <v>106760</v>
+      </c>
+      <c r="B209" t="n">
+        <v>851</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n">
-        <v>102255</v>
+        <v>105666</v>
       </c>
       <c r="B210" s="4" t="n">
-        <v>209</v>
+        <v>820</v>
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>J-120</t>
+          <t>J-320</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr"/>
@@ -9131,14 +9111,14 @@
     </row>
     <row r="211">
       <c r="A211" s="4" t="n">
-        <v>117302</v>
+        <v>105666</v>
       </c>
       <c r="B211" s="4" t="n">
-        <v>763</v>
+        <v>820</v>
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>J-320</t>
         </is>
       </c>
       <c r="D211" s="4" t="inlineStr"/>
@@ -9147,14 +9127,14 @@
     </row>
     <row r="212">
       <c r="A212" s="4" t="n">
-        <v>117302</v>
+        <v>105666</v>
       </c>
       <c r="B212" s="4" t="n">
-        <v>763</v>
+        <v>820</v>
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>J-320</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr"/>
@@ -9163,14 +9143,14 @@
     </row>
     <row r="213">
       <c r="A213" s="4" t="n">
-        <v>117302</v>
+        <v>105666</v>
       </c>
       <c r="B213" s="4" t="n">
-        <v>721</v>
+        <v>820</v>
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>J-320</t>
         </is>
       </c>
       <c r="D213" s="4" t="inlineStr"/>
@@ -9179,14 +9159,14 @@
     </row>
     <row r="214">
       <c r="A214" s="4" t="n">
-        <v>117302</v>
+        <v>105666</v>
       </c>
       <c r="B214" s="4" t="n">
-        <v>721</v>
+        <v>810</v>
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>J-320</t>
         </is>
       </c>
       <c r="D214" s="4" t="inlineStr"/>
@@ -9195,14 +9175,14 @@
     </row>
     <row r="215">
       <c r="A215" s="4" t="n">
-        <v>117302</v>
+        <v>102255</v>
       </c>
       <c r="B215" s="4" t="n">
-        <v>721</v>
+        <v>206</v>
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>J-120</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr"/>
@@ -9211,14 +9191,14 @@
     </row>
     <row r="216">
       <c r="A216" s="4" t="n">
-        <v>105642</v>
+        <v>102255</v>
       </c>
       <c r="B216" s="4" t="n">
-        <v>955</v>
+        <v>203</v>
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Success Center</t>
+          <t>J-120</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr"/>
@@ -9227,14 +9207,14 @@
     </row>
     <row r="217">
       <c r="A217" s="4" t="n">
-        <v>105642</v>
+        <v>102255</v>
       </c>
       <c r="B217" s="4" t="n">
-        <v>955</v>
+        <v>203</v>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Success Center</t>
+          <t>J-120</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr"/>
@@ -9243,14 +9223,14 @@
     </row>
     <row r="218">
       <c r="A218" s="4" t="n">
-        <v>105642</v>
+        <v>102255</v>
       </c>
       <c r="B218" s="4" t="n">
-        <v>955</v>
+        <v>201</v>
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>Success Center</t>
+          <t>J-120</t>
         </is>
       </c>
       <c r="D218" s="4" t="inlineStr"/>
@@ -9259,14 +9239,14 @@
     </row>
     <row r="219">
       <c r="A219" s="4" t="n">
-        <v>105642</v>
+        <v>102255</v>
       </c>
       <c r="B219" s="4" t="n">
-        <v>122</v>
+        <v>220</v>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>J-120</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr"/>
@@ -9275,14 +9255,14 @@
     </row>
     <row r="220">
       <c r="A220" s="4" t="n">
-        <v>117304</v>
+        <v>102255</v>
       </c>
       <c r="B220" s="4" t="n">
-        <v>570</v>
+        <v>209</v>
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>J-120</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr"/>
@@ -9290,47 +9270,51 @@
       <c r="F220" s="4" t="inlineStr"/>
     </row>
     <row r="221">
-      <c r="A221" s="4" t="n">
-        <v>117304</v>
-      </c>
-      <c r="B221" s="4" t="n">
-        <v>570</v>
-      </c>
-      <c r="C221" s="4" t="inlineStr">
-        <is>
-          <t>S-338</t>
-        </is>
-      </c>
-      <c r="D221" s="4" t="inlineStr"/>
-      <c r="E221" s="4" t="inlineStr"/>
-      <c r="F221" s="4" t="inlineStr"/>
+      <c r="A221" t="n">
+        <v>102255</v>
+      </c>
+      <c r="B221" t="n">
+        <v>201</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>J-120</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
     </row>
     <row r="222">
-      <c r="A222" s="4" t="n">
-        <v>117304</v>
-      </c>
-      <c r="B222" s="4" t="n">
-        <v>585</v>
-      </c>
-      <c r="C222" s="4" t="inlineStr">
-        <is>
-          <t>S-338</t>
-        </is>
-      </c>
-      <c r="D222" s="4" t="inlineStr"/>
-      <c r="E222" s="4" t="inlineStr"/>
-      <c r="F222" s="4" t="inlineStr"/>
+      <c r="A222" t="n">
+        <v>102255</v>
+      </c>
+      <c r="B222" t="n">
+        <v>201</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>J-120</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n">
-        <v>117304</v>
+        <v>117302</v>
       </c>
       <c r="B223" s="4" t="n">
-        <v>585</v>
+        <v>763</v>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr"/>
@@ -9339,14 +9323,14 @@
     </row>
     <row r="224">
       <c r="A224" s="4" t="n">
-        <v>117304</v>
+        <v>117302</v>
       </c>
       <c r="B224" s="4" t="n">
-        <v>580</v>
+        <v>763</v>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr"/>
@@ -9355,14 +9339,14 @@
     </row>
     <row r="225">
       <c r="A225" s="4" t="n">
-        <v>117304</v>
+        <v>117302</v>
       </c>
       <c r="B225" s="4" t="n">
-        <v>580</v>
+        <v>721</v>
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr"/>
@@ -9371,14 +9355,14 @@
     </row>
     <row r="226">
       <c r="A226" s="4" t="n">
-        <v>117304</v>
+        <v>117302</v>
       </c>
       <c r="B226" s="4" t="n">
-        <v>580</v>
+        <v>721</v>
       </c>
       <c r="C226" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D226" s="4" t="inlineStr"/>
@@ -9387,14 +9371,14 @@
     </row>
     <row r="227">
       <c r="A227" s="4" t="n">
-        <v>117304</v>
+        <v>117302</v>
       </c>
       <c r="B227" s="4" t="n">
-        <v>580</v>
+        <v>721</v>
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr"/>
@@ -9403,94 +9387,78 @@
     </row>
     <row r="228">
       <c r="A228" s="4" t="n">
-        <v>117304</v>
+        <v>105642</v>
       </c>
       <c r="B228" s="4" t="n">
-        <v>590</v>
+        <v>955</v>
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>Success Center</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr"/>
-      <c r="E228" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E228" s="4" t="inlineStr"/>
       <c r="F228" s="4" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="n">
-        <v>117304</v>
+        <v>105642</v>
       </c>
       <c r="B229" s="4" t="n">
-        <v>590</v>
+        <v>955</v>
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>Success Center</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr"/>
-      <c r="E229" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E229" s="4" t="inlineStr"/>
       <c r="F229" s="4" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="n">
-        <v>117304</v>
+        <v>105642</v>
       </c>
       <c r="B230" s="4" t="n">
-        <v>591</v>
+        <v>955</v>
       </c>
       <c r="C230" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>Success Center</t>
         </is>
       </c>
       <c r="D230" s="4" t="inlineStr"/>
-      <c r="E230" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E230" s="4" t="inlineStr"/>
       <c r="F230" s="4" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="n">
-        <v>117304</v>
+        <v>105642</v>
       </c>
       <c r="B231" s="4" t="n">
-        <v>591</v>
+        <v>122</v>
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr"/>
-      <c r="E231" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E231" s="4" t="inlineStr"/>
       <c r="F231" s="4" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="n">
-        <v>112092</v>
+        <v>117304</v>
       </c>
       <c r="B232" s="4" t="n">
-        <v>521</v>
+        <v>570</v>
       </c>
       <c r="C232" s="4" t="inlineStr">
         <is>
-          <t>D-204</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D232" s="4" t="inlineStr"/>
@@ -9499,14 +9467,14 @@
     </row>
     <row r="233">
       <c r="A233" s="4" t="n">
-        <v>112092</v>
+        <v>117304</v>
       </c>
       <c r="B233" s="4" t="n">
-        <v>521</v>
+        <v>570</v>
       </c>
       <c r="C233" s="4" t="inlineStr">
         <is>
-          <t>D-204</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D233" s="4" t="inlineStr"/>
@@ -9515,14 +9483,14 @@
     </row>
     <row r="234">
       <c r="A234" s="4" t="n">
-        <v>112092</v>
+        <v>117304</v>
       </c>
       <c r="B234" s="4" t="n">
-        <v>521</v>
+        <v>585</v>
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
-          <t>D-204</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D234" s="4" t="inlineStr"/>
@@ -9531,14 +9499,14 @@
     </row>
     <row r="235">
       <c r="A235" s="4" t="n">
-        <v>112092</v>
+        <v>117304</v>
       </c>
       <c r="B235" s="4" t="n">
-        <v>521</v>
+        <v>585</v>
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
-          <t>D-204</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D235" s="4" t="inlineStr"/>
@@ -9547,14 +9515,14 @@
     </row>
     <row r="236">
       <c r="A236" s="4" t="n">
-        <v>112092</v>
+        <v>117304</v>
       </c>
       <c r="B236" s="4" t="n">
-        <v>531</v>
+        <v>580</v>
       </c>
       <c r="C236" s="4" t="inlineStr">
         <is>
-          <t>D-204</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D236" s="4" t="inlineStr"/>
@@ -9563,14 +9531,14 @@
     </row>
     <row r="237">
       <c r="A237" s="4" t="n">
-        <v>105671</v>
+        <v>117304</v>
       </c>
       <c r="B237" s="4" t="n">
-        <v>720</v>
+        <v>580</v>
       </c>
       <c r="C237" s="4" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D237" s="4" t="inlineStr"/>
@@ -9579,14 +9547,14 @@
     </row>
     <row r="238">
       <c r="A238" s="4" t="n">
-        <v>105671</v>
+        <v>117304</v>
       </c>
       <c r="B238" s="4" t="n">
-        <v>720</v>
+        <v>580</v>
       </c>
       <c r="C238" s="4" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D238" s="4" t="inlineStr"/>
@@ -9595,14 +9563,14 @@
     </row>
     <row r="239">
       <c r="A239" s="4" t="n">
-        <v>105671</v>
+        <v>117304</v>
       </c>
       <c r="B239" s="4" t="n">
-        <v>720</v>
+        <v>580</v>
       </c>
       <c r="C239" s="4" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D239" s="4" t="inlineStr"/>
@@ -9611,78 +9579,94 @@
     </row>
     <row r="240">
       <c r="A240" s="4" t="n">
-        <v>105671</v>
+        <v>117304</v>
       </c>
       <c r="B240" s="4" t="n">
-        <v>720</v>
+        <v>590</v>
       </c>
       <c r="C240" s="4" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D240" s="4" t="inlineStr"/>
-      <c r="E240" s="4" t="inlineStr"/>
+      <c r="E240" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F240" s="4" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="n">
-        <v>105671</v>
+        <v>117304</v>
       </c>
       <c r="B241" s="4" t="n">
-        <v>720</v>
+        <v>590</v>
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D241" s="4" t="inlineStr"/>
-      <c r="E241" s="4" t="inlineStr"/>
+      <c r="E241" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F241" s="4" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="n">
-        <v>106762</v>
+        <v>117304</v>
       </c>
       <c r="B242" s="4" t="n">
-        <v>352</v>
+        <v>591</v>
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D242" s="4" t="inlineStr"/>
-      <c r="E242" s="4" t="inlineStr"/>
+      <c r="E242" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F242" s="4" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="n">
-        <v>106762</v>
+        <v>117304</v>
       </c>
       <c r="B243" s="4" t="n">
-        <v>322</v>
+        <v>591</v>
       </c>
       <c r="C243" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D243" s="4" t="inlineStr"/>
-      <c r="E243" s="4" t="inlineStr"/>
+      <c r="E243" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F243" s="4" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="n">
-        <v>106762</v>
+        <v>112092</v>
       </c>
       <c r="B244" s="4" t="n">
-        <v>322</v>
+        <v>521</v>
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>D-204</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr"/>
@@ -9691,14 +9675,14 @@
     </row>
     <row r="245">
       <c r="A245" s="4" t="n">
-        <v>106762</v>
+        <v>112092</v>
       </c>
       <c r="B245" s="4" t="n">
-        <v>323</v>
+        <v>521</v>
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>D-204</t>
         </is>
       </c>
       <c r="D245" s="4" t="inlineStr"/>
@@ -9707,14 +9691,14 @@
     </row>
     <row r="246">
       <c r="A246" s="4" t="n">
-        <v>106762</v>
+        <v>112092</v>
       </c>
       <c r="B246" s="4" t="n">
-        <v>332</v>
+        <v>521</v>
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>D-204</t>
         </is>
       </c>
       <c r="D246" s="4" t="inlineStr"/>
@@ -9723,14 +9707,14 @@
     </row>
     <row r="247">
       <c r="A247" s="4" t="n">
-        <v>106762</v>
+        <v>112092</v>
       </c>
       <c r="B247" s="4" t="n">
-        <v>333</v>
+        <v>521</v>
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>D-204</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr"/>
@@ -9739,14 +9723,14 @@
     </row>
     <row r="248">
       <c r="A248" s="4" t="n">
-        <v>105616</v>
+        <v>112092</v>
       </c>
       <c r="B248" s="4" t="n">
-        <v>722</v>
+        <v>531</v>
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>I-119</t>
+          <t>D-204</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr"/>
@@ -9755,14 +9739,14 @@
     </row>
     <row r="249">
       <c r="A249" s="4" t="n">
-        <v>105616</v>
+        <v>105671</v>
       </c>
       <c r="B249" s="4" t="n">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
-          <t>I-119</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="D249" s="4" t="inlineStr"/>
@@ -9771,14 +9755,14 @@
     </row>
     <row r="250">
       <c r="A250" s="4" t="n">
-        <v>105616</v>
+        <v>105671</v>
       </c>
       <c r="B250" s="4" t="n">
-        <v>733</v>
+        <v>720</v>
       </c>
       <c r="C250" s="4" t="inlineStr">
         <is>
-          <t>I-119</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="D250" s="4" t="inlineStr"/>
@@ -9787,14 +9771,14 @@
     </row>
     <row r="251">
       <c r="A251" s="4" t="n">
-        <v>105616</v>
+        <v>105671</v>
       </c>
       <c r="B251" s="4" t="n">
-        <v>733</v>
+        <v>720</v>
       </c>
       <c r="C251" s="4" t="inlineStr">
         <is>
-          <t>I-119</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="D251" s="4" t="inlineStr"/>
@@ -9803,14 +9787,14 @@
     </row>
     <row r="252">
       <c r="A252" s="4" t="n">
-        <v>105616</v>
+        <v>105671</v>
       </c>
       <c r="B252" s="4" t="n">
-        <v>733</v>
+        <v>720</v>
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>I-119</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr"/>
@@ -9819,14 +9803,14 @@
     </row>
     <row r="253">
       <c r="A253" s="4" t="n">
-        <v>108420</v>
+        <v>105671</v>
       </c>
       <c r="B253" s="4" t="n">
-        <v>120</v>
+        <v>720</v>
       </c>
       <c r="C253" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="D253" s="4" t="inlineStr"/>
@@ -9835,14 +9819,14 @@
     </row>
     <row r="254">
       <c r="A254" s="4" t="n">
-        <v>108420</v>
+        <v>106762</v>
       </c>
       <c r="B254" s="4" t="n">
-        <v>140</v>
+        <v>352</v>
       </c>
       <c r="C254" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D254" s="4" t="inlineStr"/>
@@ -9851,14 +9835,14 @@
     </row>
     <row r="255">
       <c r="A255" s="4" t="n">
-        <v>108420</v>
+        <v>106762</v>
       </c>
       <c r="B255" s="4" t="n">
-        <v>140</v>
+        <v>322</v>
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D255" s="4" t="inlineStr"/>
@@ -9867,14 +9851,14 @@
     </row>
     <row r="256">
       <c r="A256" s="4" t="n">
-        <v>108420</v>
+        <v>106762</v>
       </c>
       <c r="B256" s="4" t="n">
-        <v>140</v>
+        <v>322</v>
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D256" s="4" t="inlineStr"/>
@@ -9883,14 +9867,14 @@
     </row>
     <row r="257">
       <c r="A257" s="4" t="n">
-        <v>108420</v>
+        <v>106762</v>
       </c>
       <c r="B257" s="4" t="n">
-        <v>146</v>
+        <v>323</v>
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D257" s="4" t="inlineStr"/>
@@ -9899,14 +9883,14 @@
     </row>
     <row r="258">
       <c r="A258" s="4" t="n">
-        <v>105617</v>
+        <v>106762</v>
       </c>
       <c r="B258" s="4" t="n">
-        <v>121</v>
+        <v>332</v>
       </c>
       <c r="C258" s="4" t="inlineStr">
         <is>
-          <t>D-101</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D258" s="4" t="inlineStr"/>
@@ -9915,14 +9899,14 @@
     </row>
     <row r="259">
       <c r="A259" s="4" t="n">
-        <v>105617</v>
+        <v>106762</v>
       </c>
       <c r="B259" s="4" t="n">
-        <v>121</v>
+        <v>333</v>
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>D-101</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr"/>
@@ -9931,14 +9915,14 @@
     </row>
     <row r="260">
       <c r="A260" s="4" t="n">
-        <v>105617</v>
+        <v>105616</v>
       </c>
       <c r="B260" s="4" t="n">
-        <v>149</v>
+        <v>722</v>
       </c>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>D-101</t>
+          <t>I-119</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr"/>
@@ -9947,14 +9931,14 @@
     </row>
     <row r="261">
       <c r="A261" s="4" t="n">
-        <v>105617</v>
+        <v>105616</v>
       </c>
       <c r="B261" s="4" t="n">
-        <v>149</v>
+        <v>722</v>
       </c>
       <c r="C261" s="4" t="inlineStr">
         <is>
-          <t>D-101</t>
+          <t>I-119</t>
         </is>
       </c>
       <c r="D261" s="4" t="inlineStr"/>
@@ -9963,14 +9947,14 @@
     </row>
     <row r="262">
       <c r="A262" s="4" t="n">
-        <v>105617</v>
+        <v>105616</v>
       </c>
       <c r="B262" s="4" t="n">
-        <v>110</v>
+        <v>733</v>
       </c>
       <c r="C262" s="4" t="inlineStr">
         <is>
-          <t>D-101</t>
+          <t>I-119</t>
         </is>
       </c>
       <c r="D262" s="4" t="inlineStr"/>
@@ -9979,74 +9963,94 @@
     </row>
     <row r="263">
       <c r="A263" s="4" t="n">
-        <v>122121</v>
+        <v>105616</v>
       </c>
       <c r="B263" s="4" t="n">
-        <v>410</v>
-      </c>
-      <c r="C263" s="4" t="inlineStr"/>
+        <v>733</v>
+      </c>
+      <c r="C263" s="4" t="inlineStr">
+        <is>
+          <t>I-119</t>
+        </is>
+      </c>
       <c r="D263" s="4" t="inlineStr"/>
       <c r="E263" s="4" t="inlineStr"/>
       <c r="F263" s="4" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n">
-        <v>122121</v>
+        <v>105616</v>
       </c>
       <c r="B264" s="4" t="n">
-        <v>410</v>
-      </c>
-      <c r="C264" s="4" t="inlineStr"/>
+        <v>733</v>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>I-119</t>
+        </is>
+      </c>
       <c r="D264" s="4" t="inlineStr"/>
       <c r="E264" s="4" t="inlineStr"/>
       <c r="F264" s="4" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n">
-        <v>122121</v>
+        <v>108420</v>
       </c>
       <c r="B265" s="4" t="n">
-        <v>410</v>
-      </c>
-      <c r="C265" s="4" t="inlineStr"/>
+        <v>120</v>
+      </c>
+      <c r="C265" s="4" t="inlineStr">
+        <is>
+          <t>D-104</t>
+        </is>
+      </c>
       <c r="D265" s="4" t="inlineStr"/>
       <c r="E265" s="4" t="inlineStr"/>
       <c r="F265" s="4" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n">
-        <v>122121</v>
+        <v>108420</v>
       </c>
       <c r="B266" s="4" t="n">
-        <v>420</v>
-      </c>
-      <c r="C266" s="4" t="inlineStr"/>
+        <v>140</v>
+      </c>
+      <c r="C266" s="4" t="inlineStr">
+        <is>
+          <t>D-104</t>
+        </is>
+      </c>
       <c r="D266" s="4" t="inlineStr"/>
       <c r="E266" s="4" t="inlineStr"/>
       <c r="F266" s="4" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n">
-        <v>122121</v>
+        <v>108420</v>
       </c>
       <c r="B267" s="4" t="n">
-        <v>420</v>
-      </c>
-      <c r="C267" s="4" t="inlineStr"/>
+        <v>140</v>
+      </c>
+      <c r="C267" s="4" t="inlineStr">
+        <is>
+          <t>D-104</t>
+        </is>
+      </c>
       <c r="D267" s="4" t="inlineStr"/>
       <c r="E267" s="4" t="inlineStr"/>
       <c r="F267" s="4" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n">
-        <v>105624</v>
+        <v>108420</v>
       </c>
       <c r="B268" s="4" t="n">
-        <v>830</v>
+        <v>140</v>
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>D-104</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr"/>
@@ -10055,14 +10059,14 @@
     </row>
     <row r="269">
       <c r="A269" s="4" t="n">
-        <v>105624</v>
+        <v>108420</v>
       </c>
       <c r="B269" s="4" t="n">
-        <v>830</v>
+        <v>146</v>
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>D-104</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr"/>
@@ -10071,14 +10075,14 @@
     </row>
     <row r="270">
       <c r="A270" s="4" t="n">
-        <v>105624</v>
+        <v>105617</v>
       </c>
       <c r="B270" s="4" t="n">
-        <v>830</v>
+        <v>121</v>
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr"/>
@@ -10087,14 +10091,14 @@
     </row>
     <row r="271">
       <c r="A271" s="4" t="n">
-        <v>105624</v>
+        <v>105617</v>
       </c>
       <c r="B271" s="4" t="n">
-        <v>830</v>
+        <v>121</v>
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr"/>
@@ -10103,14 +10107,14 @@
     </row>
     <row r="272">
       <c r="A272" s="4" t="n">
-        <v>105624</v>
+        <v>105617</v>
       </c>
       <c r="B272" s="4" t="n">
-        <v>830</v>
+        <v>149</v>
       </c>
       <c r="C272" s="4" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="D272" s="4" t="inlineStr"/>
@@ -10119,14 +10123,14 @@
     </row>
     <row r="273">
       <c r="A273" s="4" t="n">
-        <v>122122</v>
+        <v>105617</v>
       </c>
       <c r="B273" s="4" t="n">
-        <v>2054</v>
+        <v>149</v>
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>I-111</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr"/>
@@ -10135,14 +10139,14 @@
     </row>
     <row r="274">
       <c r="A274" s="4" t="n">
-        <v>122122</v>
+        <v>105617</v>
       </c>
       <c r="B274" s="4" t="n">
-        <v>2054</v>
+        <v>110</v>
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
-          <t>I-111</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr"/>
@@ -10151,94 +10155,74 @@
     </row>
     <row r="275">
       <c r="A275" s="4" t="n">
-        <v>122122</v>
+        <v>122121</v>
       </c>
       <c r="B275" s="4" t="n">
-        <v>2014</v>
-      </c>
-      <c r="C275" s="4" t="inlineStr">
-        <is>
-          <t>I-111</t>
-        </is>
-      </c>
+        <v>410</v>
+      </c>
+      <c r="C275" s="4" t="inlineStr"/>
       <c r="D275" s="4" t="inlineStr"/>
       <c r="E275" s="4" t="inlineStr"/>
       <c r="F275" s="4" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n">
-        <v>122122</v>
+        <v>122121</v>
       </c>
       <c r="B276" s="4" t="n">
-        <v>2014</v>
-      </c>
-      <c r="C276" s="4" t="inlineStr">
-        <is>
-          <t>I-111</t>
-        </is>
-      </c>
+        <v>410</v>
+      </c>
+      <c r="C276" s="4" t="inlineStr"/>
       <c r="D276" s="4" t="inlineStr"/>
       <c r="E276" s="4" t="inlineStr"/>
       <c r="F276" s="4" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="n">
-        <v>122122</v>
+        <v>122121</v>
       </c>
       <c r="B277" s="4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C277" s="4" t="inlineStr">
-        <is>
-          <t>I-111</t>
-        </is>
-      </c>
+        <v>410</v>
+      </c>
+      <c r="C277" s="4" t="inlineStr"/>
       <c r="D277" s="4" t="inlineStr"/>
       <c r="E277" s="4" t="inlineStr"/>
       <c r="F277" s="4" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="n">
-        <v>122122</v>
+        <v>122121</v>
       </c>
       <c r="B278" s="4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C278" s="4" t="inlineStr">
-        <is>
-          <t>I-111</t>
-        </is>
-      </c>
+        <v>420</v>
+      </c>
+      <c r="C278" s="4" t="inlineStr"/>
       <c r="D278" s="4" t="inlineStr"/>
       <c r="E278" s="4" t="inlineStr"/>
       <c r="F278" s="4" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n">
-        <v>122122</v>
+        <v>122121</v>
       </c>
       <c r="B279" s="4" t="n">
-        <v>2034</v>
-      </c>
-      <c r="C279" s="4" t="inlineStr">
-        <is>
-          <t>I-111</t>
-        </is>
-      </c>
+        <v>420</v>
+      </c>
+      <c r="C279" s="4" t="inlineStr"/>
       <c r="D279" s="4" t="inlineStr"/>
       <c r="E279" s="4" t="inlineStr"/>
       <c r="F279" s="4" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n">
-        <v>122122</v>
+        <v>105624</v>
       </c>
       <c r="B280" s="4" t="n">
-        <v>2044</v>
+        <v>830</v>
       </c>
       <c r="C280" s="4" t="inlineStr">
         <is>
-          <t>I-111</t>
+          <t>J-221</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr"/>
@@ -10247,14 +10231,14 @@
     </row>
     <row r="281">
       <c r="A281" s="4" t="n">
-        <v>122122</v>
+        <v>105624</v>
       </c>
       <c r="B281" s="4" t="n">
-        <v>2044</v>
+        <v>830</v>
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>I-111</t>
+          <t>J-221</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr"/>
@@ -10263,14 +10247,14 @@
     </row>
     <row r="282">
       <c r="A282" s="4" t="n">
-        <v>105651</v>
+        <v>105624</v>
       </c>
       <c r="B282" s="4" t="n">
-        <v>743</v>
+        <v>830</v>
       </c>
       <c r="C282" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>J-221</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr"/>
@@ -10279,14 +10263,14 @@
     </row>
     <row r="283">
       <c r="A283" s="4" t="n">
-        <v>105651</v>
+        <v>105624</v>
       </c>
       <c r="B283" s="4" t="n">
-        <v>713</v>
+        <v>830</v>
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>J-221</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr"/>
@@ -10295,14 +10279,14 @@
     </row>
     <row r="284">
       <c r="A284" s="4" t="n">
-        <v>105651</v>
+        <v>105624</v>
       </c>
       <c r="B284" s="4" t="n">
-        <v>713</v>
+        <v>830</v>
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>J-221</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr"/>
@@ -10311,14 +10295,14 @@
     </row>
     <row r="285">
       <c r="A285" s="4" t="n">
-        <v>105651</v>
+        <v>122122</v>
       </c>
       <c r="B285" s="4" t="n">
-        <v>744</v>
+        <v>2054</v>
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr"/>
@@ -10327,14 +10311,14 @@
     </row>
     <row r="286">
       <c r="A286" s="4" t="n">
-        <v>105651</v>
+        <v>122122</v>
       </c>
       <c r="B286" s="4" t="n">
-        <v>744</v>
+        <v>2054</v>
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr"/>
@@ -10343,14 +10327,14 @@
     </row>
     <row r="287">
       <c r="A287" s="4" t="n">
-        <v>105651</v>
+        <v>122122</v>
       </c>
       <c r="B287" s="4" t="n">
-        <v>711</v>
+        <v>2014</v>
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr"/>
@@ -10359,14 +10343,14 @@
     </row>
     <row r="288">
       <c r="A288" s="4" t="n">
-        <v>105651</v>
+        <v>122122</v>
       </c>
       <c r="B288" s="4" t="n">
-        <v>711</v>
+        <v>2014</v>
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr"/>
@@ -10375,14 +10359,14 @@
     </row>
     <row r="289">
       <c r="A289" s="4" t="n">
-        <v>105618</v>
+        <v>122122</v>
       </c>
       <c r="B289" s="4" t="n">
-        <v>330</v>
+        <v>2024</v>
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>S-232</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr"/>
@@ -10391,14 +10375,14 @@
     </row>
     <row r="290">
       <c r="A290" s="4" t="n">
-        <v>105618</v>
+        <v>122122</v>
       </c>
       <c r="B290" s="4" t="n">
-        <v>330</v>
+        <v>2024</v>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>S-232</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr"/>
@@ -10407,14 +10391,14 @@
     </row>
     <row r="291">
       <c r="A291" s="4" t="n">
-        <v>105618</v>
+        <v>122122</v>
       </c>
       <c r="B291" s="4" t="n">
-        <v>331</v>
+        <v>2034</v>
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>S-232</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr"/>
@@ -10423,14 +10407,14 @@
     </row>
     <row r="292">
       <c r="A292" s="4" t="n">
-        <v>105618</v>
+        <v>122122</v>
       </c>
       <c r="B292" s="4" t="n">
-        <v>331</v>
+        <v>2044</v>
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>S-232</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr"/>
@@ -10439,14 +10423,14 @@
     </row>
     <row r="293">
       <c r="A293" s="4" t="n">
-        <v>105618</v>
+        <v>122122</v>
       </c>
       <c r="B293" s="4" t="n">
-        <v>331</v>
+        <v>2044</v>
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>S-232</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr"/>
@@ -10455,254 +10439,282 @@
     </row>
     <row r="294">
       <c r="A294" s="4" t="n">
-        <v>105808</v>
+        <v>105651</v>
       </c>
       <c r="B294" s="4" t="n">
-        <v>708</v>
-      </c>
-      <c r="C294" s="4" t="inlineStr"/>
+        <v>743</v>
+      </c>
+      <c r="C294" s="4" t="inlineStr">
+        <is>
+          <t>I-117</t>
+        </is>
+      </c>
       <c r="D294" s="4" t="inlineStr"/>
-      <c r="E294" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E294" s="4" t="inlineStr"/>
       <c r="F294" s="4" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n">
-        <v>105808</v>
+        <v>105651</v>
       </c>
       <c r="B295" s="4" t="n">
-        <v>708</v>
-      </c>
-      <c r="C295" s="4" t="inlineStr"/>
+        <v>713</v>
+      </c>
+      <c r="C295" s="4" t="inlineStr">
+        <is>
+          <t>I-117</t>
+        </is>
+      </c>
       <c r="D295" s="4" t="inlineStr"/>
-      <c r="E295" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E295" s="4" t="inlineStr"/>
       <c r="F295" s="4" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n">
-        <v>105808</v>
+        <v>105651</v>
       </c>
       <c r="B296" s="4" t="n">
-        <v>708</v>
-      </c>
-      <c r="C296" s="4" t="inlineStr"/>
+        <v>713</v>
+      </c>
+      <c r="C296" s="4" t="inlineStr">
+        <is>
+          <t>I-117</t>
+        </is>
+      </c>
       <c r="D296" s="4" t="inlineStr"/>
-      <c r="E296" s="4" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+      <c r="E296" s="4" t="inlineStr"/>
       <c r="F296" s="4" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n">
-        <v>105808</v>
+        <v>105651</v>
       </c>
       <c r="B297" s="4" t="n">
-        <v>708</v>
-      </c>
-      <c r="C297" s="4" t="inlineStr"/>
+        <v>744</v>
+      </c>
+      <c r="C297" s="4" t="inlineStr">
+        <is>
+          <t>I-117</t>
+        </is>
+      </c>
       <c r="D297" s="4" t="inlineStr"/>
-      <c r="E297" s="4" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+      <c r="E297" s="4" t="inlineStr"/>
       <c r="F297" s="4" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n">
-        <v>105808</v>
+        <v>105651</v>
       </c>
       <c r="B298" s="4" t="n">
-        <v>708</v>
-      </c>
-      <c r="C298" s="4" t="inlineStr"/>
+        <v>744</v>
+      </c>
+      <c r="C298" s="4" t="inlineStr">
+        <is>
+          <t>I-117</t>
+        </is>
+      </c>
       <c r="D298" s="4" t="inlineStr"/>
-      <c r="E298" s="4" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+      <c r="E298" s="4" t="inlineStr"/>
       <c r="F298" s="4" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n">
-        <v>117711</v>
+        <v>105651</v>
       </c>
       <c r="B299" s="4" t="n">
-        <v>751</v>
-      </c>
-      <c r="C299" s="4" t="inlineStr"/>
+        <v>711</v>
+      </c>
+      <c r="C299" s="4" t="inlineStr">
+        <is>
+          <t>I-117</t>
+        </is>
+      </c>
       <c r="D299" s="4" t="inlineStr"/>
       <c r="E299" s="4" t="inlineStr"/>
       <c r="F299" s="4" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n">
-        <v>117711</v>
+        <v>105651</v>
       </c>
       <c r="B300" s="4" t="n">
-        <v>741</v>
-      </c>
-      <c r="C300" s="4" t="inlineStr"/>
+        <v>711</v>
+      </c>
+      <c r="C300" s="4" t="inlineStr">
+        <is>
+          <t>I-117</t>
+        </is>
+      </c>
       <c r="D300" s="4" t="inlineStr"/>
       <c r="E300" s="4" t="inlineStr"/>
       <c r="F300" s="4" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n">
-        <v>117711</v>
+        <v>105618</v>
       </c>
       <c r="B301" s="4" t="n">
-        <v>741</v>
-      </c>
-      <c r="C301" s="4" t="inlineStr"/>
+        <v>330</v>
+      </c>
+      <c r="C301" s="4" t="inlineStr">
+        <is>
+          <t>S-232</t>
+        </is>
+      </c>
       <c r="D301" s="4" t="inlineStr"/>
       <c r="E301" s="4" t="inlineStr"/>
       <c r="F301" s="4" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n">
-        <v>117711</v>
+        <v>105618</v>
       </c>
       <c r="B302" s="4" t="n">
-        <v>741</v>
-      </c>
-      <c r="C302" s="4" t="inlineStr"/>
+        <v>330</v>
+      </c>
+      <c r="C302" s="4" t="inlineStr">
+        <is>
+          <t>S-232</t>
+        </is>
+      </c>
       <c r="D302" s="4" t="inlineStr"/>
       <c r="E302" s="4" t="inlineStr"/>
       <c r="F302" s="4" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n">
-        <v>117711</v>
+        <v>105618</v>
       </c>
       <c r="B303" s="4" t="n">
-        <v>710</v>
-      </c>
-      <c r="C303" s="4" t="inlineStr"/>
+        <v>331</v>
+      </c>
+      <c r="C303" s="4" t="inlineStr">
+        <is>
+          <t>S-232</t>
+        </is>
+      </c>
       <c r="D303" s="4" t="inlineStr"/>
       <c r="E303" s="4" t="inlineStr"/>
       <c r="F303" s="4" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" s="4" t="n">
-        <v>117711</v>
+        <v>105618</v>
       </c>
       <c r="B304" s="4" t="n">
-        <v>710</v>
-      </c>
-      <c r="C304" s="4" t="inlineStr"/>
+        <v>331</v>
+      </c>
+      <c r="C304" s="4" t="inlineStr">
+        <is>
+          <t>S-232</t>
+        </is>
+      </c>
       <c r="D304" s="4" t="inlineStr"/>
       <c r="E304" s="4" t="inlineStr"/>
       <c r="F304" s="4" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" s="4" t="n">
-        <v>117711</v>
+        <v>105618</v>
       </c>
       <c r="B305" s="4" t="n">
-        <v>710</v>
-      </c>
-      <c r="C305" s="4" t="inlineStr"/>
+        <v>331</v>
+      </c>
+      <c r="C305" s="4" t="inlineStr">
+        <is>
+          <t>S-232</t>
+        </is>
+      </c>
       <c r="D305" s="4" t="inlineStr"/>
       <c r="E305" s="4" t="inlineStr"/>
       <c r="F305" s="4" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" s="4" t="n">
-        <v>105803</v>
+        <v>105808</v>
       </c>
       <c r="B306" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C306" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
+        <v>708</v>
+      </c>
+      <c r="C306" s="4" t="inlineStr"/>
       <c r="D306" s="4" t="inlineStr"/>
-      <c r="E306" s="4" t="inlineStr"/>
+      <c r="E306" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F306" s="4" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" s="4" t="n">
-        <v>105803</v>
+        <v>105808</v>
       </c>
       <c r="B307" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C307" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
+        <v>708</v>
+      </c>
+      <c r="C307" s="4" t="inlineStr"/>
       <c r="D307" s="4" t="inlineStr"/>
-      <c r="E307" s="4" t="inlineStr"/>
+      <c r="E307" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F307" s="4" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" s="4" t="n">
-        <v>105803</v>
+        <v>105808</v>
       </c>
       <c r="B308" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C308" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
+        <v>708</v>
+      </c>
+      <c r="C308" s="4" t="inlineStr"/>
       <c r="D308" s="4" t="inlineStr"/>
-      <c r="E308" s="4" t="inlineStr"/>
+      <c r="E308" s="4" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
       <c r="F308" s="4" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" s="4" t="n">
-        <v>105803</v>
+        <v>105808</v>
       </c>
       <c r="B309" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C309" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
+        <v>708</v>
+      </c>
+      <c r="C309" s="4" t="inlineStr"/>
       <c r="D309" s="4" t="inlineStr"/>
-      <c r="E309" s="4" t="inlineStr"/>
+      <c r="E309" s="4" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
       <c r="F309" s="4" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" s="4" t="n">
-        <v>105803</v>
+        <v>105808</v>
       </c>
       <c r="B310" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C310" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
+        <v>708</v>
+      </c>
+      <c r="C310" s="4" t="inlineStr"/>
       <c r="D310" s="4" t="inlineStr"/>
-      <c r="E310" s="4" t="inlineStr"/>
+      <c r="E310" s="4" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
       <c r="F310" s="4" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" s="4" t="n">
-        <v>105623</v>
+        <v>117711</v>
       </c>
       <c r="B311" s="4" t="n">
-        <v>551</v>
+        <v>751</v>
       </c>
       <c r="C311" s="4" t="inlineStr"/>
       <c r="D311" s="4" t="inlineStr"/>
@@ -10711,110 +10723,86 @@
     </row>
     <row r="312">
       <c r="A312" s="4" t="n">
-        <v>105746</v>
+        <v>117711</v>
       </c>
       <c r="B312" s="4" t="n">
-        <v>556</v>
-      </c>
-      <c r="C312" s="4" t="inlineStr">
-        <is>
-          <t>D-210</t>
-        </is>
-      </c>
+        <v>741</v>
+      </c>
+      <c r="C312" s="4" t="inlineStr"/>
       <c r="D312" s="4" t="inlineStr"/>
       <c r="E312" s="4" t="inlineStr"/>
       <c r="F312" s="4" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" s="4" t="n">
-        <v>105746</v>
+        <v>117711</v>
       </c>
       <c r="B313" s="4" t="n">
-        <v>556</v>
-      </c>
-      <c r="C313" s="4" t="inlineStr">
-        <is>
-          <t>D-210</t>
-        </is>
-      </c>
+        <v>741</v>
+      </c>
+      <c r="C313" s="4" t="inlineStr"/>
       <c r="D313" s="4" t="inlineStr"/>
       <c r="E313" s="4" t="inlineStr"/>
       <c r="F313" s="4" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" s="4" t="n">
-        <v>105746</v>
+        <v>117711</v>
       </c>
       <c r="B314" s="4" t="n">
-        <v>558</v>
-      </c>
-      <c r="C314" s="4" t="inlineStr">
-        <is>
-          <t>D-210</t>
-        </is>
-      </c>
+        <v>741</v>
+      </c>
+      <c r="C314" s="4" t="inlineStr"/>
       <c r="D314" s="4" t="inlineStr"/>
       <c r="E314" s="4" t="inlineStr"/>
       <c r="F314" s="4" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" s="4" t="n">
-        <v>105746</v>
+        <v>117711</v>
       </c>
       <c r="B315" s="4" t="n">
-        <v>531</v>
-      </c>
-      <c r="C315" s="4" t="inlineStr">
-        <is>
-          <t>D-210</t>
-        </is>
-      </c>
+        <v>710</v>
+      </c>
+      <c r="C315" s="4" t="inlineStr"/>
       <c r="D315" s="4" t="inlineStr"/>
       <c r="E315" s="4" t="inlineStr"/>
       <c r="F315" s="4" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" s="4" t="n">
-        <v>105746</v>
+        <v>117711</v>
       </c>
       <c r="B316" s="4" t="n">
-        <v>531</v>
-      </c>
-      <c r="C316" s="4" t="inlineStr">
-        <is>
-          <t>D-210</t>
-        </is>
-      </c>
+        <v>710</v>
+      </c>
+      <c r="C316" s="4" t="inlineStr"/>
       <c r="D316" s="4" t="inlineStr"/>
       <c r="E316" s="4" t="inlineStr"/>
       <c r="F316" s="4" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" s="4" t="n">
-        <v>106765</v>
+        <v>117711</v>
       </c>
       <c r="B317" s="4" t="n">
-        <v>310</v>
-      </c>
-      <c r="C317" s="4" t="inlineStr">
-        <is>
-          <t>S-235</t>
-        </is>
-      </c>
+        <v>710</v>
+      </c>
+      <c r="C317" s="4" t="inlineStr"/>
       <c r="D317" s="4" t="inlineStr"/>
       <c r="E317" s="4" t="inlineStr"/>
       <c r="F317" s="4" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" s="4" t="n">
-        <v>106765</v>
+        <v>105803</v>
       </c>
       <c r="B318" s="4" t="n">
-        <v>310</v>
+        <v>110</v>
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>S-235</t>
+          <t>D-102</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr"/>
@@ -10823,14 +10811,14 @@
     </row>
     <row r="319">
       <c r="A319" s="4" t="n">
-        <v>106765</v>
+        <v>105803</v>
       </c>
       <c r="B319" s="4" t="n">
-        <v>310</v>
+        <v>110</v>
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>S-235</t>
+          <t>D-102</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr"/>
@@ -10839,14 +10827,14 @@
     </row>
     <row r="320">
       <c r="A320" s="4" t="n">
-        <v>106765</v>
+        <v>105803</v>
       </c>
       <c r="B320" s="4" t="n">
-        <v>310</v>
+        <v>110</v>
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>S-235</t>
+          <t>D-102</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr"/>
@@ -10855,14 +10843,14 @@
     </row>
     <row r="321">
       <c r="A321" s="4" t="n">
-        <v>106765</v>
+        <v>105803</v>
       </c>
       <c r="B321" s="4" t="n">
-        <v>310</v>
+        <v>110</v>
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>S-235</t>
+          <t>D-102</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr"/>
@@ -10871,22 +10859,26 @@
     </row>
     <row r="322">
       <c r="A322" s="4" t="n">
-        <v>105768</v>
+        <v>105803</v>
       </c>
       <c r="B322" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="C322" s="4" t="inlineStr"/>
+        <v>110</v>
+      </c>
+      <c r="C322" s="4" t="inlineStr">
+        <is>
+          <t>D-102</t>
+        </is>
+      </c>
       <c r="D322" s="4" t="inlineStr"/>
       <c r="E322" s="4" t="inlineStr"/>
       <c r="F322" s="4" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" s="4" t="n">
-        <v>105768</v>
+        <v>105623</v>
       </c>
       <c r="B323" s="4" t="n">
-        <v>132</v>
+        <v>551</v>
       </c>
       <c r="C323" s="4" t="inlineStr"/>
       <c r="D323" s="4" t="inlineStr"/>
@@ -10895,38 +10887,46 @@
     </row>
     <row r="324">
       <c r="A324" s="4" t="n">
-        <v>105768</v>
+        <v>105746</v>
       </c>
       <c r="B324" s="4" t="n">
-        <v>143</v>
-      </c>
-      <c r="C324" s="4" t="inlineStr"/>
+        <v>556</v>
+      </c>
+      <c r="C324" s="4" t="inlineStr">
+        <is>
+          <t>D-210</t>
+        </is>
+      </c>
       <c r="D324" s="4" t="inlineStr"/>
       <c r="E324" s="4" t="inlineStr"/>
       <c r="F324" s="4" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" s="4" t="n">
-        <v>105768</v>
+        <v>105746</v>
       </c>
       <c r="B325" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="C325" s="4" t="inlineStr"/>
+        <v>556</v>
+      </c>
+      <c r="C325" s="4" t="inlineStr">
+        <is>
+          <t>D-210</t>
+        </is>
+      </c>
       <c r="D325" s="4" t="inlineStr"/>
       <c r="E325" s="4" t="inlineStr"/>
       <c r="F325" s="4" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" s="4" t="n">
-        <v>106623</v>
+        <v>105746</v>
       </c>
       <c r="B326" s="4" t="n">
-        <v>410</v>
+        <v>558</v>
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-210</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr"/>
@@ -10935,14 +10935,14 @@
     </row>
     <row r="327">
       <c r="A327" s="4" t="n">
-        <v>106623</v>
+        <v>105746</v>
       </c>
       <c r="B327" s="4" t="n">
-        <v>410</v>
+        <v>531</v>
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-210</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr"/>
@@ -10951,14 +10951,14 @@
     </row>
     <row r="328">
       <c r="A328" s="4" t="n">
-        <v>106623</v>
+        <v>105746</v>
       </c>
       <c r="B328" s="4" t="n">
-        <v>410</v>
+        <v>531</v>
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-210</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr"/>
@@ -10967,14 +10967,14 @@
     </row>
     <row r="329">
       <c r="A329" s="4" t="n">
-        <v>106623</v>
+        <v>106765</v>
       </c>
       <c r="B329" s="4" t="n">
-        <v>411</v>
+        <v>310</v>
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>S-235</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr"/>
@@ -10983,14 +10983,14 @@
     </row>
     <row r="330">
       <c r="A330" s="4" t="n">
-        <v>106623</v>
+        <v>106765</v>
       </c>
       <c r="B330" s="4" t="n">
-        <v>420</v>
+        <v>310</v>
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>S-235</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr"/>
@@ -10999,14 +10999,14 @@
     </row>
     <row r="331">
       <c r="A331" s="4" t="n">
-        <v>105883</v>
+        <v>106765</v>
       </c>
       <c r="B331" s="4" t="n">
-        <v>756</v>
+        <v>310</v>
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>I-012</t>
+          <t>S-235</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr"/>
@@ -11015,14 +11015,14 @@
     </row>
     <row r="332">
       <c r="A332" s="4" t="n">
-        <v>105883</v>
+        <v>106765</v>
       </c>
       <c r="B332" s="4" t="n">
-        <v>730</v>
+        <v>310</v>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>I-012</t>
+          <t>S-235</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr"/>
@@ -11031,14 +11031,14 @@
     </row>
     <row r="333">
       <c r="A333" s="4" t="n">
-        <v>105883</v>
+        <v>106765</v>
       </c>
       <c r="B333" s="4" t="n">
-        <v>731</v>
+        <v>310</v>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>I-012</t>
+          <t>S-235</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr"/>
@@ -11047,110 +11047,78 @@
     </row>
     <row r="334">
       <c r="A334" s="4" t="n">
-        <v>105883</v>
+        <v>105768</v>
       </c>
       <c r="B334" s="4" t="n">
-        <v>710</v>
-      </c>
-      <c r="C334" s="4" t="inlineStr">
-        <is>
-          <t>I-012</t>
-        </is>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="C334" s="4" t="inlineStr"/>
       <c r="D334" s="4" t="inlineStr"/>
       <c r="E334" s="4" t="inlineStr"/>
       <c r="F334" s="4" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" s="4" t="n">
-        <v>105883</v>
+        <v>105768</v>
       </c>
       <c r="B335" s="4" t="n">
-        <v>710</v>
-      </c>
-      <c r="C335" s="4" t="inlineStr">
-        <is>
-          <t>I-012</t>
-        </is>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="C335" s="4" t="inlineStr"/>
       <c r="D335" s="4" t="inlineStr"/>
       <c r="E335" s="4" t="inlineStr"/>
       <c r="F335" s="4" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" s="4" t="n">
-        <v>105883</v>
+        <v>105768</v>
       </c>
       <c r="B336" s="4" t="n">
-        <v>710</v>
-      </c>
-      <c r="C336" s="4" t="inlineStr">
-        <is>
-          <t>I-012</t>
-        </is>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="C336" s="4" t="inlineStr"/>
       <c r="D336" s="4" t="inlineStr"/>
       <c r="E336" s="4" t="inlineStr"/>
       <c r="F336" s="4" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" s="4" t="n">
-        <v>105620</v>
+        <v>105768</v>
       </c>
       <c r="B337" s="4" t="n">
-        <v>732</v>
-      </c>
-      <c r="C337" s="4" t="inlineStr">
-        <is>
-          <t>S-233</t>
-        </is>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="C337" s="4" t="inlineStr"/>
       <c r="D337" s="4" t="inlineStr"/>
       <c r="E337" s="4" t="inlineStr"/>
       <c r="F337" s="4" t="inlineStr"/>
     </row>
     <row r="338">
-      <c r="A338" s="4" t="n">
-        <v>105620</v>
-      </c>
-      <c r="B338" s="4" t="n">
-        <v>732</v>
-      </c>
-      <c r="C338" s="4" t="inlineStr">
-        <is>
-          <t>S-233</t>
-        </is>
-      </c>
-      <c r="D338" s="4" t="inlineStr"/>
-      <c r="E338" s="4" t="inlineStr"/>
-      <c r="F338" s="4" t="inlineStr"/>
+      <c r="A338" t="n">
+        <v>105768</v>
+      </c>
+      <c r="B338" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="339">
-      <c r="A339" s="4" t="n">
-        <v>105620</v>
-      </c>
-      <c r="B339" s="4" t="n">
-        <v>742</v>
-      </c>
-      <c r="C339" s="4" t="inlineStr">
-        <is>
-          <t>S-233</t>
-        </is>
-      </c>
-      <c r="D339" s="4" t="inlineStr"/>
-      <c r="E339" s="4" t="inlineStr"/>
-      <c r="F339" s="4" t="inlineStr"/>
+      <c r="A339" t="n">
+        <v>105768</v>
+      </c>
+      <c r="B339" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="4" t="n">
-        <v>105620</v>
+        <v>106623</v>
       </c>
       <c r="B340" s="4" t="n">
-        <v>742</v>
+        <v>410</v>
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
-          <t>S-233</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr"/>
@@ -11159,14 +11127,14 @@
     </row>
     <row r="341">
       <c r="A341" s="4" t="n">
-        <v>105620</v>
+        <v>106623</v>
       </c>
       <c r="B341" s="4" t="n">
-        <v>752</v>
+        <v>410</v>
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t>S-233</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr"/>
@@ -11175,14 +11143,14 @@
     </row>
     <row r="342">
       <c r="A342" s="4" t="n">
-        <v>105620</v>
+        <v>106623</v>
       </c>
       <c r="B342" s="4" t="n">
-        <v>752</v>
+        <v>410</v>
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
-          <t>S-233</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr"/>
@@ -11191,14 +11159,14 @@
     </row>
     <row r="343">
       <c r="A343" s="4" t="n">
-        <v>105729</v>
+        <v>106623</v>
       </c>
       <c r="B343" s="4" t="n">
-        <v>359</v>
+        <v>411</v>
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
-          <t>S-236</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr"/>
@@ -11207,14 +11175,14 @@
     </row>
     <row r="344">
       <c r="A344" s="4" t="n">
-        <v>105729</v>
+        <v>106623</v>
       </c>
       <c r="B344" s="4" t="n">
-        <v>312</v>
+        <v>420</v>
       </c>
       <c r="C344" s="4" t="inlineStr">
         <is>
-          <t>S-236</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr"/>
@@ -11223,14 +11191,14 @@
     </row>
     <row r="345">
       <c r="A345" s="4" t="n">
-        <v>105729</v>
+        <v>105883</v>
       </c>
       <c r="B345" s="4" t="n">
-        <v>312</v>
+        <v>756</v>
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
-          <t>S-236</t>
+          <t>I-012</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr"/>
@@ -11239,14 +11207,14 @@
     </row>
     <row r="346">
       <c r="A346" s="4" t="n">
-        <v>105729</v>
+        <v>105883</v>
       </c>
       <c r="B346" s="4" t="n">
-        <v>315</v>
+        <v>730</v>
       </c>
       <c r="C346" s="4" t="inlineStr">
         <is>
-          <t>S-236</t>
+          <t>I-012</t>
         </is>
       </c>
       <c r="D346" s="4" t="inlineStr"/>
@@ -11255,14 +11223,14 @@
     </row>
     <row r="347">
       <c r="A347" s="4" t="n">
-        <v>105729</v>
+        <v>105883</v>
       </c>
       <c r="B347" s="4" t="n">
-        <v>327</v>
+        <v>731</v>
       </c>
       <c r="C347" s="4" t="inlineStr">
         <is>
-          <t>S-236</t>
+          <t>I-012</t>
         </is>
       </c>
       <c r="D347" s="4" t="inlineStr"/>
@@ -11271,19 +11239,243 @@
     </row>
     <row r="348">
       <c r="A348" s="4" t="n">
-        <v>105729</v>
+        <v>105883</v>
       </c>
       <c r="B348" s="4" t="n">
-        <v>339</v>
+        <v>710</v>
       </c>
       <c r="C348" s="4" t="inlineStr">
         <is>
-          <t>S-236</t>
+          <t>I-012</t>
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr"/>
       <c r="E348" s="4" t="inlineStr"/>
       <c r="F348" s="4" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="4" t="n">
+        <v>105883</v>
+      </c>
+      <c r="B349" s="4" t="n">
+        <v>710</v>
+      </c>
+      <c r="C349" s="4" t="inlineStr">
+        <is>
+          <t>I-012</t>
+        </is>
+      </c>
+      <c r="D349" s="4" t="inlineStr"/>
+      <c r="E349" s="4" t="inlineStr"/>
+      <c r="F349" s="4" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="4" t="n">
+        <v>105883</v>
+      </c>
+      <c r="B350" s="4" t="n">
+        <v>710</v>
+      </c>
+      <c r="C350" s="4" t="inlineStr">
+        <is>
+          <t>I-012</t>
+        </is>
+      </c>
+      <c r="D350" s="4" t="inlineStr"/>
+      <c r="E350" s="4" t="inlineStr"/>
+      <c r="F350" s="4" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="4" t="n">
+        <v>105620</v>
+      </c>
+      <c r="B351" s="4" t="n">
+        <v>732</v>
+      </c>
+      <c r="C351" s="4" t="inlineStr">
+        <is>
+          <t>S-233</t>
+        </is>
+      </c>
+      <c r="D351" s="4" t="inlineStr"/>
+      <c r="E351" s="4" t="inlineStr"/>
+      <c r="F351" s="4" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="4" t="n">
+        <v>105620</v>
+      </c>
+      <c r="B352" s="4" t="n">
+        <v>732</v>
+      </c>
+      <c r="C352" s="4" t="inlineStr">
+        <is>
+          <t>S-233</t>
+        </is>
+      </c>
+      <c r="D352" s="4" t="inlineStr"/>
+      <c r="E352" s="4" t="inlineStr"/>
+      <c r="F352" s="4" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="4" t="n">
+        <v>105620</v>
+      </c>
+      <c r="B353" s="4" t="n">
+        <v>742</v>
+      </c>
+      <c r="C353" s="4" t="inlineStr">
+        <is>
+          <t>S-233</t>
+        </is>
+      </c>
+      <c r="D353" s="4" t="inlineStr"/>
+      <c r="E353" s="4" t="inlineStr"/>
+      <c r="F353" s="4" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="4" t="n">
+        <v>105620</v>
+      </c>
+      <c r="B354" s="4" t="n">
+        <v>742</v>
+      </c>
+      <c r="C354" s="4" t="inlineStr">
+        <is>
+          <t>S-233</t>
+        </is>
+      </c>
+      <c r="D354" s="4" t="inlineStr"/>
+      <c r="E354" s="4" t="inlineStr"/>
+      <c r="F354" s="4" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="4" t="n">
+        <v>105620</v>
+      </c>
+      <c r="B355" s="4" t="n">
+        <v>752</v>
+      </c>
+      <c r="C355" s="4" t="inlineStr">
+        <is>
+          <t>S-233</t>
+        </is>
+      </c>
+      <c r="D355" s="4" t="inlineStr"/>
+      <c r="E355" s="4" t="inlineStr"/>
+      <c r="F355" s="4" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="4" t="n">
+        <v>105620</v>
+      </c>
+      <c r="B356" s="4" t="n">
+        <v>752</v>
+      </c>
+      <c r="C356" s="4" t="inlineStr">
+        <is>
+          <t>S-233</t>
+        </is>
+      </c>
+      <c r="D356" s="4" t="inlineStr"/>
+      <c r="E356" s="4" t="inlineStr"/>
+      <c r="F356" s="4" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="4" t="n">
+        <v>105729</v>
+      </c>
+      <c r="B357" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="C357" s="4" t="inlineStr">
+        <is>
+          <t>S-236</t>
+        </is>
+      </c>
+      <c r="D357" s="4" t="inlineStr"/>
+      <c r="E357" s="4" t="inlineStr"/>
+      <c r="F357" s="4" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="4" t="n">
+        <v>105729</v>
+      </c>
+      <c r="B358" s="4" t="n">
+        <v>312</v>
+      </c>
+      <c r="C358" s="4" t="inlineStr">
+        <is>
+          <t>S-236</t>
+        </is>
+      </c>
+      <c r="D358" s="4" t="inlineStr"/>
+      <c r="E358" s="4" t="inlineStr"/>
+      <c r="F358" s="4" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="4" t="n">
+        <v>105729</v>
+      </c>
+      <c r="B359" s="4" t="n">
+        <v>312</v>
+      </c>
+      <c r="C359" s="4" t="inlineStr">
+        <is>
+          <t>S-236</t>
+        </is>
+      </c>
+      <c r="D359" s="4" t="inlineStr"/>
+      <c r="E359" s="4" t="inlineStr"/>
+      <c r="F359" s="4" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="4" t="n">
+        <v>105729</v>
+      </c>
+      <c r="B360" s="4" t="n">
+        <v>315</v>
+      </c>
+      <c r="C360" s="4" t="inlineStr">
+        <is>
+          <t>S-236</t>
+        </is>
+      </c>
+      <c r="D360" s="4" t="inlineStr"/>
+      <c r="E360" s="4" t="inlineStr"/>
+      <c r="F360" s="4" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="4" t="n">
+        <v>105729</v>
+      </c>
+      <c r="B361" s="4" t="n">
+        <v>327</v>
+      </c>
+      <c r="C361" s="4" t="inlineStr">
+        <is>
+          <t>S-236</t>
+        </is>
+      </c>
+      <c r="D361" s="4" t="inlineStr"/>
+      <c r="E361" s="4" t="inlineStr"/>
+      <c r="F361" s="4" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="4" t="n">
+        <v>105729</v>
+      </c>
+      <c r="B362" s="4" t="n">
+        <v>339</v>
+      </c>
+      <c r="C362" s="4" t="inlineStr">
+        <is>
+          <t>S-236</t>
+        </is>
+      </c>
+      <c r="D362" s="4" t="inlineStr"/>
+      <c r="E362" s="4" t="inlineStr"/>
+      <c r="F362" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 557 AP Physics 1 x2 sections for Tranate (105746) in D-210
- Template 6 Sheet 2: 2 rows added (Teacher 105746, Course 557, Room D-210)
- Template 7: 557 sections needed 1 -> 2
- priority_assignments.json: 557 = 2

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5832,7 +5832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F363"/>
+  <dimension ref="A1:F365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11495,6 +11495,32 @@
         </is>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>105746</v>
+      </c>
+      <c r="B364" t="n">
+        <v>557</v>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>D-210</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>105746</v>
+      </c>
+      <c r="B365" t="n">
+        <v>557</v>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>D-210</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix typo: Tranate course 556 -> 557 (AP Physics 1) in Template 6
- Corrected course code in rows 324-325 from 556 to 557
- Removed duplicate rows 364-365 added in prior commit
- Tranate (105746) now has: 557 x2, 558 x1, 531 x2

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5832,7 +5832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F365"/>
+  <dimension ref="A1:F363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10890,7 +10890,7 @@
         <v>105746</v>
       </c>
       <c r="B324" s="4" t="n">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
@@ -10906,7 +10906,7 @@
         <v>105746</v>
       </c>
       <c r="B325" s="4" t="n">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
@@ -11495,32 +11495,6 @@
         </is>
       </c>
     </row>
-    <row r="364">
-      <c r="A364" t="n">
-        <v>105746</v>
-      </c>
-      <c r="B364" t="n">
-        <v>557</v>
-      </c>
-      <c r="C364" t="inlineStr">
-        <is>
-          <t>D-210</t>
-        </is>
-      </c>
-    </row>
-    <row r="365">
-      <c r="A365" t="n">
-        <v>105746</v>
-      </c>
-      <c r="B365" t="n">
-        <v>557</v>
-      </c>
-      <c r="C365" t="inlineStr">
-        <is>
-          <t>D-210</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 248 Adv Drawing x1 semester section for Dennehy (105810) in J-322
- Template 6 Sheet 2: 1 row added (Teacher 105810, Course 248, Room J-322)
- priority_assignments.json: 248 = 1

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5832,7 +5832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F363"/>
+  <dimension ref="A1:F364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11495,6 +11495,19 @@
         </is>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>105810</v>
+      </c>
+      <c r="B364" t="n">
+        <v>248</v>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Theology corrections: reassign Granieri to 849, add TBD Theology teacher
- Granieri (122120): removed 810x3, 820x2, 830x1; added 849x8 + 830x1
- TBD Theology, New (999999): added to Sheet 1; assigned 810x3, 820x2, 830x1
  (Granieri's former sections transferred to placeholder teacher)
- priority_assignments.json: added 849 = 8 sections

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q64"/>
+  <dimension ref="A1:Q65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5821,6 +5821,21 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>999999</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>TBD Theology</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5832,7 +5847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F364"/>
+  <dimension ref="A1:F373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8111,7 +8126,7 @@
     </row>
     <row r="141">
       <c r="A141" s="4" t="n">
-        <v>122120</v>
+        <v>999999</v>
       </c>
       <c r="B141" s="4" t="n">
         <v>820</v>
@@ -8123,7 +8138,7 @@
     </row>
     <row r="142">
       <c r="A142" s="4" t="n">
-        <v>122120</v>
+        <v>999999</v>
       </c>
       <c r="B142" s="4" t="n">
         <v>820</v>
@@ -8135,7 +8150,7 @@
     </row>
     <row r="143">
       <c r="A143" s="4" t="n">
-        <v>122120</v>
+        <v>999999</v>
       </c>
       <c r="B143" s="4" t="n">
         <v>830</v>
@@ -8147,7 +8162,7 @@
     </row>
     <row r="144">
       <c r="A144" s="4" t="n">
-        <v>122120</v>
+        <v>999999</v>
       </c>
       <c r="B144" s="4" t="n">
         <v>810</v>
@@ -8159,7 +8174,7 @@
     </row>
     <row r="145">
       <c r="A145" s="4" t="n">
-        <v>122120</v>
+        <v>999999</v>
       </c>
       <c r="B145" s="4" t="n">
         <v>810</v>
@@ -8171,7 +8186,7 @@
     </row>
     <row r="146">
       <c r="A146" s="4" t="n">
-        <v>122120</v>
+        <v>999999</v>
       </c>
       <c r="B146" s="4" t="n">
         <v>810</v>
@@ -11508,6 +11523,78 @@
         </is>
       </c>
     </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B365" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B366" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B367" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B368" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B369" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B370" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B371" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B372" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>122120</v>
+      </c>
+      <c r="B373" t="n">
+        <v>830</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 723 Intro to Political Science x1 section for Saggio (117711)
- Template 6 Sheet 2: 1 row added (Teacher 117711, Course 723)
- priority_assignments.json: 723 = 1

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5847,7 +5847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F373"/>
+  <dimension ref="A1:F374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11595,6 +11595,14 @@
         <v>830</v>
       </c>
     </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>117711</v>
+      </c>
+      <c r="B374" t="n">
+        <v>723</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove 830 Theology 11 from TBD Theology (999999), restore to 9 sections
- Template 6 Sheet 2: deleted 830 row for 999999 (TBD now has 810x3 + 820x2 only)
- Template 7: 830 sections needed 10 -> 9

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5847,7 +5847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F374"/>
+  <dimension ref="A1:F373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8153,7 +8153,7 @@
         <v>999999</v>
       </c>
       <c r="B143" s="4" t="n">
-        <v>830</v>
+        <v>810</v>
       </c>
       <c r="C143" s="4" t="inlineStr"/>
       <c r="D143" s="4" t="inlineStr"/>
@@ -8186,10 +8186,10 @@
     </row>
     <row r="146">
       <c r="A146" s="4" t="n">
-        <v>999999</v>
+        <v>107126</v>
       </c>
       <c r="B146" s="4" t="n">
-        <v>810</v>
+        <v>542</v>
       </c>
       <c r="C146" s="4" t="inlineStr"/>
       <c r="D146" s="4" t="inlineStr"/>
@@ -8201,7 +8201,7 @@
         <v>107126</v>
       </c>
       <c r="B147" s="4" t="n">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C147" s="4" t="inlineStr"/>
       <c r="D147" s="4" t="inlineStr"/>
@@ -8222,12 +8222,16 @@
     </row>
     <row r="149">
       <c r="A149" s="4" t="n">
-        <v>107126</v>
+        <v>105669</v>
       </c>
       <c r="B149" s="4" t="n">
-        <v>543</v>
-      </c>
-      <c r="C149" s="4" t="inlineStr"/>
+        <v>430</v>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>D-108</t>
+        </is>
+      </c>
       <c r="D149" s="4" t="inlineStr"/>
       <c r="E149" s="4" t="inlineStr"/>
       <c r="F149" s="4" t="inlineStr"/>
@@ -8269,7 +8273,7 @@
         <v>105669</v>
       </c>
       <c r="B152" s="4" t="n">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
@@ -8298,14 +8302,14 @@
     </row>
     <row r="154">
       <c r="A154" s="4" t="n">
-        <v>105669</v>
+        <v>105832</v>
       </c>
       <c r="B154" s="4" t="n">
-        <v>443</v>
+        <v>761</v>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>D-108</t>
+          <t>I-113</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr"/>
@@ -8317,7 +8321,7 @@
         <v>105832</v>
       </c>
       <c r="B155" s="4" t="n">
-        <v>761</v>
+        <v>730</v>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
@@ -8349,7 +8353,7 @@
         <v>105832</v>
       </c>
       <c r="B157" s="4" t="n">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
@@ -8378,16 +8382,12 @@
     </row>
     <row r="159">
       <c r="A159" s="4" t="n">
-        <v>105832</v>
+        <v>115019</v>
       </c>
       <c r="B159" s="4" t="n">
-        <v>731</v>
-      </c>
-      <c r="C159" s="4" t="inlineStr">
-        <is>
-          <t>I-113</t>
-        </is>
-      </c>
+        <v>412</v>
+      </c>
+      <c r="C159" s="4" t="inlineStr"/>
       <c r="D159" s="4" t="inlineStr"/>
       <c r="E159" s="4" t="inlineStr"/>
       <c r="F159" s="4" t="inlineStr"/>
@@ -8421,7 +8421,7 @@
         <v>115019</v>
       </c>
       <c r="B162" s="4" t="n">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="C162" s="4" t="inlineStr"/>
       <c r="D162" s="4" t="inlineStr"/>
@@ -8442,12 +8442,16 @@
     </row>
     <row r="164">
       <c r="A164" s="4" t="n">
-        <v>115019</v>
+        <v>105829</v>
       </c>
       <c r="B164" s="4" t="n">
-        <v>420</v>
-      </c>
-      <c r="C164" s="4" t="inlineStr"/>
+        <v>510</v>
+      </c>
+      <c r="C164" s="4" t="inlineStr">
+        <is>
+          <t>D-202</t>
+        </is>
+      </c>
       <c r="D164" s="4" t="inlineStr"/>
       <c r="E164" s="4" t="inlineStr"/>
       <c r="F164" s="4" t="inlineStr"/>
@@ -8489,7 +8493,7 @@
         <v>105829</v>
       </c>
       <c r="B167" s="4" t="n">
-        <v>510</v>
+        <v>500</v>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
@@ -8518,14 +8522,14 @@
     </row>
     <row r="169">
       <c r="A169" s="4" t="n">
-        <v>105829</v>
+        <v>105767</v>
       </c>
       <c r="B169" s="4" t="n">
-        <v>500</v>
+        <v>955</v>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>D-202</t>
+          <t>Success Center</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr"/>
@@ -8585,23 +8589,19 @@
         <v>105767</v>
       </c>
       <c r="B173" s="4" t="n">
-        <v>955</v>
-      </c>
-      <c r="C173" s="4" t="inlineStr">
-        <is>
-          <t>Success Center</t>
-        </is>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="C173" s="4" t="inlineStr"/>
       <c r="D173" s="4" t="inlineStr"/>
       <c r="E173" s="4" t="inlineStr"/>
       <c r="F173" s="4" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n">
-        <v>105767</v>
+        <v>122084</v>
       </c>
       <c r="B174" s="4" t="n">
-        <v>112</v>
+        <v>810</v>
       </c>
       <c r="C174" s="4" t="inlineStr"/>
       <c r="D174" s="4" t="inlineStr"/>
@@ -8658,12 +8658,16 @@
     </row>
     <row r="179">
       <c r="A179" s="4" t="n">
-        <v>122084</v>
+        <v>105615</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>810</v>
-      </c>
-      <c r="C179" s="4" t="inlineStr"/>
+        <v>553</v>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>D-201</t>
+        </is>
+      </c>
       <c r="D179" s="4" t="inlineStr"/>
       <c r="E179" s="4" t="inlineStr"/>
       <c r="F179" s="4" t="inlineStr"/>
@@ -8673,7 +8677,7 @@
         <v>105615</v>
       </c>
       <c r="B180" s="4" t="n">
-        <v>553</v>
+        <v>511</v>
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
@@ -8734,16 +8738,12 @@
     </row>
     <row r="184">
       <c r="A184" s="4" t="n">
-        <v>105615</v>
+        <v>105625</v>
       </c>
       <c r="B184" s="4" t="n">
-        <v>511</v>
-      </c>
-      <c r="C184" s="4" t="inlineStr">
-        <is>
-          <t>D-201</t>
-        </is>
-      </c>
+        <v>765</v>
+      </c>
+      <c r="C184" s="4" t="inlineStr"/>
       <c r="D184" s="4" t="inlineStr"/>
       <c r="E184" s="4" t="inlineStr"/>
       <c r="F184" s="4" t="inlineStr"/>
@@ -8765,7 +8765,7 @@
         <v>105625</v>
       </c>
       <c r="B186" s="4" t="n">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="C186" s="4" t="inlineStr"/>
       <c r="D186" s="4" t="inlineStr"/>
@@ -8789,7 +8789,7 @@
         <v>105625</v>
       </c>
       <c r="B188" s="4" t="n">
-        <v>766</v>
+        <v>456</v>
       </c>
       <c r="C188" s="4" t="inlineStr"/>
       <c r="D188" s="4" t="inlineStr"/>
@@ -8798,12 +8798,16 @@
     </row>
     <row r="189">
       <c r="A189" s="4" t="n">
-        <v>105625</v>
+        <v>105628</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>456</v>
-      </c>
-      <c r="C189" s="4" t="inlineStr"/>
+        <v>530</v>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>D-205</t>
+        </is>
+      </c>
       <c r="D189" s="4" t="inlineStr"/>
       <c r="E189" s="4" t="inlineStr"/>
       <c r="F189" s="4" t="inlineStr"/>
@@ -8857,20 +8861,22 @@
       <c r="F192" s="4" t="inlineStr"/>
     </row>
     <row r="193">
-      <c r="A193" s="4" t="n">
+      <c r="A193" t="n">
         <v>105628</v>
       </c>
-      <c r="B193" s="4" t="n">
-        <v>530</v>
-      </c>
-      <c r="C193" s="4" t="inlineStr">
+      <c r="B193" t="n">
+        <v>595</v>
+      </c>
+      <c r="C193" t="inlineStr">
         <is>
           <t>D-205</t>
         </is>
       </c>
-      <c r="D193" s="4" t="inlineStr"/>
-      <c r="E193" s="4" t="inlineStr"/>
-      <c r="F193" s="4" t="inlineStr"/>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -8886,27 +8892,25 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="n">
-        <v>105628</v>
-      </c>
-      <c r="B195" t="n">
-        <v>595</v>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>D-205</t>
-        </is>
-      </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+      <c r="A195" s="4" t="n">
+        <v>111895</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>820</v>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t>J-323</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr"/>
+      <c r="E195" s="4" t="inlineStr"/>
+      <c r="F195" s="4" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n">
@@ -8945,7 +8949,7 @@
         <v>111895</v>
       </c>
       <c r="B198" s="4" t="n">
-        <v>820</v>
+        <v>830</v>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
@@ -8974,14 +8978,14 @@
     </row>
     <row r="200">
       <c r="A200" s="4" t="n">
-        <v>111895</v>
+        <v>106760</v>
       </c>
       <c r="B200" s="4" t="n">
         <v>830</v>
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t>J-323</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="D200" s="4" t="inlineStr"/>
@@ -8989,20 +8993,17 @@
       <c r="F200" s="4" t="inlineStr"/>
     </row>
     <row r="201">
-      <c r="A201" s="4" t="n">
+      <c r="A201" t="n">
         <v>106760</v>
       </c>
-      <c r="B201" s="4" t="n">
-        <v>830</v>
-      </c>
-      <c r="C201" s="4" t="inlineStr">
+      <c r="B201" t="n">
+        <v>851</v>
+      </c>
+      <c r="C201" t="inlineStr">
         <is>
           <t>J-020</t>
         </is>
       </c>
-      <c r="D201" s="4" t="inlineStr"/>
-      <c r="E201" s="4" t="inlineStr"/>
-      <c r="F201" s="4" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -9096,17 +9097,20 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" t="n">
-        <v>106760</v>
-      </c>
-      <c r="B209" t="n">
-        <v>851</v>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>J-020</t>
-        </is>
-      </c>
+      <c r="A209" s="4" t="n">
+        <v>105666</v>
+      </c>
+      <c r="B209" s="4" t="n">
+        <v>820</v>
+      </c>
+      <c r="C209" s="4" t="inlineStr">
+        <is>
+          <t>J-320</t>
+        </is>
+      </c>
+      <c r="D209" s="4" t="inlineStr"/>
+      <c r="E209" s="4" t="inlineStr"/>
+      <c r="F209" s="4" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n">
@@ -9161,7 +9165,7 @@
         <v>105666</v>
       </c>
       <c r="B213" s="4" t="n">
-        <v>820</v>
+        <v>810</v>
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
@@ -9174,14 +9178,14 @@
     </row>
     <row r="214">
       <c r="A214" s="4" t="n">
-        <v>105666</v>
+        <v>102255</v>
       </c>
       <c r="B214" s="4" t="n">
-        <v>810</v>
+        <v>206</v>
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>J-320</t>
+          <t>J-120</t>
         </is>
       </c>
       <c r="D214" s="4" t="inlineStr"/>
@@ -9193,7 +9197,7 @@
         <v>102255</v>
       </c>
       <c r="B215" s="4" t="n">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
@@ -9225,7 +9229,7 @@
         <v>102255</v>
       </c>
       <c r="B217" s="4" t="n">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
@@ -9241,7 +9245,7 @@
         <v>102255</v>
       </c>
       <c r="B218" s="4" t="n">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
@@ -9257,7 +9261,7 @@
         <v>102255</v>
       </c>
       <c r="B219" s="4" t="n">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
@@ -9269,20 +9273,22 @@
       <c r="F219" s="4" t="inlineStr"/>
     </row>
     <row r="220">
-      <c r="A220" s="4" t="n">
+      <c r="A220" t="n">
         <v>102255</v>
       </c>
-      <c r="B220" s="4" t="n">
-        <v>209</v>
-      </c>
-      <c r="C220" s="4" t="inlineStr">
+      <c r="B220" t="n">
+        <v>201</v>
+      </c>
+      <c r="C220" t="inlineStr">
         <is>
           <t>J-120</t>
         </is>
       </c>
-      <c r="D220" s="4" t="inlineStr"/>
-      <c r="E220" s="4" t="inlineStr"/>
-      <c r="F220" s="4" t="inlineStr"/>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -9298,27 +9304,25 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
     </row>
     <row r="222">
-      <c r="A222" t="n">
-        <v>102255</v>
-      </c>
-      <c r="B222" t="n">
-        <v>201</v>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>J-120</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+      <c r="A222" s="4" t="n">
+        <v>117302</v>
+      </c>
+      <c r="B222" s="4" t="n">
+        <v>763</v>
+      </c>
+      <c r="C222" s="4" t="inlineStr">
+        <is>
+          <t>I-011</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr"/>
+      <c r="E222" s="4" t="inlineStr"/>
+      <c r="F222" s="4" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n">
@@ -9341,7 +9345,7 @@
         <v>117302</v>
       </c>
       <c r="B224" s="4" t="n">
-        <v>763</v>
+        <v>721</v>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
@@ -9386,14 +9390,14 @@
     </row>
     <row r="227">
       <c r="A227" s="4" t="n">
-        <v>117302</v>
+        <v>105642</v>
       </c>
       <c r="B227" s="4" t="n">
-        <v>721</v>
+        <v>955</v>
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>Success Center</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr"/>
@@ -9437,11 +9441,11 @@
         <v>105642</v>
       </c>
       <c r="B230" s="4" t="n">
-        <v>955</v>
+        <v>122</v>
       </c>
       <c r="C230" s="4" t="inlineStr">
         <is>
-          <t>Success Center</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D230" s="4" t="inlineStr"/>
@@ -9450,14 +9454,14 @@
     </row>
     <row r="231">
       <c r="A231" s="4" t="n">
-        <v>105642</v>
+        <v>117304</v>
       </c>
       <c r="B231" s="4" t="n">
-        <v>122</v>
+        <v>570</v>
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr"/>
@@ -9485,7 +9489,7 @@
         <v>117304</v>
       </c>
       <c r="B233" s="4" t="n">
-        <v>570</v>
+        <v>585</v>
       </c>
       <c r="C233" s="4" t="inlineStr">
         <is>
@@ -9517,7 +9521,7 @@
         <v>117304</v>
       </c>
       <c r="B235" s="4" t="n">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
@@ -9581,7 +9585,7 @@
         <v>117304</v>
       </c>
       <c r="B239" s="4" t="n">
-        <v>580</v>
+        <v>590</v>
       </c>
       <c r="C239" s="4" t="inlineStr">
         <is>
@@ -9589,7 +9593,11 @@
         </is>
       </c>
       <c r="D239" s="4" t="inlineStr"/>
-      <c r="E239" s="4" t="inlineStr"/>
+      <c r="E239" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F239" s="4" t="inlineStr"/>
     </row>
     <row r="240">
@@ -9617,7 +9625,7 @@
         <v>117304</v>
       </c>
       <c r="B241" s="4" t="n">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
@@ -9654,22 +9662,18 @@
     </row>
     <row r="243">
       <c r="A243" s="4" t="n">
-        <v>117304</v>
+        <v>112092</v>
       </c>
       <c r="B243" s="4" t="n">
-        <v>591</v>
+        <v>521</v>
       </c>
       <c r="C243" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>D-204</t>
         </is>
       </c>
       <c r="D243" s="4" t="inlineStr"/>
-      <c r="E243" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E243" s="4" t="inlineStr"/>
       <c r="F243" s="4" t="inlineStr"/>
     </row>
     <row r="244">
@@ -9725,7 +9729,7 @@
         <v>112092</v>
       </c>
       <c r="B247" s="4" t="n">
-        <v>521</v>
+        <v>531</v>
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
@@ -9738,14 +9742,14 @@
     </row>
     <row r="248">
       <c r="A248" s="4" t="n">
-        <v>112092</v>
+        <v>105671</v>
       </c>
       <c r="B248" s="4" t="n">
-        <v>531</v>
+        <v>720</v>
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>D-204</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr"/>
@@ -9818,14 +9822,14 @@
     </row>
     <row r="253">
       <c r="A253" s="4" t="n">
-        <v>105671</v>
+        <v>106762</v>
       </c>
       <c r="B253" s="4" t="n">
-        <v>720</v>
+        <v>352</v>
       </c>
       <c r="C253" s="4" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D253" s="4" t="inlineStr"/>
@@ -9837,7 +9841,7 @@
         <v>106762</v>
       </c>
       <c r="B254" s="4" t="n">
-        <v>352</v>
+        <v>322</v>
       </c>
       <c r="C254" s="4" t="inlineStr">
         <is>
@@ -9869,7 +9873,7 @@
         <v>106762</v>
       </c>
       <c r="B256" s="4" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
@@ -9885,7 +9889,7 @@
         <v>106762</v>
       </c>
       <c r="B257" s="4" t="n">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
@@ -9901,7 +9905,7 @@
         <v>106762</v>
       </c>
       <c r="B258" s="4" t="n">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C258" s="4" t="inlineStr">
         <is>
@@ -9914,14 +9918,14 @@
     </row>
     <row r="259">
       <c r="A259" s="4" t="n">
-        <v>106762</v>
+        <v>105616</v>
       </c>
       <c r="B259" s="4" t="n">
-        <v>333</v>
+        <v>722</v>
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>I-119</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr"/>
@@ -9949,7 +9953,7 @@
         <v>105616</v>
       </c>
       <c r="B261" s="4" t="n">
-        <v>722</v>
+        <v>733</v>
       </c>
       <c r="C261" s="4" t="inlineStr">
         <is>
@@ -9994,14 +9998,14 @@
     </row>
     <row r="264">
       <c r="A264" s="4" t="n">
-        <v>105616</v>
+        <v>108420</v>
       </c>
       <c r="B264" s="4" t="n">
-        <v>733</v>
+        <v>120</v>
       </c>
       <c r="C264" s="4" t="inlineStr">
         <is>
-          <t>I-119</t>
+          <t>D-104</t>
         </is>
       </c>
       <c r="D264" s="4" t="inlineStr"/>
@@ -10013,7 +10017,7 @@
         <v>108420</v>
       </c>
       <c r="B265" s="4" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="C265" s="4" t="inlineStr">
         <is>
@@ -10061,7 +10065,7 @@
         <v>108420</v>
       </c>
       <c r="B268" s="4" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
@@ -10074,14 +10078,14 @@
     </row>
     <row r="269">
       <c r="A269" s="4" t="n">
-        <v>108420</v>
+        <v>105617</v>
       </c>
       <c r="B269" s="4" t="n">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr"/>
@@ -10109,7 +10113,7 @@
         <v>105617</v>
       </c>
       <c r="B271" s="4" t="n">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
@@ -10141,7 +10145,7 @@
         <v>105617</v>
       </c>
       <c r="B273" s="4" t="n">
-        <v>149</v>
+        <v>110</v>
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
@@ -10154,16 +10158,12 @@
     </row>
     <row r="274">
       <c r="A274" s="4" t="n">
-        <v>105617</v>
+        <v>122121</v>
       </c>
       <c r="B274" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C274" s="4" t="inlineStr">
-        <is>
-          <t>D-101</t>
-        </is>
-      </c>
+        <v>410</v>
+      </c>
+      <c r="C274" s="4" t="inlineStr"/>
       <c r="D274" s="4" t="inlineStr"/>
       <c r="E274" s="4" t="inlineStr"/>
       <c r="F274" s="4" t="inlineStr"/>
@@ -10197,7 +10197,7 @@
         <v>122121</v>
       </c>
       <c r="B277" s="4" t="n">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="C277" s="4" t="inlineStr"/>
       <c r="D277" s="4" t="inlineStr"/>
@@ -10218,12 +10218,16 @@
     </row>
     <row r="279">
       <c r="A279" s="4" t="n">
-        <v>122121</v>
+        <v>105624</v>
       </c>
       <c r="B279" s="4" t="n">
-        <v>420</v>
-      </c>
-      <c r="C279" s="4" t="inlineStr"/>
+        <v>830</v>
+      </c>
+      <c r="C279" s="4" t="inlineStr">
+        <is>
+          <t>J-221</t>
+        </is>
+      </c>
       <c r="D279" s="4" t="inlineStr"/>
       <c r="E279" s="4" t="inlineStr"/>
       <c r="F279" s="4" t="inlineStr"/>
@@ -10294,14 +10298,14 @@
     </row>
     <row r="284">
       <c r="A284" s="4" t="n">
-        <v>105624</v>
+        <v>122122</v>
       </c>
       <c r="B284" s="4" t="n">
-        <v>830</v>
+        <v>2054</v>
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr"/>
@@ -10329,7 +10333,7 @@
         <v>122122</v>
       </c>
       <c r="B286" s="4" t="n">
-        <v>2054</v>
+        <v>2014</v>
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
@@ -10361,7 +10365,7 @@
         <v>122122</v>
       </c>
       <c r="B288" s="4" t="n">
-        <v>2014</v>
+        <v>2024</v>
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
@@ -10393,7 +10397,7 @@
         <v>122122</v>
       </c>
       <c r="B290" s="4" t="n">
-        <v>2024</v>
+        <v>2034</v>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
@@ -10409,7 +10413,7 @@
         <v>122122</v>
       </c>
       <c r="B291" s="4" t="n">
-        <v>2034</v>
+        <v>2044</v>
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
@@ -10438,14 +10442,14 @@
     </row>
     <row r="293">
       <c r="A293" s="4" t="n">
-        <v>122122</v>
+        <v>105651</v>
       </c>
       <c r="B293" s="4" t="n">
-        <v>2044</v>
+        <v>743</v>
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>I-111</t>
+          <t>I-117</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr"/>
@@ -10457,7 +10461,7 @@
         <v>105651</v>
       </c>
       <c r="B294" s="4" t="n">
-        <v>743</v>
+        <v>713</v>
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
@@ -10489,7 +10493,7 @@
         <v>105651</v>
       </c>
       <c r="B296" s="4" t="n">
-        <v>713</v>
+        <v>744</v>
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
@@ -10521,7 +10525,7 @@
         <v>105651</v>
       </c>
       <c r="B298" s="4" t="n">
-        <v>744</v>
+        <v>711</v>
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
@@ -10550,14 +10554,14 @@
     </row>
     <row r="300">
       <c r="A300" s="4" t="n">
-        <v>105651</v>
+        <v>105618</v>
       </c>
       <c r="B300" s="4" t="n">
-        <v>711</v>
+        <v>330</v>
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>S-232</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr"/>
@@ -10585,7 +10589,7 @@
         <v>105618</v>
       </c>
       <c r="B302" s="4" t="n">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
@@ -10630,18 +10634,18 @@
     </row>
     <row r="305">
       <c r="A305" s="4" t="n">
-        <v>105618</v>
+        <v>105808</v>
       </c>
       <c r="B305" s="4" t="n">
-        <v>331</v>
-      </c>
-      <c r="C305" s="4" t="inlineStr">
-        <is>
-          <t>S-232</t>
-        </is>
-      </c>
+        <v>708</v>
+      </c>
+      <c r="C305" s="4" t="inlineStr"/>
       <c r="D305" s="4" t="inlineStr"/>
-      <c r="E305" s="4" t="inlineStr"/>
+      <c r="E305" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F305" s="4" t="inlineStr"/>
     </row>
     <row r="306">
@@ -10671,7 +10675,7 @@
       <c r="D307" s="4" t="inlineStr"/>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="F307" s="4" t="inlineStr"/>
@@ -10710,18 +10714,14 @@
     </row>
     <row r="310">
       <c r="A310" s="4" t="n">
-        <v>105808</v>
+        <v>117711</v>
       </c>
       <c r="B310" s="4" t="n">
-        <v>708</v>
+        <v>751</v>
       </c>
       <c r="C310" s="4" t="inlineStr"/>
       <c r="D310" s="4" t="inlineStr"/>
-      <c r="E310" s="4" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+      <c r="E310" s="4" t="inlineStr"/>
       <c r="F310" s="4" t="inlineStr"/>
     </row>
     <row r="311">
@@ -10729,7 +10729,7 @@
         <v>117711</v>
       </c>
       <c r="B311" s="4" t="n">
-        <v>751</v>
+        <v>741</v>
       </c>
       <c r="C311" s="4" t="inlineStr"/>
       <c r="D311" s="4" t="inlineStr"/>
@@ -10765,7 +10765,7 @@
         <v>117711</v>
       </c>
       <c r="B314" s="4" t="n">
-        <v>741</v>
+        <v>710</v>
       </c>
       <c r="C314" s="4" t="inlineStr"/>
       <c r="D314" s="4" t="inlineStr"/>
@@ -10798,12 +10798,16 @@
     </row>
     <row r="317">
       <c r="A317" s="4" t="n">
-        <v>117711</v>
+        <v>105803</v>
       </c>
       <c r="B317" s="4" t="n">
-        <v>710</v>
-      </c>
-      <c r="C317" s="4" t="inlineStr"/>
+        <v>110</v>
+      </c>
+      <c r="C317" s="4" t="inlineStr">
+        <is>
+          <t>D-102</t>
+        </is>
+      </c>
       <c r="D317" s="4" t="inlineStr"/>
       <c r="E317" s="4" t="inlineStr"/>
       <c r="F317" s="4" t="inlineStr"/>
@@ -10874,28 +10878,28 @@
     </row>
     <row r="322">
       <c r="A322" s="4" t="n">
-        <v>105803</v>
+        <v>105623</v>
       </c>
       <c r="B322" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C322" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
+        <v>551</v>
+      </c>
+      <c r="C322" s="4" t="inlineStr"/>
       <c r="D322" s="4" t="inlineStr"/>
       <c r="E322" s="4" t="inlineStr"/>
       <c r="F322" s="4" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" s="4" t="n">
-        <v>105623</v>
+        <v>105746</v>
       </c>
       <c r="B323" s="4" t="n">
-        <v>551</v>
-      </c>
-      <c r="C323" s="4" t="inlineStr"/>
+        <v>557</v>
+      </c>
+      <c r="C323" s="4" t="inlineStr">
+        <is>
+          <t>D-210</t>
+        </is>
+      </c>
       <c r="D323" s="4" t="inlineStr"/>
       <c r="E323" s="4" t="inlineStr"/>
       <c r="F323" s="4" t="inlineStr"/>
@@ -10921,7 +10925,7 @@
         <v>105746</v>
       </c>
       <c r="B325" s="4" t="n">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
@@ -10937,7 +10941,7 @@
         <v>105746</v>
       </c>
       <c r="B326" s="4" t="n">
-        <v>558</v>
+        <v>531</v>
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
@@ -10966,14 +10970,14 @@
     </row>
     <row r="328">
       <c r="A328" s="4" t="n">
-        <v>105746</v>
+        <v>106765</v>
       </c>
       <c r="B328" s="4" t="n">
-        <v>531</v>
+        <v>310</v>
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>D-210</t>
+          <t>S-235</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr"/>
@@ -11046,16 +11050,12 @@
     </row>
     <row r="333">
       <c r="A333" s="4" t="n">
-        <v>106765</v>
+        <v>105768</v>
       </c>
       <c r="B333" s="4" t="n">
-        <v>310</v>
-      </c>
-      <c r="C333" s="4" t="inlineStr">
-        <is>
-          <t>S-235</t>
-        </is>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="C333" s="4" t="inlineStr"/>
       <c r="D333" s="4" t="inlineStr"/>
       <c r="E333" s="4" t="inlineStr"/>
       <c r="F333" s="4" t="inlineStr"/>
@@ -11065,7 +11065,7 @@
         <v>105768</v>
       </c>
       <c r="B334" s="4" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C334" s="4" t="inlineStr"/>
       <c r="D334" s="4" t="inlineStr"/>
@@ -11077,7 +11077,7 @@
         <v>105768</v>
       </c>
       <c r="B335" s="4" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="C335" s="4" t="inlineStr"/>
       <c r="D335" s="4" t="inlineStr"/>
@@ -11089,7 +11089,7 @@
         <v>105768</v>
       </c>
       <c r="B336" s="4" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C336" s="4" t="inlineStr"/>
       <c r="D336" s="4" t="inlineStr"/>
@@ -11097,16 +11097,12 @@
       <c r="F336" s="4" t="inlineStr"/>
     </row>
     <row r="337">
-      <c r="A337" s="4" t="n">
+      <c r="A337" t="n">
         <v>105768</v>
       </c>
-      <c r="B337" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="C337" s="4" t="inlineStr"/>
-      <c r="D337" s="4" t="inlineStr"/>
-      <c r="E337" s="4" t="inlineStr"/>
-      <c r="F337" s="4" t="inlineStr"/>
+      <c r="B337" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -11117,12 +11113,20 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" t="n">
-        <v>105768</v>
-      </c>
-      <c r="B339" t="n">
-        <v>130</v>
-      </c>
+      <c r="A339" s="4" t="n">
+        <v>106623</v>
+      </c>
+      <c r="B339" s="4" t="n">
+        <v>410</v>
+      </c>
+      <c r="C339" s="4" t="inlineStr">
+        <is>
+          <t>D-110</t>
+        </is>
+      </c>
+      <c r="D339" s="4" t="inlineStr"/>
+      <c r="E339" s="4" t="inlineStr"/>
+      <c r="F339" s="4" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" s="4" t="n">
@@ -11161,7 +11165,7 @@
         <v>106623</v>
       </c>
       <c r="B342" s="4" t="n">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
@@ -11177,7 +11181,7 @@
         <v>106623</v>
       </c>
       <c r="B343" s="4" t="n">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
@@ -11190,14 +11194,14 @@
     </row>
     <row r="344">
       <c r="A344" s="4" t="n">
-        <v>106623</v>
+        <v>105883</v>
       </c>
       <c r="B344" s="4" t="n">
-        <v>420</v>
+        <v>756</v>
       </c>
       <c r="C344" s="4" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>I-012</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr"/>
@@ -11209,7 +11213,7 @@
         <v>105883</v>
       </c>
       <c r="B345" s="4" t="n">
-        <v>756</v>
+        <v>730</v>
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
@@ -11225,7 +11229,7 @@
         <v>105883</v>
       </c>
       <c r="B346" s="4" t="n">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C346" s="4" t="inlineStr">
         <is>
@@ -11241,7 +11245,7 @@
         <v>105883</v>
       </c>
       <c r="B347" s="4" t="n">
-        <v>731</v>
+        <v>710</v>
       </c>
       <c r="C347" s="4" t="inlineStr">
         <is>
@@ -11286,14 +11290,14 @@
     </row>
     <row r="350">
       <c r="A350" s="4" t="n">
-        <v>105883</v>
+        <v>105620</v>
       </c>
       <c r="B350" s="4" t="n">
-        <v>710</v>
+        <v>732</v>
       </c>
       <c r="C350" s="4" t="inlineStr">
         <is>
-          <t>I-012</t>
+          <t>S-233</t>
         </is>
       </c>
       <c r="D350" s="4" t="inlineStr"/>
@@ -11321,7 +11325,7 @@
         <v>105620</v>
       </c>
       <c r="B352" s="4" t="n">
-        <v>732</v>
+        <v>742</v>
       </c>
       <c r="C352" s="4" t="inlineStr">
         <is>
@@ -11353,7 +11357,7 @@
         <v>105620</v>
       </c>
       <c r="B354" s="4" t="n">
-        <v>742</v>
+        <v>752</v>
       </c>
       <c r="C354" s="4" t="inlineStr">
         <is>
@@ -11382,14 +11386,14 @@
     </row>
     <row r="356">
       <c r="A356" s="4" t="n">
-        <v>105620</v>
+        <v>105729</v>
       </c>
       <c r="B356" s="4" t="n">
-        <v>752</v>
+        <v>359</v>
       </c>
       <c r="C356" s="4" t="inlineStr">
         <is>
-          <t>S-233</t>
+          <t>S-236</t>
         </is>
       </c>
       <c r="D356" s="4" t="inlineStr"/>
@@ -11401,7 +11405,7 @@
         <v>105729</v>
       </c>
       <c r="B357" s="4" t="n">
-        <v>359</v>
+        <v>312</v>
       </c>
       <c r="C357" s="4" t="inlineStr">
         <is>
@@ -11433,7 +11437,7 @@
         <v>105729</v>
       </c>
       <c r="B359" s="4" t="n">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C359" s="4" t="inlineStr">
         <is>
@@ -11449,7 +11453,7 @@
         <v>105729</v>
       </c>
       <c r="B360" s="4" t="n">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="C360" s="4" t="inlineStr">
         <is>
@@ -11465,7 +11469,7 @@
         <v>105729</v>
       </c>
       <c r="B361" s="4" t="n">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="C361" s="4" t="inlineStr">
         <is>
@@ -11477,50 +11481,42 @@
       <c r="F361" s="4" t="inlineStr"/>
     </row>
     <row r="362">
-      <c r="A362" s="4" t="n">
-        <v>105729</v>
-      </c>
-      <c r="B362" s="4" t="n">
-        <v>339</v>
-      </c>
-      <c r="C362" s="4" t="inlineStr">
-        <is>
-          <t>S-236</t>
-        </is>
-      </c>
-      <c r="D362" s="4" t="inlineStr"/>
-      <c r="E362" s="4" t="inlineStr"/>
-      <c r="F362" s="4" t="inlineStr"/>
+      <c r="A362" t="n">
+        <v>106765</v>
+      </c>
+      <c r="B362" t="n">
+        <v>310</v>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>S-235</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="n">
-        <v>106765</v>
+        <v>105810</v>
       </c>
       <c r="B363" t="n">
-        <v>310</v>
+        <v>248</v>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>S-235</t>
-        </is>
-      </c>
-      <c r="D363" t="inlineStr">
-        <is>
-          <t>F</t>
+          <t>J-322</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="n">
-        <v>105810</v>
+        <v>122120</v>
       </c>
       <c r="B364" t="n">
-        <v>248</v>
-      </c>
-      <c r="C364" t="inlineStr">
-        <is>
-          <t>J-322</t>
-        </is>
+        <v>849</v>
       </c>
     </row>
     <row r="365">
@@ -11584,22 +11580,14 @@
         <v>122120</v>
       </c>
       <c r="B372" t="n">
-        <v>849</v>
+        <v>830</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="n">
-        <v>122120</v>
+        <v>117711</v>
       </c>
       <c r="B373" t="n">
-        <v>830</v>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" t="n">
-        <v>117711</v>
-      </c>
-      <c r="B374" t="n">
         <v>723</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 6th section of 631 CPR-AED Training/PE to Daniels in Template 6
631 now has 6 semester sections: Chiaravalloti (105747) x4,
Daniels (105763) x2. Matches T7 sections needed = 6.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5847,7 +5847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F373"/>
+  <dimension ref="A1:F374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11591,6 +11591,19 @@
         <v>723</v>
       </c>
     </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>105763</v>
+      </c>
+      <c r="B374" t="n">
+        <v>631</v>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Lopez 201 to 2 semester sections, Umbrino 130 to 3 FY in CLAUDE.md
Lopez (102255): removed extra 201 section (had 3, now 2 — S1 + S2),
co-scheduled with 203 Guitar Ensemble (2 FY sections). T7 updated
from 3 to 2 sections needed.

CLAUDE.md: Umbrino 130 corrected from x2 to x3 FY sections.
Chiaravalloti 631 note updated to reflect Daniels x2 (6 total).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5847,7 +5847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F374"/>
+  <dimension ref="A1:F373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9229,7 +9229,7 @@
         <v>102255</v>
       </c>
       <c r="B217" s="4" t="n">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
@@ -9245,7 +9245,7 @@
         <v>102255</v>
       </c>
       <c r="B218" s="4" t="n">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
@@ -9257,20 +9257,22 @@
       <c r="F218" s="4" t="inlineStr"/>
     </row>
     <row r="219">
-      <c r="A219" s="4" t="n">
+      <c r="A219" t="n">
         <v>102255</v>
       </c>
-      <c r="B219" s="4" t="n">
-        <v>209</v>
-      </c>
-      <c r="C219" s="4" t="inlineStr">
+      <c r="B219" t="n">
+        <v>201</v>
+      </c>
+      <c r="C219" t="inlineStr">
         <is>
           <t>J-120</t>
         </is>
       </c>
-      <c r="D219" s="4" t="inlineStr"/>
-      <c r="E219" s="4" t="inlineStr"/>
-      <c r="F219" s="4" t="inlineStr"/>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -9286,27 +9288,25 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
     </row>
     <row r="221">
-      <c r="A221" t="n">
-        <v>102255</v>
-      </c>
-      <c r="B221" t="n">
-        <v>201</v>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>J-120</t>
-        </is>
-      </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+      <c r="A221" s="4" t="n">
+        <v>117302</v>
+      </c>
+      <c r="B221" s="4" t="n">
+        <v>763</v>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>I-011</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr"/>
+      <c r="E221" s="4" t="inlineStr"/>
+      <c r="F221" s="4" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="n">
@@ -9329,7 +9329,7 @@
         <v>117302</v>
       </c>
       <c r="B223" s="4" t="n">
-        <v>763</v>
+        <v>721</v>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
@@ -9374,14 +9374,14 @@
     </row>
     <row r="226">
       <c r="A226" s="4" t="n">
-        <v>117302</v>
+        <v>105642</v>
       </c>
       <c r="B226" s="4" t="n">
-        <v>721</v>
+        <v>955</v>
       </c>
       <c r="C226" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>Success Center</t>
         </is>
       </c>
       <c r="D226" s="4" t="inlineStr"/>
@@ -9425,11 +9425,11 @@
         <v>105642</v>
       </c>
       <c r="B229" s="4" t="n">
-        <v>955</v>
+        <v>122</v>
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>Success Center</t>
+          <t>I-011</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr"/>
@@ -9438,14 +9438,14 @@
     </row>
     <row r="230">
       <c r="A230" s="4" t="n">
-        <v>105642</v>
+        <v>117304</v>
       </c>
       <c r="B230" s="4" t="n">
-        <v>122</v>
+        <v>570</v>
       </c>
       <c r="C230" s="4" t="inlineStr">
         <is>
-          <t>I-011</t>
+          <t>S-338</t>
         </is>
       </c>
       <c r="D230" s="4" t="inlineStr"/>
@@ -9473,7 +9473,7 @@
         <v>117304</v>
       </c>
       <c r="B232" s="4" t="n">
-        <v>570</v>
+        <v>585</v>
       </c>
       <c r="C232" s="4" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
         <v>117304</v>
       </c>
       <c r="B234" s="4" t="n">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
@@ -9569,7 +9569,7 @@
         <v>117304</v>
       </c>
       <c r="B238" s="4" t="n">
-        <v>580</v>
+        <v>590</v>
       </c>
       <c r="C238" s="4" t="inlineStr">
         <is>
@@ -9577,7 +9577,11 @@
         </is>
       </c>
       <c r="D238" s="4" t="inlineStr"/>
-      <c r="E238" s="4" t="inlineStr"/>
+      <c r="E238" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F238" s="4" t="inlineStr"/>
     </row>
     <row r="239">
@@ -9605,7 +9609,7 @@
         <v>117304</v>
       </c>
       <c r="B240" s="4" t="n">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C240" s="4" t="inlineStr">
         <is>
@@ -9642,22 +9646,18 @@
     </row>
     <row r="242">
       <c r="A242" s="4" t="n">
-        <v>117304</v>
+        <v>112092</v>
       </c>
       <c r="B242" s="4" t="n">
-        <v>591</v>
+        <v>521</v>
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
-          <t>S-338</t>
+          <t>D-204</t>
         </is>
       </c>
       <c r="D242" s="4" t="inlineStr"/>
-      <c r="E242" s="4" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
+      <c r="E242" s="4" t="inlineStr"/>
       <c r="F242" s="4" t="inlineStr"/>
     </row>
     <row r="243">
@@ -9713,7 +9713,7 @@
         <v>112092</v>
       </c>
       <c r="B246" s="4" t="n">
-        <v>521</v>
+        <v>531</v>
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
@@ -9726,14 +9726,14 @@
     </row>
     <row r="247">
       <c r="A247" s="4" t="n">
-        <v>112092</v>
+        <v>105671</v>
       </c>
       <c r="B247" s="4" t="n">
-        <v>531</v>
+        <v>720</v>
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>D-204</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr"/>
@@ -9806,14 +9806,14 @@
     </row>
     <row r="252">
       <c r="A252" s="4" t="n">
-        <v>105671</v>
+        <v>106762</v>
       </c>
       <c r="B252" s="4" t="n">
-        <v>720</v>
+        <v>352</v>
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>S-237</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr"/>
@@ -9825,7 +9825,7 @@
         <v>106762</v>
       </c>
       <c r="B253" s="4" t="n">
-        <v>352</v>
+        <v>322</v>
       </c>
       <c r="C253" s="4" t="inlineStr">
         <is>
@@ -9857,7 +9857,7 @@
         <v>106762</v>
       </c>
       <c r="B255" s="4" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
@@ -9873,7 +9873,7 @@
         <v>106762</v>
       </c>
       <c r="B256" s="4" t="n">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
@@ -9889,7 +9889,7 @@
         <v>106762</v>
       </c>
       <c r="B257" s="4" t="n">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
@@ -9902,14 +9902,14 @@
     </row>
     <row r="258">
       <c r="A258" s="4" t="n">
-        <v>106762</v>
+        <v>105616</v>
       </c>
       <c r="B258" s="4" t="n">
-        <v>333</v>
+        <v>722</v>
       </c>
       <c r="C258" s="4" t="inlineStr">
         <is>
-          <t>S-237</t>
+          <t>I-119</t>
         </is>
       </c>
       <c r="D258" s="4" t="inlineStr"/>
@@ -9937,7 +9937,7 @@
         <v>105616</v>
       </c>
       <c r="B260" s="4" t="n">
-        <v>722</v>
+        <v>733</v>
       </c>
       <c r="C260" s="4" t="inlineStr">
         <is>
@@ -9982,14 +9982,14 @@
     </row>
     <row r="263">
       <c r="A263" s="4" t="n">
-        <v>105616</v>
+        <v>108420</v>
       </c>
       <c r="B263" s="4" t="n">
-        <v>733</v>
+        <v>120</v>
       </c>
       <c r="C263" s="4" t="inlineStr">
         <is>
-          <t>I-119</t>
+          <t>D-104</t>
         </is>
       </c>
       <c r="D263" s="4" t="inlineStr"/>
@@ -10001,7 +10001,7 @@
         <v>108420</v>
       </c>
       <c r="B264" s="4" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="C264" s="4" t="inlineStr">
         <is>
@@ -10049,7 +10049,7 @@
         <v>108420</v>
       </c>
       <c r="B267" s="4" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
@@ -10062,14 +10062,14 @@
     </row>
     <row r="268">
       <c r="A268" s="4" t="n">
-        <v>108420</v>
+        <v>105617</v>
       </c>
       <c r="B268" s="4" t="n">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr"/>
@@ -10097,7 +10097,7 @@
         <v>105617</v>
       </c>
       <c r="B270" s="4" t="n">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
@@ -10129,7 +10129,7 @@
         <v>105617</v>
       </c>
       <c r="B272" s="4" t="n">
-        <v>149</v>
+        <v>110</v>
       </c>
       <c r="C272" s="4" t="inlineStr">
         <is>
@@ -10142,16 +10142,12 @@
     </row>
     <row r="273">
       <c r="A273" s="4" t="n">
-        <v>105617</v>
+        <v>122121</v>
       </c>
       <c r="B273" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C273" s="4" t="inlineStr">
-        <is>
-          <t>D-101</t>
-        </is>
-      </c>
+        <v>410</v>
+      </c>
+      <c r="C273" s="4" t="inlineStr"/>
       <c r="D273" s="4" t="inlineStr"/>
       <c r="E273" s="4" t="inlineStr"/>
       <c r="F273" s="4" t="inlineStr"/>
@@ -10185,7 +10181,7 @@
         <v>122121</v>
       </c>
       <c r="B276" s="4" t="n">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="C276" s="4" t="inlineStr"/>
       <c r="D276" s="4" t="inlineStr"/>
@@ -10206,12 +10202,16 @@
     </row>
     <row r="278">
       <c r="A278" s="4" t="n">
-        <v>122121</v>
+        <v>105624</v>
       </c>
       <c r="B278" s="4" t="n">
-        <v>420</v>
-      </c>
-      <c r="C278" s="4" t="inlineStr"/>
+        <v>830</v>
+      </c>
+      <c r="C278" s="4" t="inlineStr">
+        <is>
+          <t>J-221</t>
+        </is>
+      </c>
       <c r="D278" s="4" t="inlineStr"/>
       <c r="E278" s="4" t="inlineStr"/>
       <c r="F278" s="4" t="inlineStr"/>
@@ -10282,14 +10282,14 @@
     </row>
     <row r="283">
       <c r="A283" s="4" t="n">
-        <v>105624</v>
+        <v>122122</v>
       </c>
       <c r="B283" s="4" t="n">
-        <v>830</v>
+        <v>2054</v>
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>I-111</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr"/>
@@ -10317,7 +10317,7 @@
         <v>122122</v>
       </c>
       <c r="B285" s="4" t="n">
-        <v>2054</v>
+        <v>2014</v>
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
@@ -10349,7 +10349,7 @@
         <v>122122</v>
       </c>
       <c r="B287" s="4" t="n">
-        <v>2014</v>
+        <v>2024</v>
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
@@ -10381,7 +10381,7 @@
         <v>122122</v>
       </c>
       <c r="B289" s="4" t="n">
-        <v>2024</v>
+        <v>2034</v>
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
@@ -10397,7 +10397,7 @@
         <v>122122</v>
       </c>
       <c r="B290" s="4" t="n">
-        <v>2034</v>
+        <v>2044</v>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
@@ -10426,14 +10426,14 @@
     </row>
     <row r="292">
       <c r="A292" s="4" t="n">
-        <v>122122</v>
+        <v>105651</v>
       </c>
       <c r="B292" s="4" t="n">
-        <v>2044</v>
+        <v>743</v>
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>I-111</t>
+          <t>I-117</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr"/>
@@ -10445,7 +10445,7 @@
         <v>105651</v>
       </c>
       <c r="B293" s="4" t="n">
-        <v>743</v>
+        <v>713</v>
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
@@ -10477,7 +10477,7 @@
         <v>105651</v>
       </c>
       <c r="B295" s="4" t="n">
-        <v>713</v>
+        <v>744</v>
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
@@ -10509,7 +10509,7 @@
         <v>105651</v>
       </c>
       <c r="B297" s="4" t="n">
-        <v>744</v>
+        <v>711</v>
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
@@ -10538,14 +10538,14 @@
     </row>
     <row r="299">
       <c r="A299" s="4" t="n">
-        <v>105651</v>
+        <v>105618</v>
       </c>
       <c r="B299" s="4" t="n">
-        <v>711</v>
+        <v>330</v>
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>S-232</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr"/>
@@ -10573,7 +10573,7 @@
         <v>105618</v>
       </c>
       <c r="B301" s="4" t="n">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
@@ -10618,18 +10618,18 @@
     </row>
     <row r="304">
       <c r="A304" s="4" t="n">
-        <v>105618</v>
+        <v>105808</v>
       </c>
       <c r="B304" s="4" t="n">
-        <v>331</v>
-      </c>
-      <c r="C304" s="4" t="inlineStr">
-        <is>
-          <t>S-232</t>
-        </is>
-      </c>
+        <v>708</v>
+      </c>
+      <c r="C304" s="4" t="inlineStr"/>
       <c r="D304" s="4" t="inlineStr"/>
-      <c r="E304" s="4" t="inlineStr"/>
+      <c r="E304" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="F304" s="4" t="inlineStr"/>
     </row>
     <row r="305">
@@ -10659,7 +10659,7 @@
       <c r="D306" s="4" t="inlineStr"/>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="F306" s="4" t="inlineStr"/>
@@ -10698,18 +10698,14 @@
     </row>
     <row r="309">
       <c r="A309" s="4" t="n">
-        <v>105808</v>
+        <v>117711</v>
       </c>
       <c r="B309" s="4" t="n">
-        <v>708</v>
+        <v>751</v>
       </c>
       <c r="C309" s="4" t="inlineStr"/>
       <c r="D309" s="4" t="inlineStr"/>
-      <c r="E309" s="4" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+      <c r="E309" s="4" t="inlineStr"/>
       <c r="F309" s="4" t="inlineStr"/>
     </row>
     <row r="310">
@@ -10717,7 +10713,7 @@
         <v>117711</v>
       </c>
       <c r="B310" s="4" t="n">
-        <v>751</v>
+        <v>741</v>
       </c>
       <c r="C310" s="4" t="inlineStr"/>
       <c r="D310" s="4" t="inlineStr"/>
@@ -10753,7 +10749,7 @@
         <v>117711</v>
       </c>
       <c r="B313" s="4" t="n">
-        <v>741</v>
+        <v>710</v>
       </c>
       <c r="C313" s="4" t="inlineStr"/>
       <c r="D313" s="4" t="inlineStr"/>
@@ -10786,12 +10782,16 @@
     </row>
     <row r="316">
       <c r="A316" s="4" t="n">
-        <v>117711</v>
+        <v>105803</v>
       </c>
       <c r="B316" s="4" t="n">
-        <v>710</v>
-      </c>
-      <c r="C316" s="4" t="inlineStr"/>
+        <v>110</v>
+      </c>
+      <c r="C316" s="4" t="inlineStr">
+        <is>
+          <t>D-102</t>
+        </is>
+      </c>
       <c r="D316" s="4" t="inlineStr"/>
       <c r="E316" s="4" t="inlineStr"/>
       <c r="F316" s="4" t="inlineStr"/>
@@ -10862,28 +10862,28 @@
     </row>
     <row r="321">
       <c r="A321" s="4" t="n">
-        <v>105803</v>
+        <v>105623</v>
       </c>
       <c r="B321" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="C321" s="4" t="inlineStr">
-        <is>
-          <t>D-102</t>
-        </is>
-      </c>
+        <v>551</v>
+      </c>
+      <c r="C321" s="4" t="inlineStr"/>
       <c r="D321" s="4" t="inlineStr"/>
       <c r="E321" s="4" t="inlineStr"/>
       <c r="F321" s="4" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" s="4" t="n">
-        <v>105623</v>
+        <v>105746</v>
       </c>
       <c r="B322" s="4" t="n">
-        <v>551</v>
-      </c>
-      <c r="C322" s="4" t="inlineStr"/>
+        <v>557</v>
+      </c>
+      <c r="C322" s="4" t="inlineStr">
+        <is>
+          <t>D-210</t>
+        </is>
+      </c>
       <c r="D322" s="4" t="inlineStr"/>
       <c r="E322" s="4" t="inlineStr"/>
       <c r="F322" s="4" t="inlineStr"/>
@@ -10909,7 +10909,7 @@
         <v>105746</v>
       </c>
       <c r="B324" s="4" t="n">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
@@ -10925,7 +10925,7 @@
         <v>105746</v>
       </c>
       <c r="B325" s="4" t="n">
-        <v>558</v>
+        <v>531</v>
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
@@ -10954,14 +10954,14 @@
     </row>
     <row r="327">
       <c r="A327" s="4" t="n">
-        <v>105746</v>
+        <v>106765</v>
       </c>
       <c r="B327" s="4" t="n">
-        <v>531</v>
+        <v>310</v>
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>D-210</t>
+          <t>S-235</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr"/>
@@ -11034,16 +11034,12 @@
     </row>
     <row r="332">
       <c r="A332" s="4" t="n">
-        <v>106765</v>
+        <v>105768</v>
       </c>
       <c r="B332" s="4" t="n">
-        <v>310</v>
-      </c>
-      <c r="C332" s="4" t="inlineStr">
-        <is>
-          <t>S-235</t>
-        </is>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="C332" s="4" t="inlineStr"/>
       <c r="D332" s="4" t="inlineStr"/>
       <c r="E332" s="4" t="inlineStr"/>
       <c r="F332" s="4" t="inlineStr"/>
@@ -11053,7 +11049,7 @@
         <v>105768</v>
       </c>
       <c r="B333" s="4" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C333" s="4" t="inlineStr"/>
       <c r="D333" s="4" t="inlineStr"/>
@@ -11065,7 +11061,7 @@
         <v>105768</v>
       </c>
       <c r="B334" s="4" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="C334" s="4" t="inlineStr"/>
       <c r="D334" s="4" t="inlineStr"/>
@@ -11077,7 +11073,7 @@
         <v>105768</v>
       </c>
       <c r="B335" s="4" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C335" s="4" t="inlineStr"/>
       <c r="D335" s="4" t="inlineStr"/>
@@ -11085,16 +11081,12 @@
       <c r="F335" s="4" t="inlineStr"/>
     </row>
     <row r="336">
-      <c r="A336" s="4" t="n">
+      <c r="A336" t="n">
         <v>105768</v>
       </c>
-      <c r="B336" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="C336" s="4" t="inlineStr"/>
-      <c r="D336" s="4" t="inlineStr"/>
-      <c r="E336" s="4" t="inlineStr"/>
-      <c r="F336" s="4" t="inlineStr"/>
+      <c r="B336" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -11105,12 +11097,20 @@
       </c>
     </row>
     <row r="338">
-      <c r="A338" t="n">
-        <v>105768</v>
-      </c>
-      <c r="B338" t="n">
-        <v>130</v>
-      </c>
+      <c r="A338" s="4" t="n">
+        <v>106623</v>
+      </c>
+      <c r="B338" s="4" t="n">
+        <v>410</v>
+      </c>
+      <c r="C338" s="4" t="inlineStr">
+        <is>
+          <t>D-110</t>
+        </is>
+      </c>
+      <c r="D338" s="4" t="inlineStr"/>
+      <c r="E338" s="4" t="inlineStr"/>
+      <c r="F338" s="4" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" s="4" t="n">
@@ -11149,7 +11149,7 @@
         <v>106623</v>
       </c>
       <c r="B341" s="4" t="n">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
@@ -11165,7 +11165,7 @@
         <v>106623</v>
       </c>
       <c r="B342" s="4" t="n">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
@@ -11178,14 +11178,14 @@
     </row>
     <row r="343">
       <c r="A343" s="4" t="n">
-        <v>106623</v>
+        <v>105883</v>
       </c>
       <c r="B343" s="4" t="n">
-        <v>420</v>
+        <v>756</v>
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>I-012</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr"/>
@@ -11197,7 +11197,7 @@
         <v>105883</v>
       </c>
       <c r="B344" s="4" t="n">
-        <v>756</v>
+        <v>730</v>
       </c>
       <c r="C344" s="4" t="inlineStr">
         <is>
@@ -11213,7 +11213,7 @@
         <v>105883</v>
       </c>
       <c r="B345" s="4" t="n">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
@@ -11229,7 +11229,7 @@
         <v>105883</v>
       </c>
       <c r="B346" s="4" t="n">
-        <v>731</v>
+        <v>710</v>
       </c>
       <c r="C346" s="4" t="inlineStr">
         <is>
@@ -11274,14 +11274,14 @@
     </row>
     <row r="349">
       <c r="A349" s="4" t="n">
-        <v>105883</v>
+        <v>105620</v>
       </c>
       <c r="B349" s="4" t="n">
-        <v>710</v>
+        <v>732</v>
       </c>
       <c r="C349" s="4" t="inlineStr">
         <is>
-          <t>I-012</t>
+          <t>S-233</t>
         </is>
       </c>
       <c r="D349" s="4" t="inlineStr"/>
@@ -11309,7 +11309,7 @@
         <v>105620</v>
       </c>
       <c r="B351" s="4" t="n">
-        <v>732</v>
+        <v>742</v>
       </c>
       <c r="C351" s="4" t="inlineStr">
         <is>
@@ -11341,7 +11341,7 @@
         <v>105620</v>
       </c>
       <c r="B353" s="4" t="n">
-        <v>742</v>
+        <v>752</v>
       </c>
       <c r="C353" s="4" t="inlineStr">
         <is>
@@ -11370,14 +11370,14 @@
     </row>
     <row r="355">
       <c r="A355" s="4" t="n">
-        <v>105620</v>
+        <v>105729</v>
       </c>
       <c r="B355" s="4" t="n">
-        <v>752</v>
+        <v>359</v>
       </c>
       <c r="C355" s="4" t="inlineStr">
         <is>
-          <t>S-233</t>
+          <t>S-236</t>
         </is>
       </c>
       <c r="D355" s="4" t="inlineStr"/>
@@ -11389,7 +11389,7 @@
         <v>105729</v>
       </c>
       <c r="B356" s="4" t="n">
-        <v>359</v>
+        <v>312</v>
       </c>
       <c r="C356" s="4" t="inlineStr">
         <is>
@@ -11421,7 +11421,7 @@
         <v>105729</v>
       </c>
       <c r="B358" s="4" t="n">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C358" s="4" t="inlineStr">
         <is>
@@ -11437,7 +11437,7 @@
         <v>105729</v>
       </c>
       <c r="B359" s="4" t="n">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="C359" s="4" t="inlineStr">
         <is>
@@ -11453,7 +11453,7 @@
         <v>105729</v>
       </c>
       <c r="B360" s="4" t="n">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="C360" s="4" t="inlineStr">
         <is>
@@ -11465,50 +11465,42 @@
       <c r="F360" s="4" t="inlineStr"/>
     </row>
     <row r="361">
-      <c r="A361" s="4" t="n">
-        <v>105729</v>
-      </c>
-      <c r="B361" s="4" t="n">
-        <v>339</v>
-      </c>
-      <c r="C361" s="4" t="inlineStr">
-        <is>
-          <t>S-236</t>
-        </is>
-      </c>
-      <c r="D361" s="4" t="inlineStr"/>
-      <c r="E361" s="4" t="inlineStr"/>
-      <c r="F361" s="4" t="inlineStr"/>
+      <c r="A361" t="n">
+        <v>106765</v>
+      </c>
+      <c r="B361" t="n">
+        <v>310</v>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>S-235</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="n">
-        <v>106765</v>
+        <v>105810</v>
       </c>
       <c r="B362" t="n">
-        <v>310</v>
+        <v>248</v>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>S-235</t>
-        </is>
-      </c>
-      <c r="D362" t="inlineStr">
-        <is>
-          <t>F</t>
+          <t>J-322</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="n">
-        <v>105810</v>
+        <v>122120</v>
       </c>
       <c r="B363" t="n">
-        <v>248</v>
-      </c>
-      <c r="C363" t="inlineStr">
-        <is>
-          <t>J-322</t>
-        </is>
+        <v>849</v>
       </c>
     </row>
     <row r="364">
@@ -11572,33 +11564,25 @@
         <v>122120</v>
       </c>
       <c r="B371" t="n">
-        <v>849</v>
+        <v>830</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="n">
-        <v>122120</v>
+        <v>117711</v>
       </c>
       <c r="B372" t="n">
-        <v>830</v>
+        <v>723</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="n">
-        <v>117711</v>
+        <v>105763</v>
       </c>
       <c r="B373" t="n">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" t="n">
-        <v>105763</v>
-      </c>
-      <c r="B374" t="n">
         <v>631</v>
       </c>
-      <c r="C374" t="inlineStr">
+      <c r="C373" t="inlineStr">
         <is>
           <t>Gym</t>
         </is>

</xml_diff>

<commit_message>
Fix room name mismatch: "AUD" → "Auditorium" in Template 6
Template 9 defines the room as "Auditorium", but Template 6 used "AUD"
for 3 sections (courses 225, 227, 228). Standardized to match T9.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -6091,7 +6091,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>AUD</t>
+          <t>Auditorium</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>AUD</t>
+          <t>Auditorium</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr"/>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>AUD</t>
+          <t>Auditorium</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Remove erroneous prescribed period F from Tuesta 310 Spanish I
No Don Bosco Prep courses have a prescribed period — the engine
determines period placement. Cleared the Period F entry from row 361.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -11476,11 +11476,6 @@
           <t>S-235</t>
         </is>
       </c>
-      <c r="D361" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
     </row>
     <row r="362">
       <c r="A362" t="n">

</xml_diff>

<commit_message>
Update Template 6: Saggio approved 6th S2 only, Tuesta approved 6th FY
- Saggio (117711): Approved 6th Period S2 Only = Y (was N)
- Tuesta (106765): Approved 6th Period FY = Y (was N)
- Per JC Iofalo directive: these teachers are now approved for overload

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -5026,7 +5026,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Fix #7: Standardize cohort naming L.E.O. II → LEO II in Template 6
- Changed 2 cells in T6 Sheet 2 'Prescribed Cohort' column (rows 296, 297)
- Now consistent with T7, T8, engine CLI flags, and all documentation
- Engine uses non-empty check only — no functional impact, cosmetic consistency

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -11630,7 +11630,7 @@
       </c>
       <c r="F296" s="4" t="inlineStr">
         <is>
-          <t>L.E.O. II</t>
+          <t>LEO II</t>
         </is>
       </c>
     </row>
@@ -11654,7 +11654,7 @@
       </c>
       <c r="F297" s="4" t="inlineStr">
         <is>
-          <t>L.E.O. II</t>
+          <t>LEO II</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prescribe J-321 (Theology room) to 6 sections across 3 teachers
J-321 historically used as Theology room, now prescribed in T6 Sheet 2:
- Junis, Thomas (122084): 810 Theology 9 × 2 sections (rows 318-319)
- Granieri, William (122120): 830 × 1 + 849 × 1 sections (rows 341-342)
- TBD Theology, New (999999): 810 Theology 9 × 2 sections (rows 315-316)

6 of 7 periods filled. 7th period left open for use by any teacher/section.
Engine has Engine Choice on which teacher is placed in which specific periods.
Per JC directive: J-321 is a Theology room available to other departments
when no Theology class is scheduled.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_6_Teacher_Profiles.xlsx
+++ b/templates/Template_6_Teacher_Profiles.xlsx
@@ -11985,7 +11985,11 @@
       <c r="B315" s="4" t="n">
         <v>810</v>
       </c>
-      <c r="C315" s="4" t="n"/>
+      <c r="C315" s="4" t="inlineStr">
+        <is>
+          <t>J-321</t>
+        </is>
+      </c>
       <c r="D315" s="4" t="n"/>
       <c r="E315" s="4" t="inlineStr">
         <is>
@@ -12001,7 +12005,11 @@
       <c r="B316" s="4" t="n">
         <v>810</v>
       </c>
-      <c r="C316" s="4" t="n"/>
+      <c r="C316" s="4" t="inlineStr">
+        <is>
+          <t>J-321</t>
+        </is>
+      </c>
       <c r="D316" s="4" t="n"/>
       <c r="E316" s="4" t="inlineStr">
         <is>
@@ -12033,7 +12041,11 @@
       <c r="B318" s="4" t="n">
         <v>810</v>
       </c>
-      <c r="C318" s="4" t="n"/>
+      <c r="C318" s="4" t="inlineStr">
+        <is>
+          <t>J-321</t>
+        </is>
+      </c>
       <c r="D318" s="4" t="n"/>
       <c r="E318" s="4" t="inlineStr">
         <is>
@@ -12049,7 +12061,11 @@
       <c r="B319" s="4" t="n">
         <v>810</v>
       </c>
-      <c r="C319" s="4" t="n"/>
+      <c r="C319" s="4" t="inlineStr">
+        <is>
+          <t>J-321</t>
+        </is>
+      </c>
       <c r="D319" s="4" t="n"/>
       <c r="E319" s="4" t="inlineStr">
         <is>
@@ -12465,7 +12481,11 @@
       <c r="B341" s="5" t="n">
         <v>830</v>
       </c>
-      <c r="C341" s="5" t="n"/>
+      <c r="C341" s="5" t="inlineStr">
+        <is>
+          <t>J-321</t>
+        </is>
+      </c>
       <c r="D341" s="5" t="n"/>
       <c r="E341" s="4" t="inlineStr">
         <is>
@@ -12481,7 +12501,11 @@
       <c r="B342" s="5" t="n">
         <v>849</v>
       </c>
-      <c r="C342" s="5" t="n"/>
+      <c r="C342" s="5" t="inlineStr">
+        <is>
+          <t>J-321</t>
+        </is>
+      </c>
       <c r="D342" s="5" t="n"/>
       <c r="E342" s="4" t="inlineStr">
         <is>

</xml_diff>